<commit_message>
Add word "henhold" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AB2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -517,9 +517,95 @@
         <v>Lapses_EN</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>6cebe36d-5d01-40b2-906b-8a829745c73d</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>henhold</v>
+      </c>
+      <c r="D2" t="str">
+        <v>henhold</v>
+      </c>
+      <c r="E2" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>[ˈhεnˌhʌlˀ]</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://static.ordnet.dk/mp3/11020/11020419_1.mp3</v>
+      </c>
+      <c r="J2" t="str">
+        <v>kun i udtrykket:</v>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+      </c>
+      <c r="N2" t="str">
+        <v>chrome-extension://mhjfbmdgcfjbbpaeojofohoefgiehjai/edge_pdf/index.html</v>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>partial</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -528,28 +614,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -631,8 +717,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="16.83203125"/>
+    <col min="2" max="2" customWidth="1" width="28.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "brugsloven" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AB3"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -603,9 +603,95 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>0d3fc2e5-0c30-4cd1-a873-0cdfc98007a4</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C3" t="str">
+        <v>brugsloven</v>
+      </c>
+      <c r="D3" t="str">
+        <v>brugslov</v>
+      </c>
+      <c r="E3" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F3" t="str">
+        <v>en</v>
+      </c>
+      <c r="G3" t="str">
+        <v>-en, -e, -ene</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v>sammensat af brugs + lov</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Utility Act</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+      </c>
+      <c r="N3" t="str">
+        <v>chrome-extension://mhjfbmdgcfjbbpaeojofohoefgiehjai/edge_pdf/index.html</v>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "gennemføres" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AB4"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -689,9 +689,95 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>05d5014c-1bc9-48f5-ac80-9c6659843c67</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C4" t="str">
+        <v>gennemføres</v>
+      </c>
+      <c r="D4" t="str">
+        <v>gennemføre</v>
+      </c>
+      <c r="E4" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>-r, ..førte, ..ført</v>
+      </c>
+      <c r="H4" t="str">
+        <v>[ˈgεnəmˌføˀʌ]</v>
+      </c>
+      <c r="I4" t="str">
+        <v>https://static.ordnet.dk/mp3/11017/11017622_1.mp3</v>
+      </c>
+      <c r="J4" t="str">
+        <v>udføre og afslutte (med godt resultat)</v>
+      </c>
+      <c r="K4" t="str">
+        <v>be carried out</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "væsentlige" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AB5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -775,9 +775,95 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>956f08a1-4407-41d9-9dec-b137931c6d72</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C5" t="str">
+        <v>væsentlige</v>
+      </c>
+      <c r="D5" t="str">
+        <v>væsentlig</v>
+      </c>
+      <c r="E5" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H5" t="str">
+        <v>[ˈvεˀsənli]</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://static.ordnet.dk/mp3/12007/12007582_1.mp3</v>
+      </c>
+      <c r="J5" t="str">
+        <v>som udgør eller vedrører en tings inderste og egentlige væsen, og som derfor er yderst vigtig</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Essential</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v/>
+      </c>
+      <c r="Z5" t="str">
+        <v/>
+      </c>
+      <c r="AA5" t="str">
+        <v/>
+      </c>
+      <c r="AB5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "påvirkninger" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB5"/>
+  <dimension ref="A1:AB6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -861,9 +861,95 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C6" t="str">
+        <v>påvirkninger</v>
+      </c>
+      <c r="D6" t="str">
+        <v>påvirkning</v>
+      </c>
+      <c r="E6" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F6" t="str">
+        <v>en</v>
+      </c>
+      <c r="G6" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H6" t="str">
+        <v>[ˈpʌˌviɐ̯gneŋ]</v>
+      </c>
+      <c r="I6" t="str">
+        <v>https://static.ordnet.dk/mp3/11041/11041875_1.mp3</v>
+      </c>
+      <c r="J6" t="str">
+        <v>det at noget har en bestemt virkning på nogen eller noget, oftest med en ændring til følge</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Influences</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v/>
+      </c>
+      <c r="Y6" t="str">
+        <v/>
+      </c>
+      <c r="Z6" t="str">
+        <v/>
+      </c>
+      <c r="AA6" t="str">
+        <v/>
+      </c>
+      <c r="AB6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB6"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "omfatter" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB6"/>
+  <dimension ref="A1:AB7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -947,9 +947,95 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>8e0306d1-6036-4774-8e44-a607339a1174</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C7" t="str">
+        <v>omfatter</v>
+      </c>
+      <c r="D7" t="str">
+        <v>omfatte</v>
+      </c>
+      <c r="E7" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v>https://static.ordnet.dk/mp3/11037/11037099_1.mp3</v>
+      </c>
+      <c r="J7" t="str">
+        <v>have som bestanddele; bestå eller udgøres af</v>
+      </c>
+      <c r="K7" t="str">
+        <v>includes</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+      <c r="X7" t="str">
+        <v/>
+      </c>
+      <c r="Y7" t="str">
+        <v/>
+      </c>
+      <c r="Z7" t="str">
+        <v/>
+      </c>
+      <c r="AA7" t="str">
+        <v/>
+      </c>
+      <c r="AB7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Klage" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB7"/>
+  <dimension ref="A1:AB8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1033,9 +1033,95 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>0254c900-1cbd-4360-853b-baf63aadaf10</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Klage</v>
+      </c>
+      <c r="D8" t="str">
+        <v>klage</v>
+      </c>
+      <c r="E8" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F8" t="str">
+        <v>en</v>
+      </c>
+      <c r="G8" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H8" t="str">
+        <v>[ˈklæːjə]</v>
+      </c>
+      <c r="I8" t="str">
+        <v>https://static.ordnet.dk/mp3/11026/11026090_1.mp3</v>
+      </c>
+      <c r="J8" t="str">
+        <v>mundtlig eller især skriftlig henvendelse til en ledende person eller myndighed med anmodning om undersøgelse eller påtale af et (påstået) kritisabelt, uretfærdigt eller retsstridigt forhold</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Complaint</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
+      <c r="Y8" t="str">
+        <v/>
+      </c>
+      <c r="Z8" t="str">
+        <v/>
+      </c>
+      <c r="AA8" t="str">
+        <v/>
+      </c>
+      <c r="AB8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "samt" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB8"/>
+  <dimension ref="A1:AB9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1119,9 +1119,95 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>8732aac0-4d2b-43cc-9af1-60bf3151752b</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C9" t="str">
+        <v>samt</v>
+      </c>
+      <c r="D9" t="str">
+        <v>samt</v>
+      </c>
+      <c r="E9" t="str">
+        <v>konjunktion</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>[ˈsɑmˀd]</v>
+      </c>
+      <c r="I9" t="str">
+        <v>https://static.ordnet.dk/mp3/11044/11044804_1.mp3</v>
+      </c>
+      <c r="J9" t="str">
+        <v>bruges for at forbinde ord og sætningsled i sideordnet rækkefølge undertiden angivende en større afstand mellem leddene end og</v>
+      </c>
+      <c r="K9" t="str">
+        <v>and</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
+      <c r="X9" t="str">
+        <v/>
+      </c>
+      <c r="Y9" t="str">
+        <v/>
+      </c>
+      <c r="Z9" t="str">
+        <v/>
+      </c>
+      <c r="AA9" t="str">
+        <v/>
+      </c>
+      <c r="AB9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "miljøredegørelse" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,36 +399,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB9"/>
+  <dimension ref="A1:AB10"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1205,9 +1205,95 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>0933c06d-fcdc-4401-9d43-79f732aadad7</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C10" t="str">
+        <v>miljøredegørelse</v>
+      </c>
+      <c r="D10" t="str">
+        <v>miljøredegørelse</v>
+      </c>
+      <c r="E10" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F10" t="str">
+        <v>en</v>
+      </c>
+      <c r="G10" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v>sammensat af miljø + redegørelse</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Environmental statement</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
+      <c r="Y10" t="str">
+        <v/>
+      </c>
+      <c r="Z10" t="str">
+        <v/>
+      </c>
+      <c r="AA10" t="str">
+        <v/>
+      </c>
+      <c r="AB10" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "ANSØGNING" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB10"/>
+  <dimension ref="A1:AB11"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1291,9 +1291,95 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="C11" t="str">
+        <v>ANSØGNING</v>
+      </c>
+      <c r="D11" t="str">
+        <v>ansøgning</v>
+      </c>
+      <c r="E11" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F11" t="str">
+        <v>en</v>
+      </c>
+      <c r="G11" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H11" t="str">
+        <v>[ˈanˌsøjˀneŋ]</v>
+      </c>
+      <c r="I11" t="str">
+        <v>https://static.ordnet.dk/mp3/11002/11002018_1.mp3</v>
+      </c>
+      <c r="J11" t="str">
+        <v>det at ansøge om noget</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Application</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
+      </c>
+      <c r="X11" t="str">
+        <v/>
+      </c>
+      <c r="Y11" t="str">
+        <v/>
+      </c>
+      <c r="Z11" t="str">
+        <v/>
+      </c>
+      <c r="AA11" t="str">
+        <v/>
+      </c>
+      <c r="AB11" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "bryder" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB11"/>
+  <dimension ref="A1:AB12"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1377,9 +1377,95 @@
         <v/>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>87f910eb-6aa4-4751-ad3a-14ec49047ac6</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C12" t="str">
+        <v>bryder</v>
+      </c>
+      <c r="D12" t="str">
+        <v>bryder</v>
+      </c>
+      <c r="E12" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F12" t="str">
+        <v>en</v>
+      </c>
+      <c r="G12" t="str">
+        <v>-en, -e, -ne</v>
+      </c>
+      <c r="H12" t="str">
+        <v>[ˈbʁyːðʌ]</v>
+      </c>
+      <c r="I12" t="str">
+        <v>https://static.ordnet.dk/mp3/11006/11006414_1.mp3</v>
+      </c>
+      <c r="J12" t="str">
+        <v>person der udøver sportsgrenen brydning</v>
+      </c>
+      <c r="K12" t="str">
+        <v>breaks</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N12" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O12" t="str">
+        <v>https://ing.dk/#:~:text=bryder</v>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
+        <v/>
+      </c>
+      <c r="X12" t="str">
+        <v/>
+      </c>
+      <c r="Y12" t="str">
+        <v/>
+      </c>
+      <c r="Z12" t="str">
+        <v/>
+      </c>
+      <c r="AA12" t="str">
+        <v/>
+      </c>
+      <c r="AB12" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Pløjer" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB12"/>
+  <dimension ref="A1:AB13"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1463,9 +1463,95 @@
         <v/>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>c2d45936-5793-42b4-968a-e066bcb27036</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Pløjer</v>
+      </c>
+      <c r="D13" t="str">
+        <v>pløje</v>
+      </c>
+      <c r="E13" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H13" t="str">
+        <v>[ˈplʌjə]</v>
+      </c>
+      <c r="I13" t="str">
+        <v>https://static.ordnet.dk/mp3/11040/11040224_1.mp3</v>
+      </c>
+      <c r="J13" t="str">
+        <v>vende det øverste jordlag med en plov inden man sår eller planter afgrøder</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Plows</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N13" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O13" t="str">
+        <v>https://ing.dk/#:~:text=Pl%C3%B8jer</v>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
+        <v/>
+      </c>
+      <c r="X13" t="str">
+        <v/>
+      </c>
+      <c r="Y13" t="str">
+        <v/>
+      </c>
+      <c r="Z13" t="str">
+        <v/>
+      </c>
+      <c r="AA13" t="str">
+        <v/>
+      </c>
+      <c r="AB13" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "vandløb" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB13"/>
+  <dimension ref="A1:AB14"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1549,9 +1549,95 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>03f5e6c8-8aee-4335-872b-3d6af367eeee</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C14" t="str">
+        <v>vandløb</v>
+      </c>
+      <c r="D14" t="str">
+        <v>vandløb</v>
+      </c>
+      <c r="E14" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F14" t="str">
+        <v>et</v>
+      </c>
+      <c r="G14" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v>https://static.ordnet.dk/mp3/12005/12005692_1.mp3</v>
+      </c>
+      <c r="J14" t="str">
+        <v>lang, let skrånende fordybning i landskabet med strømmende vand fx en bæk, en å eller en flod</v>
+      </c>
+      <c r="K14" t="str">
+        <v>stream</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="N14" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="O14" t="str">
+        <v>https://ing.dk/#:~:text=vandl%C3%B8b</v>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v/>
+      </c>
+      <c r="U14" t="str">
+        <v/>
+      </c>
+      <c r="V14" t="str">
+        <v/>
+      </c>
+      <c r="W14" t="str">
+        <v/>
+      </c>
+      <c r="X14" t="str">
+        <v/>
+      </c>
+      <c r="Y14" t="str">
+        <v/>
+      </c>
+      <c r="Z14" t="str">
+        <v/>
+      </c>
+      <c r="AA14" t="str">
+        <v/>
+      </c>
+      <c r="AB14" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "helt ud til" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -401,34 +401,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB14"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1644,30 +1644,30 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V1"/>
+  <dimension ref="A1:V2"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1738,9 +1738,77 @@
         <v>Lapses_EN</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>a0876471-cbaf-41fc-a1d7-5d58d6045929</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C2" t="str">
+        <v>helt ud til</v>
+      </c>
+      <c r="D2" t="str">
+        <v>helt=quite · ud=out · til=to</v>
+      </c>
+      <c r="E2" t="str">
+        <v>all the way to</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+      </c>
+      <c r="H2" t="str">
+        <v>https://ing.dk/</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://ing.dk/#:~:text=helt%20ud%20til</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "utroligt" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,36 +399,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB14"/>
+  <dimension ref="A1:AB15"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1635,9 +1635,95 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>6d8e9813-5550-45ab-9874-78033b6c2cd6</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C15" t="str">
+        <v>utroligt</v>
+      </c>
+      <c r="D15" t="str">
+        <v>utrolig</v>
+      </c>
+      <c r="E15" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H15" t="str">
+        <v>[uˈtʁoˀli]</v>
+      </c>
+      <c r="I15" t="str">
+        <v>https://static.ordnet.dk/mp3/12005/12005364_1.mp3</v>
+      </c>
+      <c r="J15" t="str">
+        <v>for usædvanlig eller usandsynlig til at man kan tro det</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Unbelievable</v>
+      </c>
+      <c r="L15" t="str">
+        <v>DN: »Helt utroligt«</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb | Ingeniøren</v>
+      </c>
+      <c r="N15" t="str">
+        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb</v>
+      </c>
+      <c r="O15" t="str">
+        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb#:~:text=utroligt</v>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
+      <c r="W15" t="str">
+        <v/>
+      </c>
+      <c r="X15" t="str">
+        <v/>
+      </c>
+      <c r="Y15" t="str">
+        <v/>
+      </c>
+      <c r="Z15" t="str">
+        <v/>
+      </c>
+      <c r="AA15" t="str">
+        <v/>
+      </c>
+      <c r="AB15" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1646,28 +1732,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:V2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "forargede" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB15"/>
+  <dimension ref="A1:AB16"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1721,9 +1721,95 @@
         <v/>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>369d0ecd-e56f-4e9b-882e-e7c44c687a79</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C16" t="str">
+        <v>forargede</v>
+      </c>
+      <c r="D16" t="str">
+        <v>forarge</v>
+      </c>
+      <c r="E16" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H16" t="str">
+        <v>[fʌˈɑˀwə]</v>
+      </c>
+      <c r="I16" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014199_1.mp3</v>
+      </c>
+      <c r="J16" t="str">
+        <v>vække afsky, harme, vrede, modvilje el.lign. ved at krænke moralske normer</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Outraged</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Også i Danmarks Naturfredningsforening (DN) er man forargede over, at der ikke er større fokus på naturbeskyttelsen både hos landbruget og på kommunernes kontorer.</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb | Ingeniøren</v>
+      </c>
+      <c r="N16" t="str">
+        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb</v>
+      </c>
+      <c r="O16" t="str">
+        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb#:~:text=forargede</v>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16" t="str">
+        <v/>
+      </c>
+      <c r="V16" t="str">
+        <v/>
+      </c>
+      <c r="W16" t="str">
+        <v/>
+      </c>
+      <c r="X16" t="str">
+        <v/>
+      </c>
+      <c r="Y16" t="str">
+        <v/>
+      </c>
+      <c r="Z16" t="str">
+        <v/>
+      </c>
+      <c r="AA16" t="str">
+        <v/>
+      </c>
+      <c r="AB16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "To" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB16"/>
+  <dimension ref="A1:AB17"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1807,9 +1807,95 @@
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2ae5b453-b4ee-456f-8c22-324aba8103d0</v>
+      </c>
+      <c r="B17" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C17" t="str">
+        <v>To</v>
+      </c>
+      <c r="D17" t="str">
+        <v>to.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>forkortelse</v>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v>= torsdag</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Two.</v>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
+      <c r="S17" t="str">
+        <v/>
+      </c>
+      <c r="T17" t="str">
+        <v/>
+      </c>
+      <c r="U17" t="str">
+        <v/>
+      </c>
+      <c r="V17" t="str">
+        <v/>
+      </c>
+      <c r="W17" t="str">
+        <v/>
+      </c>
+      <c r="X17" t="str">
+        <v/>
+      </c>
+      <c r="Y17" t="str">
+        <v/>
+      </c>
+      <c r="Z17" t="str">
+        <v/>
+      </c>
+      <c r="AA17" t="str">
+        <v/>
+      </c>
+      <c r="AB17" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Rådgivning" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB17"/>
+  <dimension ref="A1:AB18"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1893,9 +1893,95 @@
         <v/>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>94801dbf-f81c-46cc-a320-3e40b0903e79</v>
+      </c>
+      <c r="B18" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Rådgivning</v>
+      </c>
+      <c r="D18" t="str">
+        <v>rådgivning</v>
+      </c>
+      <c r="E18" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F18" t="str">
+        <v>en</v>
+      </c>
+      <c r="G18" t="str">
+        <v>-en, -er, -erne</v>
+      </c>
+      <c r="H18" t="str">
+        <v>[ˈʁʌðˌgiwˀneŋ]</v>
+      </c>
+      <c r="I18" t="str">
+        <v>https://static.ordnet.dk/mp3/11044/11044289_1.mp3</v>
+      </c>
+      <c r="J18" t="str">
+        <v>det at rådgive</v>
+      </c>
+      <c r="K18" t="str">
+        <v>counseling</v>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
+      <c r="U18" t="str">
+        <v/>
+      </c>
+      <c r="V18" t="str">
+        <v/>
+      </c>
+      <c r="W18" t="str">
+        <v/>
+      </c>
+      <c r="X18" t="str">
+        <v/>
+      </c>
+      <c r="Y18" t="str">
+        <v/>
+      </c>
+      <c r="Z18" t="str">
+        <v/>
+      </c>
+      <c r="AA18" t="str">
+        <v/>
+      </c>
+      <c r="AB18" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB18"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "indgreb" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB18"/>
+  <dimension ref="A1:AB19"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -1979,9 +1979,95 @@
         <v/>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>71eb02a5-f505-41e4-b9a7-2dd955f74d3e</v>
+      </c>
+      <c r="B19" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C19" t="str">
+        <v>indgreb</v>
+      </c>
+      <c r="D19" t="str">
+        <v>indgreb</v>
+      </c>
+      <c r="E19" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F19" t="str">
+        <v>et</v>
+      </c>
+      <c r="G19" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v>https://static.ordnet.dk/mp3/11023/11023304_1.mp3</v>
+      </c>
+      <c r="J19" t="str">
+        <v>handling hvormed man blander sig i noget for at ændre den aktuelle situation</v>
+      </c>
+      <c r="K19" t="str">
+        <v>intervention</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Datacentre jagter sort energi efter politisk indgreb: »Det vil være en katastrofe«</v>
+      </c>
+      <c r="M19" t="str">
+        <v>AI-lyskryds fjerner bilkøer på vejene: Men nogle må holde længe for rødt - yihengldavid@gmail.com - Gmail</v>
+      </c>
+      <c r="N19" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
+      </c>
+      <c r="O19" t="str">
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=indgreb</v>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
+      <c r="U19" t="str">
+        <v/>
+      </c>
+      <c r="V19" t="str">
+        <v/>
+      </c>
+      <c r="W19" t="str">
+        <v/>
+      </c>
+      <c r="X19" t="str">
+        <v/>
+      </c>
+      <c r="Y19" t="str">
+        <v/>
+      </c>
+      <c r="Z19" t="str">
+        <v/>
+      </c>
+      <c r="AA19" t="str">
+        <v/>
+      </c>
+      <c r="AB19" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "afslørede" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB19"/>
+  <dimension ref="A1:AB20"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2065,9 +2065,95 @@
         <v/>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>fcee3e04-b744-426b-9a14-215fcad6e55b</v>
+      </c>
+      <c r="B20" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C20" t="str">
+        <v>afslørede</v>
+      </c>
+      <c r="D20" t="str">
+        <v>afsløre</v>
+      </c>
+      <c r="E20" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H20" t="str">
+        <v>[-ˌsløˀʌ]</v>
+      </c>
+      <c r="I20" t="str">
+        <v>https://static.ordnet.dk/mp3/11000/11000720_1.mp3</v>
+      </c>
+      <c r="J20" t="str">
+        <v>opdage at nogen har begået en (kriminel eller uhæderlig) handling eller har en egenskab eller fortid som vedkommende har forsøgt at skjule</v>
+      </c>
+      <c r="K20" t="str">
+        <v>revealed</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark | Ingeniøren</v>
+      </c>
+      <c r="N20" t="str">
+        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
+      </c>
+      <c r="O20" t="str">
+        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=afsl%C3%B8rede</v>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20" t="str">
+        <v/>
+      </c>
+      <c r="T20" t="str">
+        <v/>
+      </c>
+      <c r="U20" t="str">
+        <v/>
+      </c>
+      <c r="V20" t="str">
+        <v/>
+      </c>
+      <c r="W20" t="str">
+        <v/>
+      </c>
+      <c r="X20" t="str">
+        <v/>
+      </c>
+      <c r="Y20" t="str">
+        <v/>
+      </c>
+      <c r="Z20" t="str">
+        <v/>
+      </c>
+      <c r="AA20" t="str">
+        <v/>
+      </c>
+      <c r="AB20" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "lovbrud" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB20"/>
+  <dimension ref="A1:AB21"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2151,9 +2151,95 @@
         <v/>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>23d95731-816a-467a-a38d-9e6f6a7dced9</v>
+      </c>
+      <c r="B21" t="str">
+        <v>2026-07-02</v>
+      </c>
+      <c r="C21" t="str">
+        <v>lovbrud</v>
+      </c>
+      <c r="D21" t="str">
+        <v>lovbrud</v>
+      </c>
+      <c r="E21" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F21" t="str">
+        <v>et</v>
+      </c>
+      <c r="G21" t="str">
+        <v>-det, -, -dene</v>
+      </c>
+      <c r="H21" t="str">
+        <v>[-ˌbʁuð]</v>
+      </c>
+      <c r="I21" t="str">
+        <v>https://static.ordnet.dk/mp3/11030/11030992_1.mp3</v>
+      </c>
+      <c r="J21" t="str">
+        <v>det at bryde loven; overtrædelse af loven</v>
+      </c>
+      <c r="K21" t="str">
+        <v>violation of law</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark | Ingeniøren</v>
+      </c>
+      <c r="N21" t="str">
+        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
+      </c>
+      <c r="O21" t="str">
+        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=lovbrud</v>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R21" t="str">
+        <v/>
+      </c>
+      <c r="S21" t="str">
+        <v/>
+      </c>
+      <c r="T21" t="str">
+        <v/>
+      </c>
+      <c r="U21" t="str">
+        <v/>
+      </c>
+      <c r="V21" t="str">
+        <v/>
+      </c>
+      <c r="W21" t="str">
+        <v/>
+      </c>
+      <c r="X21" t="str">
+        <v/>
+      </c>
+      <c r="Y21" t="str">
+        <v/>
+      </c>
+      <c r="Z21" t="str">
+        <v/>
+      </c>
+      <c r="AA21" t="str">
+        <v/>
+      </c>
+      <c r="AB21" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB21"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: progress 1, log 1 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Words" sheetId="1" r:id="rId1"/>
     <sheet name="Phrases" sheetId="2" r:id="rId2"/>
     <sheet name="Meta" sheetId="3" r:id="rId3"/>
+    <sheet name="ReviewLog" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -123,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,36 +400,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB21"/>
+  <dimension ref="A1:AH21"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="29" max="29" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="11.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -516,6 +523,24 @@
       <c r="AB1" t="str">
         <v>Lapses_EN</v>
       </c>
+      <c r="AC1" t="str">
+        <v>Stability</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>Difficulty</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>LastReview</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>Stability_EN</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>Difficulty_EN</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>LastReview_EN</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1347,19 +1372,19 @@
         <v/>
       </c>
       <c r="S11" t="str">
-        <v/>
+        <v>2026-07-03</v>
       </c>
       <c r="T11" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="U11" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V11" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="W11" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X11" t="str">
         <v/>
@@ -1375,6 +1400,15 @@
       </c>
       <c r="AB11" t="str">
         <v/>
+      </c>
+      <c r="AC11" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="AD11" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="AE11" t="str">
+        <v>2026-07-03</v>
       </c>
     </row>
     <row r="12">
@@ -2239,14 +2273,14 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:AB2"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="10.83203125"/>
     <col min="2" max="2" customWidth="1" width="11.83203125"/>
@@ -2270,6 +2304,12 @@
     <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
     <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
     <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="23" max="23" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="11.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2339,6 +2379,24 @@
       <c r="V1" t="str">
         <v>Lapses_EN</v>
       </c>
+      <c r="W1" t="str">
+        <v>Stability</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Difficulty</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>LastReview</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>Stability_EN</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>Difficulty_EN</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>LastReview_EN</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -2410,7 +2468,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2460,4 +2518,77 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H2"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Dir</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Time</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Grade</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Elapsed</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Stability</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Difficulty</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Interval</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
+      </c>
+      <c r="B2" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-07-03T04:41:15.141Z</v>
+      </c>
+      <c r="D2" t="str">
+        <v>again</v>
+      </c>
+      <c r="E2" t="str">
+        <v>0</v>
+      </c>
+      <c r="F2" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G2" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H2" t="str">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add phrase "tunge maskiner" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -2289,36 +2289,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AB3"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2475,9 +2475,95 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>1e5fc340-099b-4123-bd6d-fd6305ee96d7</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-07-03</v>
+      </c>
+      <c r="C3" t="str">
+        <v>tunge maskiner</v>
+      </c>
+      <c r="D3" t="str">
+        <v>tunge=tongue · maskiner=machines</v>
+      </c>
+      <c r="E3" t="str">
+        <v>heavy machinery</v>
+      </c>
+      <c r="F3" t="str">
+        <v>På dyrkede marker rundt om i landet bliver jorden vendt, så gødet, så sprøjtet og så høstet. Alt sammen med store, tunge maskiner.</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb | Ingeniøren</v>
+      </c>
+      <c r="H3" t="str">
+        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb</v>
+      </c>
+      <c r="I3" t="str">
+        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb#:~:text=tunge%20maskiner</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: progress 2, log 2 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1123,19 +1123,19 @@
         <v/>
       </c>
       <c r="S8" t="str">
-        <v/>
+        <v>2026-07-04</v>
       </c>
       <c r="T8" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="U8" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V8" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="W8" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X8" t="str">
         <v/>
@@ -1151,6 +1151,15 @@
       </c>
       <c r="AB8" t="str">
         <v/>
+      </c>
+      <c r="AC8" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="AD8" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="AE8" t="str">
+        <v>2026-07-04</v>
       </c>
     </row>
     <row r="9">
@@ -1209,19 +1218,19 @@
         <v/>
       </c>
       <c r="S9" t="str">
-        <v/>
+        <v>2026-07-05</v>
       </c>
       <c r="T9" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U9" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V9" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W9" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X9" t="str">
         <v/>
@@ -1237,6 +1246,15 @@
       </c>
       <c r="AB9" t="str">
         <v/>
+      </c>
+      <c r="AC9" t="str">
+        <v>1.18</v>
+      </c>
+      <c r="AD9" t="str">
+        <v>6.49</v>
+      </c>
+      <c r="AE9" t="str">
+        <v>2026-07-04</v>
       </c>
     </row>
     <row r="10">
@@ -2291,34 +2309,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB3"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2617,7 +2635,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -2707,9 +2725,61 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>0254c900-1cbd-4360-853b-baf63aadaf10</v>
+      </c>
+      <c r="B4" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-07-04T19:04:13.878Z</v>
+      </c>
+      <c r="D4" t="str">
+        <v>again</v>
+      </c>
+      <c r="E4" t="str">
+        <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G4" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H4" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>8732aac0-4d2b-43cc-9af1-60bf3151752b</v>
+      </c>
+      <c r="B5" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2026-07-04T19:04:24.398Z</v>
+      </c>
+      <c r="D5" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E5" t="str">
+        <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <v>1.18</v>
+      </c>
+      <c r="G5" t="str">
+        <v>6.49</v>
+      </c>
+      <c r="H5" t="str">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 2, log 6 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -598,19 +598,19 @@
         <v/>
       </c>
       <c r="S2" t="str">
-        <v/>
+        <v>2026-07-20</v>
       </c>
       <c r="T2" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="U2" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V2" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="W2" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X2" t="str">
         <v/>
@@ -626,6 +626,15 @@
       </c>
       <c r="AB2" t="str">
         <v/>
+      </c>
+      <c r="AC2" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="AD2" t="str">
+        <v>8.68</v>
+      </c>
+      <c r="AE2" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="3">
@@ -779,19 +788,19 @@
         <v/>
       </c>
       <c r="S4" t="str">
-        <v/>
+        <v>2026-07-21</v>
       </c>
       <c r="T4" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U4" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V4" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W4" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X4" t="str">
         <v/>
@@ -807,6 +816,15 @@
       </c>
       <c r="AB4" t="str">
         <v/>
+      </c>
+      <c r="AC4" t="str">
+        <v>0.17</v>
+      </c>
+      <c r="AD4" t="str">
+        <v>8.37</v>
+      </c>
+      <c r="AE4" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="5">
@@ -2635,7 +2653,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H11"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -2777,9 +2795,165 @@
         <v>1</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>6cebe36d-5d01-40b2-906b-8a829745c73d</v>
+      </c>
+      <c r="B6" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C6" t="str">
+        <v>2026-07-20T10:30:37.900Z</v>
+      </c>
+      <c r="D6" t="str">
+        <v>again</v>
+      </c>
+      <c r="E6" t="str">
+        <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G6" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H6" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>05d5014c-1bc9-48f5-ac80-9c6659843c67</v>
+      </c>
+      <c r="B7" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C7" t="str">
+        <v>2026-07-20T10:30:46.071Z</v>
+      </c>
+      <c r="D7" t="str">
+        <v>again</v>
+      </c>
+      <c r="E7" t="str">
+        <v>0</v>
+      </c>
+      <c r="F7" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G7" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H7" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>6cebe36d-5d01-40b2-906b-8a829745c73d</v>
+      </c>
+      <c r="B8" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C8" t="str">
+        <v>2026-07-20T10:31:01.140Z</v>
+      </c>
+      <c r="D8" t="str">
+        <v>again</v>
+      </c>
+      <c r="E8" t="str">
+        <v>0</v>
+      </c>
+      <c r="F8" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="G8" t="str">
+        <v>8.08</v>
+      </c>
+      <c r="H8" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>05d5014c-1bc9-48f5-ac80-9c6659843c67</v>
+      </c>
+      <c r="B9" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C9" t="str">
+        <v>2026-07-20T10:31:05.593Z</v>
+      </c>
+      <c r="D9" t="str">
+        <v>again</v>
+      </c>
+      <c r="E9" t="str">
+        <v>0</v>
+      </c>
+      <c r="F9" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="G9" t="str">
+        <v>8.08</v>
+      </c>
+      <c r="H9" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>6cebe36d-5d01-40b2-906b-8a829745c73d</v>
+      </c>
+      <c r="B10" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C10" t="str">
+        <v>2026-07-20T10:31:18.399Z</v>
+      </c>
+      <c r="D10" t="str">
+        <v>again</v>
+      </c>
+      <c r="E10" t="str">
+        <v>0</v>
+      </c>
+      <c r="F10" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="G10" t="str">
+        <v>8.68</v>
+      </c>
+      <c r="H10" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>05d5014c-1bc9-48f5-ac80-9c6659843c67</v>
+      </c>
+      <c r="B11" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C11" t="str">
+        <v>2026-07-20T10:31:27.137Z</v>
+      </c>
+      <c r="D11" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E11" t="str">
+        <v>0</v>
+      </c>
+      <c r="F11" t="str">
+        <v>0.17</v>
+      </c>
+      <c r="G11" t="str">
+        <v>8.37</v>
+      </c>
+      <c r="H11" t="str">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 3, log 5 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -598,16 +598,16 @@
         <v/>
       </c>
       <c r="S2" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-21</v>
       </c>
       <c r="T2" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2" t="str">
         <v>2.5</v>
       </c>
       <c r="V2" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W2" t="str">
         <v>0</v>
@@ -628,10 +628,10 @@
         <v/>
       </c>
       <c r="AC2" t="str">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="AD2" t="str">
-        <v>8.68</v>
+        <v>8.87</v>
       </c>
       <c r="AE2" t="str">
         <v>2026-07-20</v>
@@ -969,19 +969,19 @@
         <v/>
       </c>
       <c r="S6" t="str">
-        <v/>
+        <v>2026-07-20</v>
       </c>
       <c r="T6" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="U6" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V6" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="W6" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X6" t="str">
         <v/>
@@ -997,6 +997,15 @@
       </c>
       <c r="AB6" t="str">
         <v/>
+      </c>
+      <c r="AC6" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="AD6" t="str">
+        <v>8.68</v>
+      </c>
+      <c r="AE6" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="7">
@@ -1770,19 +1779,19 @@
         <v/>
       </c>
       <c r="S15" t="str">
-        <v/>
+        <v>2026-07-20</v>
       </c>
       <c r="T15" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="U15" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V15" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="W15" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X15" t="str">
         <v/>
@@ -1798,6 +1807,15 @@
       </c>
       <c r="AB15" t="str">
         <v/>
+      </c>
+      <c r="AC15" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="AD15" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="AE15" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="16">
@@ -2653,7 +2671,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H16"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -2951,9 +2969,139 @@
         <v>1</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>6cebe36d-5d01-40b2-906b-8a829745c73d</v>
+      </c>
+      <c r="B12" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C12" t="str">
+        <v>2026-07-20T10:31:42.725Z</v>
+      </c>
+      <c r="D12" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E12" t="str">
+        <v>0</v>
+      </c>
+      <c r="F12" t="str">
+        <v>0.08</v>
+      </c>
+      <c r="G12" t="str">
+        <v>8.87</v>
+      </c>
+      <c r="H12" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B13" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C13" t="str">
+        <v>2026-07-20T10:32:39.566Z</v>
+      </c>
+      <c r="D13" t="str">
+        <v>again</v>
+      </c>
+      <c r="E13" t="str">
+        <v>0</v>
+      </c>
+      <c r="F13" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G13" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H13" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B14" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C14" t="str">
+        <v>2026-07-20T10:32:54.593Z</v>
+      </c>
+      <c r="D14" t="str">
+        <v>again</v>
+      </c>
+      <c r="E14" t="str">
+        <v>0</v>
+      </c>
+      <c r="F14" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="G14" t="str">
+        <v>8.08</v>
+      </c>
+      <c r="H14" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B15" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C15" t="str">
+        <v>2026-07-20T10:34:20.384Z</v>
+      </c>
+      <c r="D15" t="str">
+        <v>again</v>
+      </c>
+      <c r="E15" t="str">
+        <v>0</v>
+      </c>
+      <c r="F15" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="G15" t="str">
+        <v>8.68</v>
+      </c>
+      <c r="H15" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>6d8e9813-5550-45ab-9874-78033b6c2cd6</v>
+      </c>
+      <c r="B16" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C16" t="str">
+        <v>2026-07-20T10:35:56.493Z</v>
+      </c>
+      <c r="D16" t="str">
+        <v>again</v>
+      </c>
+      <c r="E16" t="str">
+        <v>0</v>
+      </c>
+      <c r="F16" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G16" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H16" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 4, log 5 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -969,16 +969,16 @@
         <v/>
       </c>
       <c r="S6" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-21</v>
       </c>
       <c r="T6" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U6" t="str">
         <v>2.5</v>
       </c>
       <c r="V6" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W6" t="str">
         <v>0</v>
@@ -999,10 +999,10 @@
         <v/>
       </c>
       <c r="AC6" t="str">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="AD6" t="str">
-        <v>8.68</v>
+        <v>8.87</v>
       </c>
       <c r="AE6" t="str">
         <v>2026-07-20</v>
@@ -1150,16 +1150,16 @@
         <v/>
       </c>
       <c r="S8" t="str">
-        <v>2026-07-04</v>
+        <v>2026-07-29</v>
       </c>
       <c r="T8" t="str">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="U8" t="str">
         <v>2.5</v>
       </c>
       <c r="V8" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W8" t="str">
         <v>0</v>
@@ -1180,13 +1180,13 @@
         <v/>
       </c>
       <c r="AC8" t="str">
-        <v>0.4</v>
+        <v>8.57</v>
       </c>
       <c r="AD8" t="str">
-        <v>7.19</v>
+        <v>7.17</v>
       </c>
       <c r="AE8" t="str">
-        <v>2026-07-04</v>
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="9">
@@ -1340,19 +1340,19 @@
         <v/>
       </c>
       <c r="S10" t="str">
-        <v/>
+        <v>2026-07-20</v>
       </c>
       <c r="T10" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="U10" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V10" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="W10" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X10" t="str">
         <v/>
@@ -1368,6 +1368,15 @@
       </c>
       <c r="AB10" t="str">
         <v/>
+      </c>
+      <c r="AC10" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="AD10" t="str">
+        <v>8.08</v>
+      </c>
+      <c r="AE10" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="11">
@@ -1779,16 +1788,16 @@
         <v/>
       </c>
       <c r="S15" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-21</v>
       </c>
       <c r="T15" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U15" t="str">
         <v>2.5</v>
       </c>
       <c r="V15" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W15" t="str">
         <v>0</v>
@@ -1809,10 +1818,10 @@
         <v/>
       </c>
       <c r="AC15" t="str">
-        <v>0.4</v>
+        <v>0.56</v>
       </c>
       <c r="AD15" t="str">
-        <v>7.19</v>
+        <v>7.17</v>
       </c>
       <c r="AE15" t="str">
         <v>2026-07-20</v>
@@ -2671,7 +2680,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H21"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -3099,9 +3108,139 @@
         <v>0</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B17" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C17" t="str">
+        <v>2026-07-20T10:36:22.486Z</v>
+      </c>
+      <c r="D17" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E17" t="str">
+        <v>0</v>
+      </c>
+      <c r="F17" t="str">
+        <v>0.08</v>
+      </c>
+      <c r="G17" t="str">
+        <v>8.87</v>
+      </c>
+      <c r="H17" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>6d8e9813-5550-45ab-9874-78033b6c2cd6</v>
+      </c>
+      <c r="B18" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C18" t="str">
+        <v>2026-07-20T10:36:28.769Z</v>
+      </c>
+      <c r="D18" t="str">
+        <v>good</v>
+      </c>
+      <c r="E18" t="str">
+        <v>0</v>
+      </c>
+      <c r="F18" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="G18" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="H18" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>0254c900-1cbd-4360-853b-baf63aadaf10</v>
+      </c>
+      <c r="B19" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C19" t="str">
+        <v>2026-07-20T10:36:31.202Z</v>
+      </c>
+      <c r="D19" t="str">
+        <v>good</v>
+      </c>
+      <c r="E19" t="str">
+        <v>16</v>
+      </c>
+      <c r="F19" t="str">
+        <v>8.57</v>
+      </c>
+      <c r="G19" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="H19" t="str">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>0933c06d-fcdc-4401-9d43-79f732aadad7</v>
+      </c>
+      <c r="B20" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C20" t="str">
+        <v>2026-07-20T10:37:38.905Z</v>
+      </c>
+      <c r="D20" t="str">
+        <v>again</v>
+      </c>
+      <c r="E20" t="str">
+        <v>0</v>
+      </c>
+      <c r="F20" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G20" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H20" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>0933c06d-fcdc-4401-9d43-79f732aadad7</v>
+      </c>
+      <c r="B21" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C21" t="str">
+        <v>2026-07-20T10:38:15.073Z</v>
+      </c>
+      <c r="D21" t="str">
+        <v>again</v>
+      </c>
+      <c r="E21" t="str">
+        <v>0</v>
+      </c>
+      <c r="F21" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="G21" t="str">
+        <v>8.08</v>
+      </c>
+      <c r="H21" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 2, log 4 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -883,19 +883,19 @@
         <v/>
       </c>
       <c r="S5" t="str">
-        <v/>
+        <v>2026-07-21</v>
       </c>
       <c r="T5" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U5" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V5" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W5" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X5" t="str">
         <v/>
@@ -911,6 +911,15 @@
       </c>
       <c r="AB5" t="str">
         <v/>
+      </c>
+      <c r="AC5" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="AD5" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="AE5" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="6">
@@ -1340,16 +1349,16 @@
         <v/>
       </c>
       <c r="S10" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-21</v>
       </c>
       <c r="T10" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U10" t="str">
         <v>2.5</v>
       </c>
       <c r="V10" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W10" t="str">
         <v>0</v>
@@ -1370,10 +1379,10 @@
         <v/>
       </c>
       <c r="AC10" t="str">
-        <v>0.2</v>
+        <v>0.14</v>
       </c>
       <c r="AD10" t="str">
-        <v>8.08</v>
+        <v>8.65</v>
       </c>
       <c r="AE10" t="str">
         <v>2026-07-20</v>
@@ -2680,7 +2689,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H25"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -3238,9 +3247,113 @@
         <v>0</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>0933c06d-fcdc-4401-9d43-79f732aadad7</v>
+      </c>
+      <c r="B22" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C22" t="str">
+        <v>2026-07-20T10:39:23.573Z</v>
+      </c>
+      <c r="D22" t="str">
+        <v>again</v>
+      </c>
+      <c r="E22" t="str">
+        <v>0</v>
+      </c>
+      <c r="F22" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="G22" t="str">
+        <v>8.68</v>
+      </c>
+      <c r="H22" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>0933c06d-fcdc-4401-9d43-79f732aadad7</v>
+      </c>
+      <c r="B23" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C23" t="str">
+        <v>2026-07-20T10:39:41.443Z</v>
+      </c>
+      <c r="D23" t="str">
+        <v>good</v>
+      </c>
+      <c r="E23" t="str">
+        <v>0</v>
+      </c>
+      <c r="F23" t="str">
+        <v>0.14</v>
+      </c>
+      <c r="G23" t="str">
+        <v>8.65</v>
+      </c>
+      <c r="H23" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>956f08a1-4407-41d9-9dec-b137931c6d72</v>
+      </c>
+      <c r="B24" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C24" t="str">
+        <v>2026-07-20T10:40:07.074Z</v>
+      </c>
+      <c r="D24" t="str">
+        <v>again</v>
+      </c>
+      <c r="E24" t="str">
+        <v>0</v>
+      </c>
+      <c r="F24" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G24" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H24" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>956f08a1-4407-41d9-9dec-b137931c6d72</v>
+      </c>
+      <c r="B25" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C25" t="str">
+        <v>2026-07-20T10:40:35.017Z</v>
+      </c>
+      <c r="D25" t="str">
+        <v>good</v>
+      </c>
+      <c r="E25" t="str">
+        <v>0</v>
+      </c>
+      <c r="F25" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="G25" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="H25" t="str">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 4, log 8 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1073,19 +1073,19 @@
         <v/>
       </c>
       <c r="S7" t="str">
-        <v/>
+        <v>2026-07-20</v>
       </c>
       <c r="T7" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="U7" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V7" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="W7" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X7" t="str">
         <v/>
@@ -1101,6 +1101,15 @@
       </c>
       <c r="AB7" t="str">
         <v/>
+      </c>
+      <c r="AC7" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="AD7" t="str">
+        <v>8.68</v>
+      </c>
+      <c r="AE7" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="8">
@@ -1254,20 +1263,20 @@
         <v/>
       </c>
       <c r="S9" t="str">
-        <v>2026-07-05</v>
+        <v>2026-07-20</v>
       </c>
       <c r="T9" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U9" t="str">
         <v>2.5</v>
       </c>
       <c r="V9" t="str">
+        <v>0</v>
+      </c>
+      <c r="W9" t="str">
         <v>1</v>
       </c>
-      <c r="W9" t="str">
-        <v>0</v>
-      </c>
       <c r="X9" t="str">
         <v/>
       </c>
@@ -1284,13 +1293,13 @@
         <v/>
       </c>
       <c r="AC9" t="str">
-        <v>1.18</v>
+        <v>0.59</v>
       </c>
       <c r="AD9" t="str">
-        <v>6.49</v>
+        <v>8.36</v>
       </c>
       <c r="AE9" t="str">
-        <v>2026-07-04</v>
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="10">
@@ -1625,19 +1634,19 @@
         <v/>
       </c>
       <c r="S13" t="str">
-        <v/>
+        <v>2026-07-23</v>
       </c>
       <c r="T13" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="U13" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V13" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W13" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X13" t="str">
         <v/>
@@ -1653,6 +1662,15 @@
       </c>
       <c r="AB13" t="str">
         <v/>
+      </c>
+      <c r="AC13" t="str">
+        <v>3.17</v>
+      </c>
+      <c r="AD13" t="str">
+        <v>5.28</v>
+      </c>
+      <c r="AE13" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="14">
@@ -1711,19 +1729,19 @@
         <v/>
       </c>
       <c r="S14" t="str">
-        <v/>
+        <v>2026-07-21</v>
       </c>
       <c r="T14" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U14" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V14" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W14" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X14" t="str">
         <v/>
@@ -1739,6 +1757,15 @@
       </c>
       <c r="AB14" t="str">
         <v/>
+      </c>
+      <c r="AC14" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="AD14" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="AE14" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="15">
@@ -2689,7 +2716,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H33"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -3351,9 +3378,217 @@
         <v>1</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>8e0306d1-6036-4774-8e44-a607339a1174</v>
+      </c>
+      <c r="B26" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C26" t="str">
+        <v>2026-07-20T10:41:16.980Z</v>
+      </c>
+      <c r="D26" t="str">
+        <v>again</v>
+      </c>
+      <c r="E26" t="str">
+        <v>0</v>
+      </c>
+      <c r="F26" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G26" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H26" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>03f5e6c8-8aee-4335-872b-3d6af367eeee</v>
+      </c>
+      <c r="B27" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C27" t="str">
+        <v>2026-07-20T10:41:26.114Z</v>
+      </c>
+      <c r="D27" t="str">
+        <v>again</v>
+      </c>
+      <c r="E27" t="str">
+        <v>0</v>
+      </c>
+      <c r="F27" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G27" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H27" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>8732aac0-4d2b-43cc-9af1-60bf3151752b</v>
+      </c>
+      <c r="B28" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C28" t="str">
+        <v>2026-07-20T10:41:29.064Z</v>
+      </c>
+      <c r="D28" t="str">
+        <v>again</v>
+      </c>
+      <c r="E28" t="str">
+        <v>16</v>
+      </c>
+      <c r="F28" t="str">
+        <v>1.18</v>
+      </c>
+      <c r="G28" t="str">
+        <v>7.61</v>
+      </c>
+      <c r="H28" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>8e0306d1-6036-4774-8e44-a607339a1174</v>
+      </c>
+      <c r="B29" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C29" t="str">
+        <v>2026-07-20T10:41:40.386Z</v>
+      </c>
+      <c r="D29" t="str">
+        <v>again</v>
+      </c>
+      <c r="E29" t="str">
+        <v>0</v>
+      </c>
+      <c r="F29" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="G29" t="str">
+        <v>8.08</v>
+      </c>
+      <c r="H29" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>03f5e6c8-8aee-4335-872b-3d6af367eeee</v>
+      </c>
+      <c r="B30" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C30" t="str">
+        <v>2026-07-20T10:42:04.775Z</v>
+      </c>
+      <c r="D30" t="str">
+        <v>good</v>
+      </c>
+      <c r="E30" t="str">
+        <v>0</v>
+      </c>
+      <c r="F30" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="G30" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="H30" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>8732aac0-4d2b-43cc-9af1-60bf3151752b</v>
+      </c>
+      <c r="B31" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C31" t="str">
+        <v>2026-07-20T10:42:45.840Z</v>
+      </c>
+      <c r="D31" t="str">
+        <v>again</v>
+      </c>
+      <c r="E31" t="str">
+        <v>0</v>
+      </c>
+      <c r="F31" t="str">
+        <v>0.59</v>
+      </c>
+      <c r="G31" t="str">
+        <v>8.36</v>
+      </c>
+      <c r="H31" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>8e0306d1-6036-4774-8e44-a607339a1174</v>
+      </c>
+      <c r="B32" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C32" t="str">
+        <v>2026-07-20T10:42:50.555Z</v>
+      </c>
+      <c r="D32" t="str">
+        <v>again</v>
+      </c>
+      <c r="E32" t="str">
+        <v>0</v>
+      </c>
+      <c r="F32" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="G32" t="str">
+        <v>8.68</v>
+      </c>
+      <c r="H32" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>c2d45936-5793-42b4-968a-e066bcb27036</v>
+      </c>
+      <c r="B33" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C33" t="str">
+        <v>2026-07-20T10:42:54.157Z</v>
+      </c>
+      <c r="D33" t="str">
+        <v>good</v>
+      </c>
+      <c r="E33" t="str">
+        <v>0</v>
+      </c>
+      <c r="F33" t="str">
+        <v>3.17</v>
+      </c>
+      <c r="G33" t="str">
+        <v>5.28</v>
+      </c>
+      <c r="H33" t="str">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H33"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 5, log 8 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -693,16 +693,16 @@
         <v/>
       </c>
       <c r="S3" t="str">
-        <v>2026-07-03</v>
+        <v>2026-07-21</v>
       </c>
       <c r="T3" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U3" t="str">
         <v>2.5</v>
       </c>
       <c r="V3" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W3" t="str">
         <v>0</v>
@@ -723,13 +723,13 @@
         <v/>
       </c>
       <c r="AC3" t="str">
-        <v>0.4</v>
+        <v>0.56</v>
       </c>
       <c r="AD3" t="str">
-        <v>7.19</v>
+        <v>8.06</v>
       </c>
       <c r="AE3" t="str">
-        <v>2026-07-03</v>
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="4">
@@ -1073,16 +1073,16 @@
         <v/>
       </c>
       <c r="S7" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-21</v>
       </c>
       <c r="T7" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U7" t="str">
         <v>2.5</v>
       </c>
       <c r="V7" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W7" t="str">
         <v>0</v>
@@ -1103,10 +1103,10 @@
         <v/>
       </c>
       <c r="AC7" t="str">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="AD7" t="str">
-        <v>8.68</v>
+        <v>8.87</v>
       </c>
       <c r="AE7" t="str">
         <v>2026-07-20</v>
@@ -1263,16 +1263,16 @@
         <v/>
       </c>
       <c r="S9" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-21</v>
       </c>
       <c r="T9" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U9" t="str">
         <v>2.5</v>
       </c>
       <c r="V9" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W9" t="str">
         <v>1</v>
@@ -1293,10 +1293,10 @@
         <v/>
       </c>
       <c r="AC9" t="str">
-        <v>0.59</v>
+        <v>0.5</v>
       </c>
       <c r="AD9" t="str">
-        <v>8.36</v>
+        <v>8.6</v>
       </c>
       <c r="AE9" t="str">
         <v>2026-07-20</v>
@@ -1453,16 +1453,16 @@
         <v/>
       </c>
       <c r="S11" t="str">
-        <v>2026-07-03</v>
+        <v>2026-07-21</v>
       </c>
       <c r="T11" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U11" t="str">
         <v>2.5</v>
       </c>
       <c r="V11" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W11" t="str">
         <v>0</v>
@@ -1483,13 +1483,13 @@
         <v/>
       </c>
       <c r="AC11" t="str">
-        <v>0.4</v>
+        <v>0.28</v>
       </c>
       <c r="AD11" t="str">
-        <v>7.19</v>
+        <v>8.65</v>
       </c>
       <c r="AE11" t="str">
-        <v>2026-07-03</v>
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="12">
@@ -1548,19 +1548,19 @@
         <v/>
       </c>
       <c r="S12" t="str">
-        <v/>
+        <v>2026-07-23</v>
       </c>
       <c r="T12" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="U12" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V12" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W12" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X12" t="str">
         <v/>
@@ -1576,6 +1576,15 @@
       </c>
       <c r="AB12" t="str">
         <v/>
+      </c>
+      <c r="AC12" t="str">
+        <v>3.17</v>
+      </c>
+      <c r="AD12" t="str">
+        <v>5.28</v>
+      </c>
+      <c r="AE12" t="str">
+        <v>2026-07-20</v>
       </c>
     </row>
     <row r="13">
@@ -2716,7 +2725,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H41"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -3586,9 +3595,217 @@
         <v>3</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>8732aac0-4d2b-43cc-9af1-60bf3151752b</v>
+      </c>
+      <c r="B34" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C34" t="str">
+        <v>2026-07-20T10:42:58.563Z</v>
+      </c>
+      <c r="D34" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E34" t="str">
+        <v>0</v>
+      </c>
+      <c r="F34" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="G34" t="str">
+        <v>8.6</v>
+      </c>
+      <c r="H34" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>8e0306d1-6036-4774-8e44-a607339a1174</v>
+      </c>
+      <c r="B35" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C35" t="str">
+        <v>2026-07-20T10:43:02.780Z</v>
+      </c>
+      <c r="D35" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E35" t="str">
+        <v>0</v>
+      </c>
+      <c r="F35" t="str">
+        <v>0.08</v>
+      </c>
+      <c r="G35" t="str">
+        <v>8.87</v>
+      </c>
+      <c r="H35" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>87f910eb-6aa4-4751-ad3a-14ec49047ac6</v>
+      </c>
+      <c r="B36" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C36" t="str">
+        <v>2026-07-20T10:43:07.479Z</v>
+      </c>
+      <c r="D36" t="str">
+        <v>good</v>
+      </c>
+      <c r="E36" t="str">
+        <v>0</v>
+      </c>
+      <c r="F36" t="str">
+        <v>3.17</v>
+      </c>
+      <c r="G36" t="str">
+        <v>5.28</v>
+      </c>
+      <c r="H36" t="str">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>0d3fc2e5-0c30-4cd1-a873-0cdfc98007a4</v>
+      </c>
+      <c r="B37" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C37" t="str">
+        <v>2026-07-20T10:43:27.509Z</v>
+      </c>
+      <c r="D37" t="str">
+        <v>again</v>
+      </c>
+      <c r="E37" t="str">
+        <v>17</v>
+      </c>
+      <c r="F37" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G37" t="str">
+        <v>8.08</v>
+      </c>
+      <c r="H37" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>0d3fc2e5-0c30-4cd1-a873-0cdfc98007a4</v>
+      </c>
+      <c r="B38" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C38" t="str">
+        <v>2026-07-20T10:43:44.366Z</v>
+      </c>
+      <c r="D38" t="str">
+        <v>good</v>
+      </c>
+      <c r="E38" t="str">
+        <v>0</v>
+      </c>
+      <c r="F38" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="G38" t="str">
+        <v>8.06</v>
+      </c>
+      <c r="H38" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
+      </c>
+      <c r="B39" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C39" t="str">
+        <v>2026-07-20T10:44:00.434Z</v>
+      </c>
+      <c r="D39" t="str">
+        <v>again</v>
+      </c>
+      <c r="E39" t="str">
+        <v>17</v>
+      </c>
+      <c r="F39" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G39" t="str">
+        <v>8.08</v>
+      </c>
+      <c r="H39" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
+      </c>
+      <c r="B40" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C40" t="str">
+        <v>2026-07-20T10:44:04.869Z</v>
+      </c>
+      <c r="D40" t="str">
+        <v>again</v>
+      </c>
+      <c r="E40" t="str">
+        <v>0</v>
+      </c>
+      <c r="F40" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="G40" t="str">
+        <v>8.68</v>
+      </c>
+      <c r="H40" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
+      </c>
+      <c r="B41" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C41" t="str">
+        <v>2026-07-20T10:44:07.333Z</v>
+      </c>
+      <c r="D41" t="str">
+        <v>good</v>
+      </c>
+      <c r="E41" t="str">
+        <v>0</v>
+      </c>
+      <c r="F41" t="str">
+        <v>0.28</v>
+      </c>
+      <c r="G41" t="str">
+        <v>8.65</v>
+      </c>
+      <c r="H41" t="str">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H41"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add word "overvejer" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -400,42 +400,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH21"/>
+  <dimension ref="A1:AH22"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="29" max="29" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="30" max="30" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="31" max="31" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="32" max="32" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="33" max="33" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="34" max="34" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2388,9 +2388,113 @@
         <v/>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>039ba62e-8413-430f-ac17-4b365506303e</v>
+      </c>
+      <c r="B22" t="str">
+        <v>2026-07-22</v>
+      </c>
+      <c r="C22" t="str">
+        <v>overvejer</v>
+      </c>
+      <c r="D22" t="str">
+        <v>overveje</v>
+      </c>
+      <c r="E22" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H22" t="str">
+        <v>[-ˌvɑjˀə]</v>
+      </c>
+      <c r="I22" t="str">
+        <v>https://static.ordnet.dk/mp3/11038/11038552_1.mp3</v>
+      </c>
+      <c r="J22" t="str">
+        <v>tænke over noget eller tænke på at gøre noget idet man vurderer hvad der taler for og imod</v>
+      </c>
+      <c r="K22" t="str">
+        <v>reflect</v>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
+      <c r="S22" t="str">
+        <v/>
+      </c>
+      <c r="T22" t="str">
+        <v/>
+      </c>
+      <c r="U22" t="str">
+        <v/>
+      </c>
+      <c r="V22" t="str">
+        <v/>
+      </c>
+      <c r="W22" t="str">
+        <v/>
+      </c>
+      <c r="X22" t="str">
+        <v/>
+      </c>
+      <c r="Y22" t="str">
+        <v/>
+      </c>
+      <c r="Z22" t="str">
+        <v/>
+      </c>
+      <c r="AA22" t="str">
+        <v/>
+      </c>
+      <c r="AB22" t="str">
+        <v/>
+      </c>
+      <c r="AC22" t="str">
+        <v/>
+      </c>
+      <c r="AD22" t="str">
+        <v/>
+      </c>
+      <c r="AE22" t="str">
+        <v/>
+      </c>
+      <c r="AF22" t="str">
+        <v/>
+      </c>
+      <c r="AG22" t="str">
+        <v/>
+      </c>
+      <c r="AH22" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH22"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "Knapt" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH22"/>
+  <dimension ref="A1:AH23"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2492,9 +2492,113 @@
         <v/>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>c8b4f170-aa1f-4fe2-a8d4-5be8e34cc7a2</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-07-22</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Knapt</v>
+      </c>
+      <c r="D23" t="str">
+        <v>knap</v>
+      </c>
+      <c r="E23" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v>-t, -pe</v>
+      </c>
+      <c r="H23" t="str">
+        <v>[ˈknɑb]</v>
+      </c>
+      <c r="I23" t="str">
+        <v>https://static.ordnet.dk/mp3/11026/11026578_1.mp3</v>
+      </c>
+      <c r="J23" t="str">
+        <v>af begrænset eller ringe omfang eller mængde</v>
+      </c>
+      <c r="K23" t="str">
+        <v>barely</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse | SønderborgNYT</v>
+      </c>
+      <c r="N23" t="str">
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA</v>
+      </c>
+      <c r="O23" t="str">
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA#:~:text=Knapt</v>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str">
+        <v/>
+      </c>
+      <c r="V23" t="str">
+        <v/>
+      </c>
+      <c r="W23" t="str">
+        <v/>
+      </c>
+      <c r="X23" t="str">
+        <v/>
+      </c>
+      <c r="Y23" t="str">
+        <v/>
+      </c>
+      <c r="Z23" t="str">
+        <v/>
+      </c>
+      <c r="AA23" t="str">
+        <v/>
+      </c>
+      <c r="AB23" t="str">
+        <v/>
+      </c>
+      <c r="AC23" t="str">
+        <v/>
+      </c>
+      <c r="AD23" t="str">
+        <v/>
+      </c>
+      <c r="AE23" t="str">
+        <v/>
+      </c>
+      <c r="AF23" t="str">
+        <v/>
+      </c>
+      <c r="AG23" t="str">
+        <v/>
+      </c>
+      <c r="AH23" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "gennemsnit" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH23"/>
+  <dimension ref="A1:AH24"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2596,9 +2596,113 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>e370b465-1be4-4af6-9ce3-6dbf2118fc91</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-07-22</v>
+      </c>
+      <c r="C24" t="str">
+        <v>gennemsnit</v>
+      </c>
+      <c r="D24" t="str">
+        <v>gennemsnit</v>
+      </c>
+      <c r="E24" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F24" t="str">
+        <v>et</v>
+      </c>
+      <c r="G24" t="str">
+        <v>-tet, -, -tene</v>
+      </c>
+      <c r="H24" t="str">
+        <v>[ˈgεnəmˌsnid]</v>
+      </c>
+      <c r="I24" t="str">
+        <v>https://static.ordnet.dk/mp3/11017/11017684_1.mp3</v>
+      </c>
+      <c r="J24" t="str">
+        <v>værdi der fås ved at dividere en sammenlagt sum med antallet af værdier der indgår i den sammenlagte sum</v>
+      </c>
+      <c r="K24" t="str">
+        <v>average</v>
+      </c>
+      <c r="L24" t="str">
+        <v>375 studenter fra Sønderborg Kommune står uden en uddannelse fem år efter gymnasiet. Det svarer til knap hver tiende eller 9,5 procent. Selv om det er lidt under landsgennemsnittet på 10,3 procent, er andelen steget med to procentpoint siden 2020.</v>
+      </c>
+      <c r="M24" t="str">
+        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse | SønderborgNYT</v>
+      </c>
+      <c r="N24" t="str">
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA</v>
+      </c>
+      <c r="O24" t="str">
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA#:~:text=gennemsnit</v>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
+      <c r="U24" t="str">
+        <v/>
+      </c>
+      <c r="V24" t="str">
+        <v/>
+      </c>
+      <c r="W24" t="str">
+        <v/>
+      </c>
+      <c r="X24" t="str">
+        <v/>
+      </c>
+      <c r="Y24" t="str">
+        <v/>
+      </c>
+      <c r="Z24" t="str">
+        <v/>
+      </c>
+      <c r="AA24" t="str">
+        <v/>
+      </c>
+      <c r="AB24" t="str">
+        <v/>
+      </c>
+      <c r="AC24" t="str">
+        <v/>
+      </c>
+      <c r="AD24" t="str">
+        <v/>
+      </c>
+      <c r="AE24" t="str">
+        <v/>
+      </c>
+      <c r="AF24" t="str">
+        <v/>
+      </c>
+      <c r="AG24" t="str">
+        <v/>
+      </c>
+      <c r="AH24" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH24"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "steget med" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -402,40 +402,40 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AH24"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2709,36 +2709,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AB4"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2981,9 +2981,95 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>7bea74c7-5aab-4f05-909c-e9bdd96906fb</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-07-22</v>
+      </c>
+      <c r="C4" t="str">
+        <v>steget med</v>
+      </c>
+      <c r="D4" t="str">
+        <v>steget=increased · med=with</v>
+      </c>
+      <c r="E4" t="str">
+        <v>increased by</v>
+      </c>
+      <c r="F4" t="str">
+        <v>375 studenter fra Sønderborg Kommune står uden en uddannelse fem år efter gymnasiet. Det svarer til knap hver tiende eller 9,5 procent. Selv om det er lidt under landsgennemsnittet på 10,3 procent, er andelen steget med to procentpoint siden 2020.</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse | SønderborgNYT</v>
+      </c>
+      <c r="H4" t="str">
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA</v>
+      </c>
+      <c r="I4" t="str">
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA#:~:text=steget%20med</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: delete 1 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -400,42 +400,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH24"/>
+  <dimension ref="A1:AH23"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -636,6 +636,15 @@
       <c r="AE2" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF2" t="str">
+        <v/>
+      </c>
+      <c r="AG2" t="str">
+        <v/>
+      </c>
+      <c r="AH2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -731,6 +740,15 @@
       <c r="AE3" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF3" t="str">
+        <v/>
+      </c>
+      <c r="AG3" t="str">
+        <v/>
+      </c>
+      <c r="AH3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -826,6 +844,15 @@
       <c r="AE4" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF4" t="str">
+        <v/>
+      </c>
+      <c r="AG4" t="str">
+        <v/>
+      </c>
+      <c r="AH4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -921,6 +948,15 @@
       <c r="AE5" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF5" t="str">
+        <v/>
+      </c>
+      <c r="AG5" t="str">
+        <v/>
+      </c>
+      <c r="AH5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1016,6 +1052,15 @@
       <c r="AE6" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF6" t="str">
+        <v/>
+      </c>
+      <c r="AG6" t="str">
+        <v/>
+      </c>
+      <c r="AH6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1111,6 +1156,15 @@
       <c r="AE7" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF7" t="str">
+        <v/>
+      </c>
+      <c r="AG7" t="str">
+        <v/>
+      </c>
+      <c r="AH7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1206,6 +1260,15 @@
       <c r="AE8" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF8" t="str">
+        <v/>
+      </c>
+      <c r="AG8" t="str">
+        <v/>
+      </c>
+      <c r="AH8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -1301,6 +1364,15 @@
       <c r="AE9" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF9" t="str">
+        <v/>
+      </c>
+      <c r="AG9" t="str">
+        <v/>
+      </c>
+      <c r="AH9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -1396,6 +1468,15 @@
       <c r="AE10" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF10" t="str">
+        <v/>
+      </c>
+      <c r="AG10" t="str">
+        <v/>
+      </c>
+      <c r="AH10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -1491,6 +1572,15 @@
       <c r="AE11" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF11" t="str">
+        <v/>
+      </c>
+      <c r="AG11" t="str">
+        <v/>
+      </c>
+      <c r="AH11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1586,6 +1676,15 @@
       <c r="AE12" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF12" t="str">
+        <v/>
+      </c>
+      <c r="AG12" t="str">
+        <v/>
+      </c>
+      <c r="AH12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1681,6 +1780,15 @@
       <c r="AE13" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF13" t="str">
+        <v/>
+      </c>
+      <c r="AG13" t="str">
+        <v/>
+      </c>
+      <c r="AH13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1776,6 +1884,15 @@
       <c r="AE14" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF14" t="str">
+        <v/>
+      </c>
+      <c r="AG14" t="str">
+        <v/>
+      </c>
+      <c r="AH14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1871,6 +1988,15 @@
       <c r="AE15" t="str">
         <v>2026-07-20</v>
       </c>
+      <c r="AF15" t="str">
+        <v/>
+      </c>
+      <c r="AG15" t="str">
+        <v/>
+      </c>
+      <c r="AH15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1957,40 +2083,58 @@
       <c r="AB16" t="str">
         <v/>
       </c>
+      <c r="AC16" t="str">
+        <v/>
+      </c>
+      <c r="AD16" t="str">
+        <v/>
+      </c>
+      <c r="AE16" t="str">
+        <v/>
+      </c>
+      <c r="AF16" t="str">
+        <v/>
+      </c>
+      <c r="AG16" t="str">
+        <v/>
+      </c>
+      <c r="AH16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2ae5b453-b4ee-456f-8c22-324aba8103d0</v>
+        <v>94801dbf-f81c-46cc-a320-3e40b0903e79</v>
       </c>
       <c r="B17" t="str">
         <v>2026-07-02</v>
       </c>
       <c r="C17" t="str">
-        <v>To</v>
+        <v>Rådgivning</v>
       </c>
       <c r="D17" t="str">
-        <v>to.</v>
+        <v>rådgivning</v>
       </c>
       <c r="E17" t="str">
-        <v>forkortelse</v>
+        <v>substantiv</v>
       </c>
       <c r="F17" t="str">
-        <v/>
+        <v>en</v>
       </c>
       <c r="G17" t="str">
-        <v/>
+        <v>-en, -er, -erne</v>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>[ˈʁʌðˌgiwˀneŋ]</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>https://static.ordnet.dk/mp3/11044/11044289_1.mp3</v>
       </c>
       <c r="J17" t="str">
-        <v>= torsdag</v>
+        <v>det at rådgive</v>
       </c>
       <c r="K17" t="str">
-        <v>Two.</v>
+        <v>counseling</v>
       </c>
       <c r="L17" t="str">
         <v/>
@@ -2043,52 +2187,70 @@
       <c r="AB17" t="str">
         <v/>
       </c>
+      <c r="AC17" t="str">
+        <v/>
+      </c>
+      <c r="AD17" t="str">
+        <v/>
+      </c>
+      <c r="AE17" t="str">
+        <v/>
+      </c>
+      <c r="AF17" t="str">
+        <v/>
+      </c>
+      <c r="AG17" t="str">
+        <v/>
+      </c>
+      <c r="AH17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>94801dbf-f81c-46cc-a320-3e40b0903e79</v>
+        <v>71eb02a5-f505-41e4-b9a7-2dd955f74d3e</v>
       </c>
       <c r="B18" t="str">
         <v>2026-07-02</v>
       </c>
       <c r="C18" t="str">
-        <v>Rådgivning</v>
+        <v>indgreb</v>
       </c>
       <c r="D18" t="str">
-        <v>rådgivning</v>
+        <v>indgreb</v>
       </c>
       <c r="E18" t="str">
         <v>substantiv</v>
       </c>
       <c r="F18" t="str">
-        <v>en</v>
+        <v>et</v>
       </c>
       <c r="G18" t="str">
-        <v>-en, -er, -erne</v>
+        <v>-et, -, -ene</v>
       </c>
       <c r="H18" t="str">
-        <v>[ˈʁʌðˌgiwˀneŋ]</v>
+        <v/>
       </c>
       <c r="I18" t="str">
-        <v>https://static.ordnet.dk/mp3/11044/11044289_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11023/11023304_1.mp3</v>
       </c>
       <c r="J18" t="str">
-        <v>det at rådgive</v>
+        <v>handling hvormed man blander sig i noget for at ændre den aktuelle situation</v>
       </c>
       <c r="K18" t="str">
-        <v>counseling</v>
+        <v>intervention</v>
       </c>
       <c r="L18" t="str">
-        <v/>
+        <v>Datacentre jagter sort energi efter politisk indgreb: »Det vil være en katastrofe«</v>
       </c>
       <c r="M18" t="str">
-        <v/>
+        <v>AI-lyskryds fjerner bilkøer på vejene: Men nogle må holde længe for rødt - yihengldavid@gmail.com - Gmail</v>
       </c>
       <c r="N18" t="str">
-        <v/>
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
       </c>
       <c r="O18" t="str">
-        <v/>
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=indgreb</v>
       </c>
       <c r="P18" t="str">
         <v/>
@@ -2129,52 +2291,70 @@
       <c r="AB18" t="str">
         <v/>
       </c>
+      <c r="AC18" t="str">
+        <v/>
+      </c>
+      <c r="AD18" t="str">
+        <v/>
+      </c>
+      <c r="AE18" t="str">
+        <v/>
+      </c>
+      <c r="AF18" t="str">
+        <v/>
+      </c>
+      <c r="AG18" t="str">
+        <v/>
+      </c>
+      <c r="AH18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>71eb02a5-f505-41e4-b9a7-2dd955f74d3e</v>
+        <v>fcee3e04-b744-426b-9a14-215fcad6e55b</v>
       </c>
       <c r="B19" t="str">
         <v>2026-07-02</v>
       </c>
       <c r="C19" t="str">
-        <v>indgreb</v>
+        <v>afslørede</v>
       </c>
       <c r="D19" t="str">
-        <v>indgreb</v>
+        <v>afsløre</v>
       </c>
       <c r="E19" t="str">
-        <v>substantiv</v>
+        <v>verbum</v>
       </c>
       <c r="F19" t="str">
-        <v>et</v>
+        <v/>
       </c>
       <c r="G19" t="str">
-        <v>-et, -, -ene</v>
+        <v>-r, -de, -t</v>
       </c>
       <c r="H19" t="str">
-        <v/>
+        <v>[-ˌsløˀʌ]</v>
       </c>
       <c r="I19" t="str">
-        <v>https://static.ordnet.dk/mp3/11023/11023304_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11000/11000720_1.mp3</v>
       </c>
       <c r="J19" t="str">
-        <v>handling hvormed man blander sig i noget for at ændre den aktuelle situation</v>
+        <v>opdage at nogen har begået en (kriminel eller uhæderlig) handling eller har en egenskab eller fortid som vedkommende har forsøgt at skjule</v>
       </c>
       <c r="K19" t="str">
-        <v>intervention</v>
+        <v>revealed</v>
       </c>
       <c r="L19" t="str">
-        <v>Datacentre jagter sort energi efter politisk indgreb: »Det vil være en katastrofe«</v>
+        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark</v>
       </c>
       <c r="M19" t="str">
-        <v>AI-lyskryds fjerner bilkøer på vejene: Men nogle må holde længe for rødt - yihengldavid@gmail.com - Gmail</v>
+        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark | Ingeniøren</v>
       </c>
       <c r="N19" t="str">
-        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
+        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
       </c>
       <c r="O19" t="str">
-        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=indgreb</v>
+        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=afsl%C3%B8rede</v>
       </c>
       <c r="P19" t="str">
         <v/>
@@ -2215,40 +2395,58 @@
       <c r="AB19" t="str">
         <v/>
       </c>
+      <c r="AC19" t="str">
+        <v/>
+      </c>
+      <c r="AD19" t="str">
+        <v/>
+      </c>
+      <c r="AE19" t="str">
+        <v/>
+      </c>
+      <c r="AF19" t="str">
+        <v/>
+      </c>
+      <c r="AG19" t="str">
+        <v/>
+      </c>
+      <c r="AH19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>fcee3e04-b744-426b-9a14-215fcad6e55b</v>
+        <v>23d95731-816a-467a-a38d-9e6f6a7dced9</v>
       </c>
       <c r="B20" t="str">
         <v>2026-07-02</v>
       </c>
       <c r="C20" t="str">
-        <v>afslørede</v>
+        <v>lovbrud</v>
       </c>
       <c r="D20" t="str">
-        <v>afsløre</v>
+        <v>lovbrud</v>
       </c>
       <c r="E20" t="str">
-        <v>verbum</v>
+        <v>substantiv</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>et</v>
       </c>
       <c r="G20" t="str">
-        <v>-r, -de, -t</v>
+        <v>-det, -, -dene</v>
       </c>
       <c r="H20" t="str">
-        <v>[-ˌsløˀʌ]</v>
+        <v>[-ˌbʁuð]</v>
       </c>
       <c r="I20" t="str">
-        <v>https://static.ordnet.dk/mp3/11000/11000720_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11030/11030992_1.mp3</v>
       </c>
       <c r="J20" t="str">
-        <v>opdage at nogen har begået en (kriminel eller uhæderlig) handling eller har en egenskab eller fortid som vedkommende har forsøgt at skjule</v>
+        <v>det at bryde loven; overtrædelse af loven</v>
       </c>
       <c r="K20" t="str">
-        <v>revealed</v>
+        <v>violation of law</v>
       </c>
       <c r="L20" t="str">
         <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark</v>
@@ -2260,7 +2458,7 @@
         <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
       </c>
       <c r="O20" t="str">
-        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=afsl%C3%B8rede</v>
+        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=lovbrud</v>
       </c>
       <c r="P20" t="str">
         <v/>
@@ -2301,52 +2499,70 @@
       <c r="AB20" t="str">
         <v/>
       </c>
+      <c r="AC20" t="str">
+        <v/>
+      </c>
+      <c r="AD20" t="str">
+        <v/>
+      </c>
+      <c r="AE20" t="str">
+        <v/>
+      </c>
+      <c r="AF20" t="str">
+        <v/>
+      </c>
+      <c r="AG20" t="str">
+        <v/>
+      </c>
+      <c r="AH20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>23d95731-816a-467a-a38d-9e6f6a7dced9</v>
+        <v>039ba62e-8413-430f-ac17-4b365506303e</v>
       </c>
       <c r="B21" t="str">
-        <v>2026-07-02</v>
+        <v>2026-07-22</v>
       </c>
       <c r="C21" t="str">
-        <v>lovbrud</v>
+        <v>overvejer</v>
       </c>
       <c r="D21" t="str">
-        <v>lovbrud</v>
+        <v>overveje</v>
       </c>
       <c r="E21" t="str">
-        <v>substantiv</v>
+        <v>verbum</v>
       </c>
       <c r="F21" t="str">
-        <v>et</v>
+        <v/>
       </c>
       <c r="G21" t="str">
-        <v>-det, -, -dene</v>
+        <v>-r, -de, -t</v>
       </c>
       <c r="H21" t="str">
-        <v>[-ˌbʁuð]</v>
+        <v>[-ˌvɑjˀə]</v>
       </c>
       <c r="I21" t="str">
-        <v>https://static.ordnet.dk/mp3/11030/11030992_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11038/11038552_1.mp3</v>
       </c>
       <c r="J21" t="str">
-        <v>det at bryde loven; overtrædelse af loven</v>
+        <v>tænke over noget eller tænke på at gøre noget idet man vurderer hvad der taler for og imod</v>
       </c>
       <c r="K21" t="str">
-        <v>violation of law</v>
+        <v>reflect</v>
       </c>
       <c r="L21" t="str">
-        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark</v>
+        <v/>
       </c>
       <c r="M21" t="str">
-        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark | Ingeniøren</v>
+        <v/>
       </c>
       <c r="N21" t="str">
-        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
+        <v/>
       </c>
       <c r="O21" t="str">
-        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=lovbrud</v>
+        <v/>
       </c>
       <c r="P21" t="str">
         <v/>
@@ -2387,52 +2603,70 @@
       <c r="AB21" t="str">
         <v/>
       </c>
+      <c r="AC21" t="str">
+        <v/>
+      </c>
+      <c r="AD21" t="str">
+        <v/>
+      </c>
+      <c r="AE21" t="str">
+        <v/>
+      </c>
+      <c r="AF21" t="str">
+        <v/>
+      </c>
+      <c r="AG21" t="str">
+        <v/>
+      </c>
+      <c r="AH21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>039ba62e-8413-430f-ac17-4b365506303e</v>
+        <v>c8b4f170-aa1f-4fe2-a8d4-5be8e34cc7a2</v>
       </c>
       <c r="B22" t="str">
         <v>2026-07-22</v>
       </c>
       <c r="C22" t="str">
-        <v>overvejer</v>
+        <v>Knapt</v>
       </c>
       <c r="D22" t="str">
-        <v>overveje</v>
+        <v>knap</v>
       </c>
       <c r="E22" t="str">
-        <v>verbum</v>
+        <v>adjektiv</v>
       </c>
       <c r="F22" t="str">
         <v/>
       </c>
       <c r="G22" t="str">
-        <v>-r, -de, -t</v>
+        <v>-t, -pe</v>
       </c>
       <c r="H22" t="str">
-        <v>[-ˌvɑjˀə]</v>
+        <v>[ˈknɑb]</v>
       </c>
       <c r="I22" t="str">
-        <v>https://static.ordnet.dk/mp3/11038/11038552_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11026/11026578_1.mp3</v>
       </c>
       <c r="J22" t="str">
-        <v>tænke over noget eller tænke på at gøre noget idet man vurderer hvad der taler for og imod</v>
+        <v>af begrænset eller ringe omfang eller mængde</v>
       </c>
       <c r="K22" t="str">
-        <v>reflect</v>
+        <v>barely</v>
       </c>
       <c r="L22" t="str">
-        <v/>
+        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse</v>
       </c>
       <c r="M22" t="str">
-        <v/>
+        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse | SønderborgNYT</v>
       </c>
       <c r="N22" t="str">
-        <v/>
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA</v>
       </c>
       <c r="O22" t="str">
-        <v/>
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA#:~:text=Knapt</v>
       </c>
       <c r="P22" t="str">
         <v/>
@@ -2494,40 +2728,40 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>c8b4f170-aa1f-4fe2-a8d4-5be8e34cc7a2</v>
+        <v>e370b465-1be4-4af6-9ce3-6dbf2118fc91</v>
       </c>
       <c r="B23" t="str">
         <v>2026-07-22</v>
       </c>
       <c r="C23" t="str">
-        <v>Knapt</v>
+        <v>gennemsnit</v>
       </c>
       <c r="D23" t="str">
-        <v>knap</v>
+        <v>gennemsnit</v>
       </c>
       <c r="E23" t="str">
-        <v>adjektiv</v>
+        <v>substantiv</v>
       </c>
       <c r="F23" t="str">
-        <v/>
+        <v>et</v>
       </c>
       <c r="G23" t="str">
-        <v>-t, -pe</v>
+        <v>-tet, -, -tene</v>
       </c>
       <c r="H23" t="str">
-        <v>[ˈknɑb]</v>
+        <v>[ˈgεnəmˌsnid]</v>
       </c>
       <c r="I23" t="str">
-        <v>https://static.ordnet.dk/mp3/11026/11026578_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11017/11017684_1.mp3</v>
       </c>
       <c r="J23" t="str">
-        <v>af begrænset eller ringe omfang eller mængde</v>
+        <v>værdi der fås ved at dividere en sammenlagt sum med antallet af værdier der indgår i den sammenlagte sum</v>
       </c>
       <c r="K23" t="str">
-        <v>barely</v>
+        <v>average</v>
       </c>
       <c r="L23" t="str">
-        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse</v>
+        <v>375 studenter fra Sønderborg Kommune står uden en uddannelse fem år efter gymnasiet. Det svarer til knap hver tiende eller 9,5 procent. Selv om det er lidt under landsgennemsnittet på 10,3 procent, er andelen steget med to procentpoint siden 2020.</v>
       </c>
       <c r="M23" t="str">
         <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse | SønderborgNYT</v>
@@ -2536,7 +2770,7 @@
         <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA</v>
       </c>
       <c r="O23" t="str">
-        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA#:~:text=Knapt</v>
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA#:~:text=gennemsnit</v>
       </c>
       <c r="P23" t="str">
         <v/>
@@ -2596,113 +2830,9 @@
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>e370b465-1be4-4af6-9ce3-6dbf2118fc91</v>
-      </c>
-      <c r="B24" t="str">
-        <v>2026-07-22</v>
-      </c>
-      <c r="C24" t="str">
-        <v>gennemsnit</v>
-      </c>
-      <c r="D24" t="str">
-        <v>gennemsnit</v>
-      </c>
-      <c r="E24" t="str">
-        <v>substantiv</v>
-      </c>
-      <c r="F24" t="str">
-        <v>et</v>
-      </c>
-      <c r="G24" t="str">
-        <v>-tet, -, -tene</v>
-      </c>
-      <c r="H24" t="str">
-        <v>[ˈgεnəmˌsnid]</v>
-      </c>
-      <c r="I24" t="str">
-        <v>https://static.ordnet.dk/mp3/11017/11017684_1.mp3</v>
-      </c>
-      <c r="J24" t="str">
-        <v>værdi der fås ved at dividere en sammenlagt sum med antallet af værdier der indgår i den sammenlagte sum</v>
-      </c>
-      <c r="K24" t="str">
-        <v>average</v>
-      </c>
-      <c r="L24" t="str">
-        <v>375 studenter fra Sønderborg Kommune står uden en uddannelse fem år efter gymnasiet. Det svarer til knap hver tiende eller 9,5 procent. Selv om det er lidt under landsgennemsnittet på 10,3 procent, er andelen steget med to procentpoint siden 2020.</v>
-      </c>
-      <c r="M24" t="str">
-        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse | SønderborgNYT</v>
-      </c>
-      <c r="N24" t="str">
-        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA</v>
-      </c>
-      <c r="O24" t="str">
-        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA#:~:text=gennemsnit</v>
-      </c>
-      <c r="P24" t="str">
-        <v/>
-      </c>
-      <c r="Q24" t="str">
-        <v>ok</v>
-      </c>
-      <c r="R24" t="str">
-        <v/>
-      </c>
-      <c r="S24" t="str">
-        <v/>
-      </c>
-      <c r="T24" t="str">
-        <v/>
-      </c>
-      <c r="U24" t="str">
-        <v/>
-      </c>
-      <c r="V24" t="str">
-        <v/>
-      </c>
-      <c r="W24" t="str">
-        <v/>
-      </c>
-      <c r="X24" t="str">
-        <v/>
-      </c>
-      <c r="Y24" t="str">
-        <v/>
-      </c>
-      <c r="Z24" t="str">
-        <v/>
-      </c>
-      <c r="AA24" t="str">
-        <v/>
-      </c>
-      <c r="AB24" t="str">
-        <v/>
-      </c>
-      <c r="AC24" t="str">
-        <v/>
-      </c>
-      <c r="AD24" t="str">
-        <v/>
-      </c>
-      <c r="AE24" t="str">
-        <v/>
-      </c>
-      <c r="AF24" t="str">
-        <v/>
-      </c>
-      <c r="AG24" t="str">
-        <v/>
-      </c>
-      <c r="AH24" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2711,34 +2841,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AB4"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="18" max="18" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="18" max="18" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "offentliggjort" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH23"/>
+  <dimension ref="A1:AH24"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2830,9 +2830,113 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>7d3ca2e1-b34b-415c-90c7-5e9eabfa1296</v>
+      </c>
+      <c r="B24" t="str">
+        <v>2026-07-24</v>
+      </c>
+      <c r="C24" t="str">
+        <v>offentliggjort</v>
+      </c>
+      <c r="D24" t="str">
+        <v>offentliggøre</v>
+      </c>
+      <c r="E24" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
+      <c r="G24" t="str">
+        <v>..gør, ..gjorde, ..gjort</v>
+      </c>
+      <c r="H24" t="str">
+        <v>[-ˌgɶˀʌ]</v>
+      </c>
+      <c r="I24" t="str">
+        <v>https://static.ordnet.dk/mp3/11036/11036843_1.mp3</v>
+      </c>
+      <c r="J24" t="str">
+        <v>gøre kendt eller tilgængelig for offentligheden</v>
+      </c>
+      <c r="K24" t="str">
+        <v>publish</v>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
+      <c r="U24" t="str">
+        <v/>
+      </c>
+      <c r="V24" t="str">
+        <v/>
+      </c>
+      <c r="W24" t="str">
+        <v/>
+      </c>
+      <c r="X24" t="str">
+        <v/>
+      </c>
+      <c r="Y24" t="str">
+        <v/>
+      </c>
+      <c r="Z24" t="str">
+        <v/>
+      </c>
+      <c r="AA24" t="str">
+        <v/>
+      </c>
+      <c r="AB24" t="str">
+        <v/>
+      </c>
+      <c r="AC24" t="str">
+        <v/>
+      </c>
+      <c r="AD24" t="str">
+        <v/>
+      </c>
+      <c r="AE24" t="str">
+        <v/>
+      </c>
+      <c r="AF24" t="str">
+        <v/>
+      </c>
+      <c r="AG24" t="str">
+        <v/>
+      </c>
+      <c r="AH24" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH24"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: progress 3, log 6 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -402,40 +402,40 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AH24"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1430,7 +1430,7 @@
         <v/>
       </c>
       <c r="S10" t="str">
-        <v>2026-07-21</v>
+        <v>2026-07-25</v>
       </c>
       <c r="T10" t="str">
         <v>1</v>
@@ -1442,7 +1442,7 @@
         <v>1</v>
       </c>
       <c r="W10" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X10" t="str">
         <v/>
@@ -1460,13 +1460,13 @@
         <v/>
       </c>
       <c r="AC10" t="str">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="AD10" t="str">
-        <v>8.65</v>
+        <v>9.31</v>
       </c>
       <c r="AE10" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-24</v>
       </c>
       <c r="AF10" t="str">
         <v/>
@@ -2054,19 +2054,19 @@
         <v/>
       </c>
       <c r="S16" t="str">
-        <v/>
+        <v>2026-07-24</v>
       </c>
       <c r="T16" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="U16" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V16" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="W16" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X16" t="str">
         <v/>
@@ -2084,13 +2084,13 @@
         <v/>
       </c>
       <c r="AC16" t="str">
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="AD16" t="str">
-        <v/>
+        <v>7.19</v>
       </c>
       <c r="AE16" t="str">
-        <v/>
+        <v>2026-07-24</v>
       </c>
       <c r="AF16" t="str">
         <v/>
@@ -3099,19 +3099,19 @@
         <v/>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
       <c r="N2" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="O2" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="P2" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q2" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="R2" t="str">
         <v/>
@@ -3127,6 +3127,15 @@
       </c>
       <c r="V2" t="str">
         <v/>
+      </c>
+      <c r="W2" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="X2" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>2026-07-24</v>
       </c>
     </row>
     <row r="3">
@@ -3357,7 +3366,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H47"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -4435,9 +4444,165 @@
         <v>1</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>a0876471-cbaf-41fc-a1d7-5d58d6045929</v>
+      </c>
+      <c r="B42" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C42" t="str">
+        <v>2026-07-24T20:19:16.453Z</v>
+      </c>
+      <c r="D42" t="str">
+        <v>again</v>
+      </c>
+      <c r="E42" t="str">
+        <v>0</v>
+      </c>
+      <c r="F42" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G42" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H42" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>0933c06d-fcdc-4401-9d43-79f732aadad7</v>
+      </c>
+      <c r="B43" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C43" t="str">
+        <v>2026-07-24T20:19:30.980Z</v>
+      </c>
+      <c r="D43" t="str">
+        <v>again</v>
+      </c>
+      <c r="E43" t="str">
+        <v>4</v>
+      </c>
+      <c r="F43" t="str">
+        <v>0.14</v>
+      </c>
+      <c r="G43" t="str">
+        <v>9.06</v>
+      </c>
+      <c r="H43" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>a0876471-cbaf-41fc-a1d7-5d58d6045929</v>
+      </c>
+      <c r="B44" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C44" t="str">
+        <v>2026-07-24T20:19:45.805Z</v>
+      </c>
+      <c r="D44" t="str">
+        <v>good</v>
+      </c>
+      <c r="E44" t="str">
+        <v>0</v>
+      </c>
+      <c r="F44" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="G44" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="H44" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>0933c06d-fcdc-4401-9d43-79f732aadad7</v>
+      </c>
+      <c r="B45" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C45" t="str">
+        <v>2026-07-24T20:19:55.387Z</v>
+      </c>
+      <c r="D45" t="str">
+        <v>again</v>
+      </c>
+      <c r="E45" t="str">
+        <v>0</v>
+      </c>
+      <c r="F45" t="str">
+        <v>0.07</v>
+      </c>
+      <c r="G45" t="str">
+        <v>9.34</v>
+      </c>
+      <c r="H45" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>0933c06d-fcdc-4401-9d43-79f732aadad7</v>
+      </c>
+      <c r="B46" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C46" t="str">
+        <v>2026-07-24T20:20:08.435Z</v>
+      </c>
+      <c r="D46" t="str">
+        <v>good</v>
+      </c>
+      <c r="E46" t="str">
+        <v>0</v>
+      </c>
+      <c r="F46" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="G46" t="str">
+        <v>9.31</v>
+      </c>
+      <c r="H46" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>369d0ecd-e56f-4e9b-882e-e7c44c687a79</v>
+      </c>
+      <c r="B47" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C47" t="str">
+        <v>2026-07-24T20:21:00.537Z</v>
+      </c>
+      <c r="D47" t="str">
+        <v>again</v>
+      </c>
+      <c r="E47" t="str">
+        <v>0</v>
+      </c>
+      <c r="F47" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G47" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H47" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H47"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 1, log 3 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -2396,10 +2396,10 @@
         <v/>
       </c>
       <c r="AC19" t="str">
-        <v>0.4</v>
+        <v>0.05</v>
       </c>
       <c r="AD19" t="str">
-        <v>7.19</v>
+        <v>9.08</v>
       </c>
       <c r="AE19" t="str">
         <v>2026-07-24</v>
@@ -3366,7 +3366,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H58"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -4808,9 +4808,87 @@
         <v>0</v>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>fcee3e04-b744-426b-9a14-215fcad6e55b</v>
+      </c>
+      <c r="B56" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C56" t="str">
+        <v>2026-07-24T20:22:14.927Z</v>
+      </c>
+      <c r="D56" t="str">
+        <v>again</v>
+      </c>
+      <c r="E56" t="str">
+        <v>0</v>
+      </c>
+      <c r="F56" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="G56" t="str">
+        <v>8.08</v>
+      </c>
+      <c r="H56" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>fcee3e04-b744-426b-9a14-215fcad6e55b</v>
+      </c>
+      <c r="B57" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C57" t="str">
+        <v>2026-07-24T20:22:29.888Z</v>
+      </c>
+      <c r="D57" t="str">
+        <v>again</v>
+      </c>
+      <c r="E57" t="str">
+        <v>0</v>
+      </c>
+      <c r="F57" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="G57" t="str">
+        <v>8.68</v>
+      </c>
+      <c r="H57" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>fcee3e04-b744-426b-9a14-215fcad6e55b</v>
+      </c>
+      <c r="B58" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C58" t="str">
+        <v>2026-07-24T20:23:19.952Z</v>
+      </c>
+      <c r="D58" t="str">
+        <v>again</v>
+      </c>
+      <c r="E58" t="str">
+        <v>0</v>
+      </c>
+      <c r="F58" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="G58" t="str">
+        <v>9.08</v>
+      </c>
+      <c r="H58" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H58"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 5, log 7 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -702,16 +702,16 @@
         <v/>
       </c>
       <c r="S3" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-26</v>
       </c>
       <c r="T3" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U3" t="str">
         <v>2.5</v>
       </c>
       <c r="V3" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W3" t="str">
         <v>1</v>
@@ -732,10 +732,10 @@
         <v/>
       </c>
       <c r="AC3" t="str">
-        <v>0.56</v>
+        <v>1.32</v>
       </c>
       <c r="AD3" t="str">
-        <v>8.66</v>
+        <v>8.42</v>
       </c>
       <c r="AE3" t="str">
         <v>2026-07-25</v>
@@ -1534,7 +1534,7 @@
         <v/>
       </c>
       <c r="S11" t="str">
-        <v>2026-07-21</v>
+        <v>2026-07-26</v>
       </c>
       <c r="T11" t="str">
         <v>1</v>
@@ -1546,7 +1546,7 @@
         <v>1</v>
       </c>
       <c r="W11" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X11" t="str">
         <v/>
@@ -1564,13 +1564,13 @@
         <v/>
       </c>
       <c r="AC11" t="str">
-        <v>0.28</v>
+        <v>0.39</v>
       </c>
       <c r="AD11" t="str">
-        <v>8.65</v>
+        <v>9.03</v>
       </c>
       <c r="AE11" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-25</v>
       </c>
       <c r="AF11" t="str">
         <v/>
@@ -2574,19 +2574,19 @@
         <v/>
       </c>
       <c r="S21" t="str">
-        <v/>
+        <v>2026-07-26</v>
       </c>
       <c r="T21" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U21" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V21" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W21" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X21" t="str">
         <v/>
@@ -2604,13 +2604,13 @@
         <v/>
       </c>
       <c r="AC21" t="str">
-        <v/>
+        <v>0.56</v>
       </c>
       <c r="AD21" t="str">
-        <v/>
+        <v>7.17</v>
       </c>
       <c r="AE21" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
       <c r="AF21" t="str">
         <v/>
@@ -2678,16 +2678,16 @@
         <v/>
       </c>
       <c r="S22" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-26</v>
       </c>
       <c r="T22" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U22" t="str">
         <v>2.5</v>
       </c>
       <c r="V22" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W22" t="str">
         <v>0</v>
@@ -2711,7 +2711,7 @@
         <v>0.02</v>
       </c>
       <c r="AD22" t="str">
-        <v>9.65</v>
+        <v>9.68</v>
       </c>
       <c r="AE22" t="str">
         <v>2026-07-25</v>
@@ -3176,19 +3176,19 @@
         <v/>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
       <c r="N3" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="O3" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="P3" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q3" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="R3" t="str">
         <v/>
@@ -3206,13 +3206,13 @@
         <v/>
       </c>
       <c r="W3" t="str">
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="X3" t="str">
-        <v/>
+        <v>7.19</v>
       </c>
       <c r="Y3" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
       <c r="Z3" t="str">
         <v/>
@@ -3366,7 +3366,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H95"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -5666,9 +5666,191 @@
         <v>0</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>0d3fc2e5-0c30-4cd1-a873-0cdfc98007a4</v>
+      </c>
+      <c r="B89" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C89" t="str">
+        <v>2026-07-25T06:19:42.645Z</v>
+      </c>
+      <c r="D89" t="str">
+        <v>easy</v>
+      </c>
+      <c r="E89" t="str">
+        <v>0</v>
+      </c>
+      <c r="F89" t="str">
+        <v>1.32</v>
+      </c>
+      <c r="G89" t="str">
+        <v>8.42</v>
+      </c>
+      <c r="H89" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>c8b4f170-aa1f-4fe2-a8d4-5be8e34cc7a2</v>
+      </c>
+      <c r="B90" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C90" t="str">
+        <v>2026-07-25T06:20:19.482Z</v>
+      </c>
+      <c r="D90" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E90" t="str">
+        <v>0</v>
+      </c>
+      <c r="F90" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="G90" t="str">
+        <v>9.68</v>
+      </c>
+      <c r="H90" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
+      </c>
+      <c r="B91" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C91" t="str">
+        <v>2026-07-25T06:20:25.940Z</v>
+      </c>
+      <c r="D91" t="str">
+        <v>again</v>
+      </c>
+      <c r="E91" t="str">
+        <v>5</v>
+      </c>
+      <c r="F91" t="str">
+        <v>0.28</v>
+      </c>
+      <c r="G91" t="str">
+        <v>9.06</v>
+      </c>
+      <c r="H91" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>039ba62e-8413-430f-ac17-4b365506303e</v>
+      </c>
+      <c r="B92" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C92" t="str">
+        <v>2026-07-25T06:20:31.190Z</v>
+      </c>
+      <c r="D92" t="str">
+        <v>again</v>
+      </c>
+      <c r="E92" t="str">
+        <v>0</v>
+      </c>
+      <c r="F92" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G92" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H92" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
+      </c>
+      <c r="B93" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C93" t="str">
+        <v>2026-07-25T06:20:45.689Z</v>
+      </c>
+      <c r="D93" t="str">
+        <v>good</v>
+      </c>
+      <c r="E93" t="str">
+        <v>0</v>
+      </c>
+      <c r="F93" t="str">
+        <v>0.39</v>
+      </c>
+      <c r="G93" t="str">
+        <v>9.03</v>
+      </c>
+      <c r="H93" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>039ba62e-8413-430f-ac17-4b365506303e</v>
+      </c>
+      <c r="B94" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C94" t="str">
+        <v>2026-07-25T06:20:52.188Z</v>
+      </c>
+      <c r="D94" t="str">
+        <v>good</v>
+      </c>
+      <c r="E94" t="str">
+        <v>0</v>
+      </c>
+      <c r="F94" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="G94" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="H94" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>1e5fc340-099b-4123-bd6d-fd6305ee96d7</v>
+      </c>
+      <c r="B95" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C95" t="str">
+        <v>2026-07-25T06:21:01.018Z</v>
+      </c>
+      <c r="D95" t="str">
+        <v>again</v>
+      </c>
+      <c r="E95" t="str">
+        <v>0</v>
+      </c>
+      <c r="F95" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G95" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H95" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H88"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H95"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 4, log 7 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -910,16 +910,16 @@
         <v/>
       </c>
       <c r="S5" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-26</v>
       </c>
       <c r="T5" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U5" t="str">
         <v>2.5</v>
       </c>
       <c r="V5" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W5" t="str">
         <v>1</v>
@@ -940,10 +940,10 @@
         <v/>
       </c>
       <c r="AC5" t="str">
-        <v>0.28</v>
+        <v>0.39</v>
       </c>
       <c r="AD5" t="str">
-        <v>8.67</v>
+        <v>8.64</v>
       </c>
       <c r="AE5" t="str">
         <v>2026-07-25</v>
@@ -1118,7 +1118,7 @@
         <v/>
       </c>
       <c r="S7" t="str">
-        <v>2026-07-21</v>
+        <v>2026-07-26</v>
       </c>
       <c r="T7" t="str">
         <v>1</v>
@@ -1130,7 +1130,7 @@
         <v>1</v>
       </c>
       <c r="W7" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X7" t="str">
         <v/>
@@ -1148,13 +1148,13 @@
         <v/>
       </c>
       <c r="AC7" t="str">
-        <v>0.08</v>
+        <v>0.03</v>
       </c>
       <c r="AD7" t="str">
-        <v>8.87</v>
+        <v>9.5</v>
       </c>
       <c r="AE7" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-25</v>
       </c>
       <c r="AF7" t="str">
         <v/>
@@ -2262,19 +2262,19 @@
         <v/>
       </c>
       <c r="S18" t="str">
-        <v/>
+        <v>2026-07-26</v>
       </c>
       <c r="T18" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="U18" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="V18" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="W18" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="X18" t="str">
         <v/>
@@ -2292,13 +2292,13 @@
         <v/>
       </c>
       <c r="AC18" t="str">
-        <v/>
+        <v>0.56</v>
       </c>
       <c r="AD18" t="str">
-        <v/>
+        <v>7.17</v>
       </c>
       <c r="AE18" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
       <c r="AF18" t="str">
         <v/>
@@ -2470,16 +2470,16 @@
         <v/>
       </c>
       <c r="S20" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-26</v>
       </c>
       <c r="T20" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U20" t="str">
         <v>2.5</v>
       </c>
       <c r="V20" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W20" t="str">
         <v>0</v>
@@ -2500,10 +2500,10 @@
         <v/>
       </c>
       <c r="AC20" t="str">
-        <v>0.4</v>
+        <v>0.56</v>
       </c>
       <c r="AD20" t="str">
-        <v>7.19</v>
+        <v>7.17</v>
       </c>
       <c r="AE20" t="str">
         <v>2026-07-25</v>
@@ -3366,7 +3366,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H116"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -6212,9 +6212,191 @@
         <v>0</v>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>23d95731-816a-467a-a38d-9e6f6a7dced9</v>
+      </c>
+      <c r="B110" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C110" t="str">
+        <v>2026-07-25T06:33:28.928Z</v>
+      </c>
+      <c r="D110" t="str">
+        <v>good</v>
+      </c>
+      <c r="E110" t="str">
+        <v>0</v>
+      </c>
+      <c r="F110" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="G110" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="H110" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>956f08a1-4407-41d9-9dec-b137931c6d72</v>
+      </c>
+      <c r="B111" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C111" t="str">
+        <v>2026-07-25T06:33:34.029Z</v>
+      </c>
+      <c r="D111" t="str">
+        <v>good</v>
+      </c>
+      <c r="E111" t="str">
+        <v>0</v>
+      </c>
+      <c r="F111" t="str">
+        <v>0.39</v>
+      </c>
+      <c r="G111" t="str">
+        <v>8.64</v>
+      </c>
+      <c r="H111" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>8e0306d1-6036-4774-8e44-a607339a1174</v>
+      </c>
+      <c r="B112" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C112" t="str">
+        <v>2026-07-25T06:33:38.315Z</v>
+      </c>
+      <c r="D112" t="str">
+        <v>again</v>
+      </c>
+      <c r="E112" t="str">
+        <v>5</v>
+      </c>
+      <c r="F112" t="str">
+        <v>0.08</v>
+      </c>
+      <c r="G112" t="str">
+        <v>9.21</v>
+      </c>
+      <c r="H112" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>71eb02a5-f505-41e4-b9a7-2dd955f74d3e</v>
+      </c>
+      <c r="B113" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C113" t="str">
+        <v>2026-07-25T06:33:48.303Z</v>
+      </c>
+      <c r="D113" t="str">
+        <v>again</v>
+      </c>
+      <c r="E113" t="str">
+        <v>0</v>
+      </c>
+      <c r="F113" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G113" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H113" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>8e0306d1-6036-4774-8e44-a607339a1174</v>
+      </c>
+      <c r="B114" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C114" t="str">
+        <v>2026-07-25T06:34:14.550Z</v>
+      </c>
+      <c r="D114" t="str">
+        <v>again</v>
+      </c>
+      <c r="E114" t="str">
+        <v>0</v>
+      </c>
+      <c r="F114" t="str">
+        <v>0.04</v>
+      </c>
+      <c r="G114" t="str">
+        <v>9.44</v>
+      </c>
+      <c r="H114" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>71eb02a5-f505-41e4-b9a7-2dd955f74d3e</v>
+      </c>
+      <c r="B115" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C115" t="str">
+        <v>2026-07-25T06:34:18.081Z</v>
+      </c>
+      <c r="D115" t="str">
+        <v>good</v>
+      </c>
+      <c r="E115" t="str">
+        <v>0</v>
+      </c>
+      <c r="F115" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="G115" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="H115" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>8e0306d1-6036-4774-8e44-a607339a1174</v>
+      </c>
+      <c r="B116" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C116" t="str">
+        <v>2026-07-25T06:34:38.161Z</v>
+      </c>
+      <c r="D116" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E116" t="str">
+        <v>0</v>
+      </c>
+      <c r="F116" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="G116" t="str">
+        <v>9.5</v>
+      </c>
+      <c r="H116" t="str">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H109"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H116"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 6, log 10 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -613,19 +613,19 @@
         <v>2</v>
       </c>
       <c r="X2" t="str">
-        <v/>
+        <v>2026-07-26</v>
       </c>
       <c r="Y2" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Z2" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA2" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB2" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC2" t="str">
         <v>0.01</v>
@@ -637,13 +637,13 @@
         <v>2026-07-25</v>
       </c>
       <c r="AF2" t="str">
-        <v/>
+        <v>0.34</v>
       </c>
       <c r="AG2" t="str">
-        <v/>
+        <v>7.63</v>
       </c>
       <c r="AH2" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="3">
@@ -1029,19 +1029,19 @@
         <v>1</v>
       </c>
       <c r="X6" t="str">
-        <v/>
+        <v>2026-07-26</v>
       </c>
       <c r="Y6" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Z6" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA6" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB6" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC6" t="str">
         <v>0.11</v>
@@ -1053,13 +1053,13 @@
         <v>2026-07-25</v>
       </c>
       <c r="AF6" t="str">
-        <v/>
+        <v>0.28</v>
       </c>
       <c r="AG6" t="str">
-        <v/>
+        <v>8.06</v>
       </c>
       <c r="AH6" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="7">
@@ -1133,19 +1133,19 @@
         <v>1</v>
       </c>
       <c r="X7" t="str">
-        <v/>
+        <v>2026-07-26</v>
       </c>
       <c r="Y7" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Z7" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA7" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB7" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC7" t="str">
         <v>0.03</v>
@@ -1157,13 +1157,13 @@
         <v>2026-07-25</v>
       </c>
       <c r="AF7" t="str">
-        <v/>
+        <v>0.34</v>
       </c>
       <c r="AG7" t="str">
-        <v/>
+        <v>7.63</v>
       </c>
       <c r="AH7" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="8">
@@ -1237,19 +1237,19 @@
         <v>0</v>
       </c>
       <c r="X8" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
       <c r="Y8" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="Z8" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA8" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AB8" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC8" t="str">
         <v>8.57</v>
@@ -1261,13 +1261,13 @@
         <v>2026-07-20</v>
       </c>
       <c r="AF8" t="str">
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="AG8" t="str">
-        <v/>
+        <v>7.19</v>
       </c>
       <c r="AH8" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="9">
@@ -1445,19 +1445,19 @@
         <v>2</v>
       </c>
       <c r="X10" t="str">
-        <v/>
+        <v>2026-08-11</v>
       </c>
       <c r="Y10" t="str">
-        <v/>
+        <v>17</v>
       </c>
       <c r="Z10" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA10" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB10" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC10" t="str">
         <v>0.08</v>
@@ -1469,13 +1469,13 @@
         <v>2026-07-25</v>
       </c>
       <c r="AF10" t="str">
-        <v/>
+        <v>15.69</v>
       </c>
       <c r="AG10" t="str">
-        <v/>
+        <v>3.22</v>
       </c>
       <c r="AH10" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="11">
@@ -1549,19 +1549,19 @@
         <v>1</v>
       </c>
       <c r="X11" t="str">
-        <v/>
+        <v>2026-07-28</v>
       </c>
       <c r="Y11" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="Z11" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA11" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB11" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC11" t="str">
         <v>0.39</v>
@@ -1573,13 +1573,13 @@
         <v>2026-07-25</v>
       </c>
       <c r="AF11" t="str">
-        <v/>
+        <v>3.17</v>
       </c>
       <c r="AG11" t="str">
-        <v/>
+        <v>5.28</v>
       </c>
       <c r="AH11" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="12">
@@ -3366,7 +3366,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H122"/>
+  <dimension ref="A1:H132"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -6550,9 +6550,269 @@
         <v>1</v>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>8e0306d1-6036-4774-8e44-a607339a1174</v>
+      </c>
+      <c r="B123" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C123" t="str">
+        <v>2026-07-25T06:38:32.497Z</v>
+      </c>
+      <c r="D123" t="str">
+        <v>again</v>
+      </c>
+      <c r="E123" t="str">
+        <v>0</v>
+      </c>
+      <c r="F123" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G123" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H123" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>6cebe36d-5d01-40b2-906b-8a829745c73d</v>
+      </c>
+      <c r="B124" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C124" t="str">
+        <v>2026-07-25T06:38:46.355Z</v>
+      </c>
+      <c r="D124" t="str">
+        <v>again</v>
+      </c>
+      <c r="E124" t="str">
+        <v>0</v>
+      </c>
+      <c r="F124" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G124" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H124" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B125" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C125" t="str">
+        <v>2026-07-25T06:40:08.132Z</v>
+      </c>
+      <c r="D125" t="str">
+        <v>again</v>
+      </c>
+      <c r="E125" t="str">
+        <v>0</v>
+      </c>
+      <c r="F125" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G125" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H125" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>8e0306d1-6036-4774-8e44-a607339a1174</v>
+      </c>
+      <c r="B126" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C126" t="str">
+        <v>2026-07-25T06:40:18.425Z</v>
+      </c>
+      <c r="D126" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E126" t="str">
+        <v>0</v>
+      </c>
+      <c r="F126" t="str">
+        <v>0.34</v>
+      </c>
+      <c r="G126" t="str">
+        <v>7.63</v>
+      </c>
+      <c r="H126" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>6cebe36d-5d01-40b2-906b-8a829745c73d</v>
+      </c>
+      <c r="B127" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C127" t="str">
+        <v>2026-07-25T06:40:33.932Z</v>
+      </c>
+      <c r="D127" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E127" t="str">
+        <v>0</v>
+      </c>
+      <c r="F127" t="str">
+        <v>0.34</v>
+      </c>
+      <c r="G127" t="str">
+        <v>7.63</v>
+      </c>
+      <c r="H127" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B128" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C128" t="str">
+        <v>2026-07-25T06:40:45.593Z</v>
+      </c>
+      <c r="D128" t="str">
+        <v>again</v>
+      </c>
+      <c r="E128" t="str">
+        <v>0</v>
+      </c>
+      <c r="F128" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="G128" t="str">
+        <v>8.08</v>
+      </c>
+      <c r="H128" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>0933c06d-fcdc-4401-9d43-79f732aadad7</v>
+      </c>
+      <c r="B129" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C129" t="str">
+        <v>2026-07-25T06:41:06.902Z</v>
+      </c>
+      <c r="D129" t="str">
+        <v>easy</v>
+      </c>
+      <c r="E129" t="str">
+        <v>0</v>
+      </c>
+      <c r="F129" t="str">
+        <v>15.69</v>
+      </c>
+      <c r="G129" t="str">
+        <v>3.22</v>
+      </c>
+      <c r="H129" t="str">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>0254c900-1cbd-4360-853b-baf63aadaf10</v>
+      </c>
+      <c r="B130" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C130" t="str">
+        <v>2026-07-25T06:41:30.981Z</v>
+      </c>
+      <c r="D130" t="str">
+        <v>again</v>
+      </c>
+      <c r="E130" t="str">
+        <v>0</v>
+      </c>
+      <c r="F130" t="str">
+        <v>0.4</v>
+      </c>
+      <c r="G130" t="str">
+        <v>7.19</v>
+      </c>
+      <c r="H130" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B131" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C131" t="str">
+        <v>2026-07-25T06:41:36.066Z</v>
+      </c>
+      <c r="D131" t="str">
+        <v>good</v>
+      </c>
+      <c r="E131" t="str">
+        <v>0</v>
+      </c>
+      <c r="F131" t="str">
+        <v>0.28</v>
+      </c>
+      <c r="G131" t="str">
+        <v>8.06</v>
+      </c>
+      <c r="H131" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
+      </c>
+      <c r="B132" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C132" t="str">
+        <v>2026-07-25T06:41:42.587Z</v>
+      </c>
+      <c r="D132" t="str">
+        <v>good</v>
+      </c>
+      <c r="E132" t="str">
+        <v>0</v>
+      </c>
+      <c r="F132" t="str">
+        <v>3.17</v>
+      </c>
+      <c r="G132" t="str">
+        <v>5.28</v>
+      </c>
+      <c r="H132" t="str">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H122"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H132"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 6, log 6 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -402,40 +402,40 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AH24"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -717,19 +717,19 @@
         <v>1</v>
       </c>
       <c r="X3" t="str">
-        <v/>
+        <v>2026-07-26</v>
       </c>
       <c r="Y3" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Z3" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA3" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB3" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC3" t="str">
         <v>1.32</v>
@@ -741,13 +741,13 @@
         <v>2026-07-25</v>
       </c>
       <c r="AF3" t="str">
-        <v/>
+        <v>1.18</v>
       </c>
       <c r="AG3" t="str">
-        <v/>
+        <v>6.49</v>
       </c>
       <c r="AH3" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="4">
@@ -821,19 +821,19 @@
         <v>1</v>
       </c>
       <c r="X4" t="str">
-        <v/>
+        <v>2026-07-26</v>
       </c>
       <c r="Y4" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Z4" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA4" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB4" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC4" t="str">
         <v>0.24</v>
@@ -845,13 +845,13 @@
         <v>2026-07-25</v>
       </c>
       <c r="AF4" t="str">
-        <v/>
+        <v>1.18</v>
       </c>
       <c r="AG4" t="str">
-        <v/>
+        <v>6.49</v>
       </c>
       <c r="AH4" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="5">
@@ -925,19 +925,19 @@
         <v>1</v>
       </c>
       <c r="X5" t="str">
-        <v/>
+        <v>2026-07-26</v>
       </c>
       <c r="Y5" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Z5" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA5" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB5" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC5" t="str">
         <v>0.39</v>
@@ -949,13 +949,13 @@
         <v>2026-07-25</v>
       </c>
       <c r="AF5" t="str">
-        <v/>
+        <v>1.18</v>
       </c>
       <c r="AG5" t="str">
-        <v/>
+        <v>6.49</v>
       </c>
       <c r="AH5" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="6">
@@ -1237,16 +1237,16 @@
         <v>0</v>
       </c>
       <c r="X8" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-26</v>
       </c>
       <c r="Y8" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z8" t="str">
         <v>2.5</v>
       </c>
       <c r="AA8" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB8" t="str">
         <v>0</v>
@@ -1261,10 +1261,10 @@
         <v>2026-07-20</v>
       </c>
       <c r="AF8" t="str">
-        <v>0.4</v>
+        <v>0.56</v>
       </c>
       <c r="AG8" t="str">
-        <v>7.19</v>
+        <v>7.17</v>
       </c>
       <c r="AH8" t="str">
         <v>2026-07-25</v>
@@ -1341,19 +1341,19 @@
         <v>2</v>
       </c>
       <c r="X9" t="str">
-        <v/>
+        <v>2026-07-26</v>
       </c>
       <c r="Y9" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Z9" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA9" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB9" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC9" t="str">
         <v>0.53</v>
@@ -1365,13 +1365,13 @@
         <v>2026-07-25</v>
       </c>
       <c r="AF9" t="str">
-        <v/>
+        <v>1.18</v>
       </c>
       <c r="AG9" t="str">
-        <v/>
+        <v>6.49</v>
       </c>
       <c r="AH9" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="10">
@@ -1965,19 +1965,19 @@
         <v>0</v>
       </c>
       <c r="X15" t="str">
-        <v/>
+        <v>2026-07-26</v>
       </c>
       <c r="Y15" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Z15" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA15" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB15" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC15" t="str">
         <v>6.54</v>
@@ -1989,13 +1989,13 @@
         <v>2026-07-25</v>
       </c>
       <c r="AF15" t="str">
-        <v/>
+        <v>1.18</v>
       </c>
       <c r="AG15" t="str">
-        <v/>
+        <v>6.49</v>
       </c>
       <c r="AH15" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="16">
@@ -3368,7 +3368,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H132"/>
+  <dimension ref="A1:H138"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -6812,10 +6812,166 @@
         <v>3</v>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>0254c900-1cbd-4360-853b-baf63aadaf10</v>
+      </c>
+      <c r="B133" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C133" t="str">
+        <v>2026-07-25T06:41:48.512Z</v>
+      </c>
+      <c r="D133" t="str">
+        <v>good</v>
+      </c>
+      <c r="E133" t="str">
+        <v>0</v>
+      </c>
+      <c r="F133" t="str">
+        <v>0.56</v>
+      </c>
+      <c r="G133" t="str">
+        <v>7.17</v>
+      </c>
+      <c r="H133" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>0d3fc2e5-0c30-4cd1-a873-0cdfc98007a4</v>
+      </c>
+      <c r="B134" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C134" t="str">
+        <v>2026-07-25T06:41:59.483Z</v>
+      </c>
+      <c r="D134" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E134" t="str">
+        <v>0</v>
+      </c>
+      <c r="F134" t="str">
+        <v>1.18</v>
+      </c>
+      <c r="G134" t="str">
+        <v>6.49</v>
+      </c>
+      <c r="H134" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>956f08a1-4407-41d9-9dec-b137931c6d72</v>
+      </c>
+      <c r="B135" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C135" t="str">
+        <v>2026-07-25T06:42:13.968Z</v>
+      </c>
+      <c r="D135" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E135" t="str">
+        <v>0</v>
+      </c>
+      <c r="F135" t="str">
+        <v>1.18</v>
+      </c>
+      <c r="G135" t="str">
+        <v>6.49</v>
+      </c>
+      <c r="H135" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>8732aac0-4d2b-43cc-9af1-60bf3151752b</v>
+      </c>
+      <c r="B136" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C136" t="str">
+        <v>2026-07-25T06:42:18.613Z</v>
+      </c>
+      <c r="D136" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E136" t="str">
+        <v>0</v>
+      </c>
+      <c r="F136" t="str">
+        <v>1.18</v>
+      </c>
+      <c r="G136" t="str">
+        <v>6.49</v>
+      </c>
+      <c r="H136" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>05d5014c-1bc9-48f5-ac80-9c6659843c67</v>
+      </c>
+      <c r="B137" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C137" t="str">
+        <v>2026-07-25T06:42:54.275Z</v>
+      </c>
+      <c r="D137" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E137" t="str">
+        <v>0</v>
+      </c>
+      <c r="F137" t="str">
+        <v>1.18</v>
+      </c>
+      <c r="G137" t="str">
+        <v>6.49</v>
+      </c>
+      <c r="H137" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>6d8e9813-5550-45ab-9874-78033b6c2cd6</v>
+      </c>
+      <c r="B138" t="str">
+        <v>en2da</v>
+      </c>
+      <c r="C138" t="str">
+        <v>2026-07-25T06:43:55.756Z</v>
+      </c>
+      <c r="D138" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E138" t="str">
+        <v>0</v>
+      </c>
+      <c r="F138" t="str">
+        <v>1.18</v>
+      </c>
+      <c r="G138" t="str">
+        <v>6.49</v>
+      </c>
+      <c r="H138" t="str">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H132"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H138"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add word "forurenet" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -400,42 +400,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH24"/>
+  <dimension ref="A1:AH25"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2934,9 +2934,113 @@
         <v/>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>4261b3bc-9498-4eb7-95f2-89d64a918f1e</v>
+      </c>
+      <c r="B25" t="str">
+        <v>2026-07-27</v>
+      </c>
+      <c r="C25" t="str">
+        <v>forurenet</v>
+      </c>
+      <c r="D25" t="str">
+        <v>forurene</v>
+      </c>
+      <c r="E25" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
+      <c r="G25" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H25" t="str">
+        <v>[fɒuˈʁεˀnə]</v>
+      </c>
+      <c r="I25" t="str">
+        <v>https://static.ordnet.dk/mp3/11015/11015475_1.mp3</v>
+      </c>
+      <c r="J25" t="str">
+        <v>ødelægge naturen ved udledning af skadelige stoffer</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Contaminated</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Et menneskeskabt kemikalie, der har forurenet store dele af det danske grundvand og drikkevand, er farligere end antaget.</v>
+      </c>
+      <c r="M25" t="str">
+        <v>Det er utroligt lille og findes i vores drikkevand: Nu viser det sig at være farligt for mennesker | Ingeniøren</v>
+      </c>
+      <c r="N25" t="str">
+        <v>https://ing.dk/artikel/det-er-utroligt-lille-og-findes-i-vores-drikkevand-nu-viser-det-sig-vaere-farligt-mennesker</v>
+      </c>
+      <c r="O25" t="str">
+        <v>https://ing.dk/artikel/det-er-utroligt-lille-og-findes-i-vores-drikkevand-nu-viser-det-sig-vaere-farligt-mennesker#:~:text=forurenet</v>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R25" t="str">
+        <v/>
+      </c>
+      <c r="S25" t="str">
+        <v/>
+      </c>
+      <c r="T25" t="str">
+        <v/>
+      </c>
+      <c r="U25" t="str">
+        <v/>
+      </c>
+      <c r="V25" t="str">
+        <v/>
+      </c>
+      <c r="W25" t="str">
+        <v/>
+      </c>
+      <c r="X25" t="str">
+        <v/>
+      </c>
+      <c r="Y25" t="str">
+        <v/>
+      </c>
+      <c r="Z25" t="str">
+        <v/>
+      </c>
+      <c r="AA25" t="str">
+        <v/>
+      </c>
+      <c r="AB25" t="str">
+        <v/>
+      </c>
+      <c r="AC25" t="str">
+        <v/>
+      </c>
+      <c r="AD25" t="str">
+        <v/>
+      </c>
+      <c r="AE25" t="str">
+        <v/>
+      </c>
+      <c r="AF25" t="str">
+        <v/>
+      </c>
+      <c r="AG25" t="str">
+        <v/>
+      </c>
+      <c r="AH25" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: progress 5, log 6 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -1328,19 +1328,19 @@
         <v/>
       </c>
       <c r="S11" t="str">
-        <v>2026-07-26</v>
+        <v>2026-07-27</v>
       </c>
       <c r="T11" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U11" t="str">
         <v>2.5</v>
       </c>
       <c r="V11" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W11" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X11" t="str">
         <v>2026-07-28</v>
@@ -1358,13 +1358,13 @@
         <v>0</v>
       </c>
       <c r="AC11" t="str">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="AD11" t="str">
-        <v>9.03</v>
+        <v>9.32</v>
       </c>
       <c r="AE11" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-27</v>
       </c>
       <c r="AF11" t="str">
         <v>3.17</v>
@@ -1952,16 +1952,16 @@
         <v/>
       </c>
       <c r="S17" t="str">
-        <v>2026-07-26</v>
+        <v>2026-07-31</v>
       </c>
       <c r="T17" t="str">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U17" t="str">
         <v>2.5</v>
       </c>
       <c r="V17" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W17" t="str">
         <v>0</v>
@@ -1982,13 +1982,13 @@
         <v>0</v>
       </c>
       <c r="AC17" t="str">
-        <v>0.56</v>
+        <v>3.88</v>
       </c>
       <c r="AD17" t="str">
-        <v>7.17</v>
+        <v>7.15</v>
       </c>
       <c r="AE17" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-27</v>
       </c>
       <c r="AF17" t="str">
         <v>0.4</v>
@@ -2056,7 +2056,7 @@
         <v/>
       </c>
       <c r="S18" t="str">
-        <v>2026-07-26</v>
+        <v>2026-07-28</v>
       </c>
       <c r="T18" t="str">
         <v>1</v>
@@ -2068,7 +2068,7 @@
         <v>1</v>
       </c>
       <c r="W18" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X18" t="str">
         <v/>
@@ -2086,13 +2086,13 @@
         <v/>
       </c>
       <c r="AC18" t="str">
-        <v>0.56</v>
+        <v>0.55</v>
       </c>
       <c r="AD18" t="str">
-        <v>7.17</v>
+        <v>8.05</v>
       </c>
       <c r="AE18" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-27</v>
       </c>
       <c r="AF18" t="str">
         <v/>
@@ -2368,19 +2368,19 @@
         <v/>
       </c>
       <c r="S21" t="str">
-        <v>2026-07-26</v>
+        <v>2026-07-27</v>
       </c>
       <c r="T21" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U21" t="str">
         <v>2.5</v>
       </c>
       <c r="V21" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W21" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X21" t="str">
         <v/>
@@ -2401,10 +2401,10 @@
         <v>0.02</v>
       </c>
       <c r="AD21" t="str">
-        <v>9.68</v>
+        <v>9.75</v>
       </c>
       <c r="AE21" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-27</v>
       </c>
       <c r="AF21" t="str">
         <v/>
@@ -2970,16 +2970,16 @@
         <v/>
       </c>
       <c r="M3" t="str">
-        <v>2026-07-26</v>
+        <v>2026-07-31</v>
       </c>
       <c r="N3" t="str">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O3" t="str">
         <v>2.5</v>
       </c>
       <c r="P3" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q3" t="str">
         <v>0</v>
@@ -3000,13 +3000,13 @@
         <v/>
       </c>
       <c r="W3" t="str">
-        <v>0.56</v>
+        <v>3.88</v>
       </c>
       <c r="X3" t="str">
-        <v>7.17</v>
+        <v>7.15</v>
       </c>
       <c r="Y3" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-27</v>
       </c>
       <c r="Z3" t="str">
         <v/>
@@ -3162,7 +3162,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H140"/>
+  <dimension ref="A1:H146"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -6814,10 +6814,166 @@
         <v>0</v>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>1e5fc340-099b-4123-bd6d-fd6305ee96d7</v>
+      </c>
+      <c r="B141" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C141" t="str">
+        <v>2026-07-27T19:28:55.945Z</v>
+      </c>
+      <c r="D141" t="str">
+        <v>good</v>
+      </c>
+      <c r="E141" t="str">
+        <v>2</v>
+      </c>
+      <c r="F141" t="str">
+        <v>3.88</v>
+      </c>
+      <c r="G141" t="str">
+        <v>7.15</v>
+      </c>
+      <c r="H141" t="str">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>71eb02a5-f505-41e4-b9a7-2dd955f74d3e</v>
+      </c>
+      <c r="B142" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C142" t="str">
+        <v>2026-07-27T19:29:05.544Z</v>
+      </c>
+      <c r="D142" t="str">
+        <v>again</v>
+      </c>
+      <c r="E142" t="str">
+        <v>2</v>
+      </c>
+      <c r="F142" t="str">
+        <v>0.39</v>
+      </c>
+      <c r="G142" t="str">
+        <v>8.07</v>
+      </c>
+      <c r="H142" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>94801dbf-f81c-46cc-a320-3e40b0903e79</v>
+      </c>
+      <c r="B143" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C143" t="str">
+        <v>2026-07-27T19:29:09.296Z</v>
+      </c>
+      <c r="D143" t="str">
+        <v>good</v>
+      </c>
+      <c r="E143" t="str">
+        <v>2</v>
+      </c>
+      <c r="F143" t="str">
+        <v>3.88</v>
+      </c>
+      <c r="G143" t="str">
+        <v>7.15</v>
+      </c>
+      <c r="H143" t="str">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>71eb02a5-f505-41e4-b9a7-2dd955f74d3e</v>
+      </c>
+      <c r="B144" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C144" t="str">
+        <v>2026-07-27T19:29:16.951Z</v>
+      </c>
+      <c r="D144" t="str">
+        <v>good</v>
+      </c>
+      <c r="E144" t="str">
+        <v>0</v>
+      </c>
+      <c r="F144" t="str">
+        <v>0.55</v>
+      </c>
+      <c r="G144" t="str">
+        <v>8.05</v>
+      </c>
+      <c r="H144" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>c8b4f170-aa1f-4fe2-a8d4-5be8e34cc7a2</v>
+      </c>
+      <c r="B145" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C145" t="str">
+        <v>2026-07-27T19:29:29.419Z</v>
+      </c>
+      <c r="D145" t="str">
+        <v>again</v>
+      </c>
+      <c r="E145" t="str">
+        <v>2</v>
+      </c>
+      <c r="F145" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="G145" t="str">
+        <v>9.75</v>
+      </c>
+      <c r="H145" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
+      </c>
+      <c r="B146" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C146" t="str">
+        <v>2026-07-27T19:29:34.032Z</v>
+      </c>
+      <c r="D146" t="str">
+        <v>again</v>
+      </c>
+      <c r="E146" t="str">
+        <v>2</v>
+      </c>
+      <c r="F146" t="str">
+        <v>0.33</v>
+      </c>
+      <c r="G146" t="str">
+        <v>9.32</v>
+      </c>
+      <c r="H146" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H140"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H146"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 3, log 3 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -496,19 +496,19 @@
         <v/>
       </c>
       <c r="S3" t="str">
-        <v>2026-07-26</v>
+        <v>2026-07-27</v>
       </c>
       <c r="T3" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U3" t="str">
         <v>2.5</v>
       </c>
       <c r="V3" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W3" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X3" t="str">
         <v>2026-07-26</v>
@@ -526,13 +526,13 @@
         <v>0</v>
       </c>
       <c r="AC3" t="str">
-        <v>1.32</v>
+        <v>0.59</v>
       </c>
       <c r="AD3" t="str">
-        <v>8.42</v>
+        <v>8.91</v>
       </c>
       <c r="AE3" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-27</v>
       </c>
       <c r="AF3" t="str">
         <v>1.18</v>
@@ -1328,16 +1328,16 @@
         <v/>
       </c>
       <c r="S11" t="str">
-        <v>2026-07-27</v>
+        <v>2026-07-28</v>
       </c>
       <c r="T11" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U11" t="str">
         <v>2.5</v>
       </c>
       <c r="V11" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W11" t="str">
         <v>2</v>
@@ -1358,10 +1358,10 @@
         <v>0</v>
       </c>
       <c r="AC11" t="str">
-        <v>0.33</v>
+        <v>0.46</v>
       </c>
       <c r="AD11" t="str">
-        <v>9.32</v>
+        <v>9.29</v>
       </c>
       <c r="AE11" t="str">
         <v>2026-07-27</v>
@@ -2368,16 +2368,16 @@
         <v/>
       </c>
       <c r="S21" t="str">
-        <v>2026-07-27</v>
+        <v>2026-07-28</v>
       </c>
       <c r="T21" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U21" t="str">
         <v>2.5</v>
       </c>
       <c r="V21" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W21" t="str">
         <v>1</v>
@@ -2401,7 +2401,7 @@
         <v>0.02</v>
       </c>
       <c r="AD21" t="str">
-        <v>9.75</v>
+        <v>9.76</v>
       </c>
       <c r="AE21" t="str">
         <v>2026-07-27</v>
@@ -3162,7 +3162,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H146"/>
+  <dimension ref="A1:H149"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -6970,10 +6970,88 @@
         <v>0</v>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>c8b4f170-aa1f-4fe2-a8d4-5be8e34cc7a2</v>
+      </c>
+      <c r="B147" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C147" t="str">
+        <v>2026-07-27T19:31:33.590Z</v>
+      </c>
+      <c r="D147" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E147" t="str">
+        <v>0</v>
+      </c>
+      <c r="F147" t="str">
+        <v>0.02</v>
+      </c>
+      <c r="G147" t="str">
+        <v>9.76</v>
+      </c>
+      <c r="H147" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
+      </c>
+      <c r="B148" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C148" t="str">
+        <v>2026-07-27T19:31:36.298Z</v>
+      </c>
+      <c r="D148" t="str">
+        <v>good</v>
+      </c>
+      <c r="E148" t="str">
+        <v>0</v>
+      </c>
+      <c r="F148" t="str">
+        <v>0.46</v>
+      </c>
+      <c r="G148" t="str">
+        <v>9.29</v>
+      </c>
+      <c r="H148" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>0d3fc2e5-0c30-4cd1-a873-0cdfc98007a4</v>
+      </c>
+      <c r="B149" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C149" t="str">
+        <v>2026-07-27T19:32:14.471Z</v>
+      </c>
+      <c r="D149" t="str">
+        <v>again</v>
+      </c>
+      <c r="E149" t="str">
+        <v>2</v>
+      </c>
+      <c r="F149" t="str">
+        <v>0.59</v>
+      </c>
+      <c r="G149" t="str">
+        <v>8.91</v>
+      </c>
+      <c r="H149" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H146"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H149"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 6, log 11 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -704,16 +704,16 @@
         <v/>
       </c>
       <c r="S5" t="str">
-        <v>2026-07-27</v>
+        <v>2026-07-28</v>
       </c>
       <c r="T5" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U5" t="str">
         <v>2.5</v>
       </c>
       <c r="V5" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W5" t="str">
         <v>2</v>
@@ -734,10 +734,10 @@
         <v>0</v>
       </c>
       <c r="AC5" t="str">
-        <v>0.11</v>
+        <v>0.03</v>
       </c>
       <c r="AD5" t="str">
-        <v>9.57</v>
+        <v>9.76</v>
       </c>
       <c r="AE5" t="str">
         <v>2026-07-27</v>
@@ -1774,10 +1774,10 @@
         <v/>
       </c>
       <c r="AC15" t="str">
-        <v>0.19</v>
+        <v>0.1</v>
       </c>
       <c r="AD15" t="str">
-        <v>9.04</v>
+        <v>9.32</v>
       </c>
       <c r="AE15" t="str">
         <v>2026-07-27</v>
@@ -3058,7 +3058,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H174"/>
+  <dimension ref="A1:H185"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -7594,10 +7594,296 @@
         <v>0</v>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>7bea74c7-5aab-4f05-909c-e9bdd96906fb</v>
+      </c>
+      <c r="B175" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C175" t="str">
+        <v>2026-07-27T19:40:43.252Z</v>
+      </c>
+      <c r="D175" t="str">
+        <v>again</v>
+      </c>
+      <c r="E175" t="str">
+        <v>2</v>
+      </c>
+      <c r="F175" t="str">
+        <v>0.07</v>
+      </c>
+      <c r="G175" t="str">
+        <v>9.33</v>
+      </c>
+      <c r="H175" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v>7bea74c7-5aab-4f05-909c-e9bdd96906fb</v>
+      </c>
+      <c r="B176" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C176" t="str">
+        <v>2026-07-27T19:41:01.153Z</v>
+      </c>
+      <c r="D176" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E176" t="str">
+        <v>0</v>
+      </c>
+      <c r="F176" t="str">
+        <v>0.06</v>
+      </c>
+      <c r="G176" t="str">
+        <v>9.41</v>
+      </c>
+      <c r="H176" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>a0876471-cbaf-41fc-a1d7-5d58d6045929</v>
+      </c>
+      <c r="B177" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C177" t="str">
+        <v>2026-07-27T19:41:07.189Z</v>
+      </c>
+      <c r="D177" t="str">
+        <v>again</v>
+      </c>
+      <c r="E177" t="str">
+        <v>2</v>
+      </c>
+      <c r="F177" t="str">
+        <v>0.51</v>
+      </c>
+      <c r="G177" t="str">
+        <v>8.36</v>
+      </c>
+      <c r="H177" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>23d95731-816a-467a-a38d-9e6f6a7dced9</v>
+      </c>
+      <c r="B178" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C178" t="str">
+        <v>2026-07-27T19:41:13.634Z</v>
+      </c>
+      <c r="D178" t="str">
+        <v>good</v>
+      </c>
+      <c r="E178" t="str">
+        <v>2</v>
+      </c>
+      <c r="F178" t="str">
+        <v>3.88</v>
+      </c>
+      <c r="G178" t="str">
+        <v>7.15</v>
+      </c>
+      <c r="H178" t="str">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>8732aac0-4d2b-43cc-9af1-60bf3151752b</v>
+      </c>
+      <c r="B179" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C179" t="str">
+        <v>2026-07-27T19:41:16.532Z</v>
+      </c>
+      <c r="D179" t="str">
+        <v>good</v>
+      </c>
+      <c r="E179" t="str">
+        <v>2</v>
+      </c>
+      <c r="F179" t="str">
+        <v>1.94</v>
+      </c>
+      <c r="G179" t="str">
+        <v>9.35</v>
+      </c>
+      <c r="H179" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>a0876471-cbaf-41fc-a1d7-5d58d6045929</v>
+      </c>
+      <c r="B180" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C180" t="str">
+        <v>2026-07-27T19:41:19.531Z</v>
+      </c>
+      <c r="D180" t="str">
+        <v>good</v>
+      </c>
+      <c r="E180" t="str">
+        <v>0</v>
+      </c>
+      <c r="F180" t="str">
+        <v>0.72</v>
+      </c>
+      <c r="G180" t="str">
+        <v>8.34</v>
+      </c>
+      <c r="H180" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B181" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C181" t="str">
+        <v>2026-07-27T19:41:23.563Z</v>
+      </c>
+      <c r="D181" t="str">
+        <v>again</v>
+      </c>
+      <c r="E181" t="str">
+        <v>2</v>
+      </c>
+      <c r="F181" t="str">
+        <v>0.11</v>
+      </c>
+      <c r="G181" t="str">
+        <v>9.57</v>
+      </c>
+      <c r="H181" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B182" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C182" t="str">
+        <v>2026-07-27T19:41:45.289Z</v>
+      </c>
+      <c r="D182" t="str">
+        <v>again</v>
+      </c>
+      <c r="E182" t="str">
+        <v>0</v>
+      </c>
+      <c r="F182" t="str">
+        <v>0.06</v>
+      </c>
+      <c r="G182" t="str">
+        <v>9.68</v>
+      </c>
+      <c r="H182" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B183" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C183" t="str">
+        <v>2026-07-27T19:42:36.434Z</v>
+      </c>
+      <c r="D183" t="str">
+        <v>again</v>
+      </c>
+      <c r="E183" t="str">
+        <v>0</v>
+      </c>
+      <c r="F183" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="G183" t="str">
+        <v>9.75</v>
+      </c>
+      <c r="H183" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>369d0ecd-e56f-4e9b-882e-e7c44c687a79</v>
+      </c>
+      <c r="B184" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C184" t="str">
+        <v>2026-07-27T19:43:02.820Z</v>
+      </c>
+      <c r="D184" t="str">
+        <v>again</v>
+      </c>
+      <c r="E184" t="str">
+        <v>0</v>
+      </c>
+      <c r="F184" t="str">
+        <v>0.1</v>
+      </c>
+      <c r="G184" t="str">
+        <v>9.32</v>
+      </c>
+      <c r="H184" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>741aaa0a-0d8b-4d04-ba7f-9f88ddb41f54</v>
+      </c>
+      <c r="B185" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C185" t="str">
+        <v>2026-07-27T19:43:11.867Z</v>
+      </c>
+      <c r="D185" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E185" t="str">
+        <v>0</v>
+      </c>
+      <c r="F185" t="str">
+        <v>0.03</v>
+      </c>
+      <c r="G185" t="str">
+        <v>9.76</v>
+      </c>
+      <c r="H185" t="str">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H174"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H185"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: delete 1, progress 1, log 1 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH23"/>
+  <dimension ref="A1:AH22"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="10.83203125"/>
     <col min="2" max="2" customWidth="1" width="11.83203125"/>
@@ -1066,16 +1066,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>0933c06d-fcdc-4401-9d43-79f732aadad7</v>
+        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
       </c>
       <c r="B9" t="str">
         <v>2026-07-01</v>
       </c>
       <c r="C9" t="str">
-        <v>miljøredegørelse</v>
+        <v>ANSØGNING</v>
       </c>
       <c r="D9" t="str">
-        <v>miljøredegørelse</v>
+        <v>ansøgning</v>
       </c>
       <c r="E9" t="str">
         <v>substantiv</v>
@@ -1084,19 +1084,19 @@
         <v>en</v>
       </c>
       <c r="G9" t="str">
-        <v>-n, -r, -rne</v>
+        <v>-en, -er, -erne</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>[ˈanˌsøjˀneŋ]</v>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v>https://static.ordnet.dk/mp3/11002/11002018_1.mp3</v>
       </c>
       <c r="J9" t="str">
-        <v>sammensat af miljø + redegørelse</v>
+        <v>det at ansøge om noget</v>
       </c>
       <c r="K9" t="str">
-        <v>Environmental statement</v>
+        <v>Application</v>
       </c>
       <c r="L9" t="str">
         <v/>
@@ -1120,7 +1120,7 @@
         <v/>
       </c>
       <c r="S9" t="str">
-        <v>2026-07-26</v>
+        <v>2026-07-28</v>
       </c>
       <c r="T9" t="str">
         <v>1</v>
@@ -1135,10 +1135,10 @@
         <v>2</v>
       </c>
       <c r="X9" t="str">
-        <v>2026-08-11</v>
+        <v>2026-07-28</v>
       </c>
       <c r="Y9" t="str">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="Z9" t="str">
         <v>2.5</v>
@@ -1150,19 +1150,19 @@
         <v>0</v>
       </c>
       <c r="AC9" t="str">
-        <v>0.08</v>
+        <v>0.46</v>
       </c>
       <c r="AD9" t="str">
-        <v>9.55</v>
+        <v>9.29</v>
       </c>
       <c r="AE9" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-27</v>
       </c>
       <c r="AF9" t="str">
-        <v>15.69</v>
+        <v>3.17</v>
       </c>
       <c r="AG9" t="str">
-        <v>3.22</v>
+        <v>5.28</v>
       </c>
       <c r="AH9" t="str">
         <v>2026-07-25</v>
@@ -1170,16 +1170,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>8ebac409-093d-442a-9b03-6866d8b59a8a</v>
+        <v>87f910eb-6aa4-4751-ad3a-14ec49047ac6</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-07-01</v>
+        <v>2026-07-02</v>
       </c>
       <c r="C10" t="str">
-        <v>ANSØGNING</v>
+        <v>bryder</v>
       </c>
       <c r="D10" t="str">
-        <v>ansøgning</v>
+        <v>bryder</v>
       </c>
       <c r="E10" t="str">
         <v>substantiv</v>
@@ -1188,31 +1188,31 @@
         <v>en</v>
       </c>
       <c r="G10" t="str">
-        <v>-en, -er, -erne</v>
+        <v>-en, -e, -ne</v>
       </c>
       <c r="H10" t="str">
-        <v>[ˈanˌsøjˀneŋ]</v>
+        <v>[ˈbʁyːðʌ]</v>
       </c>
       <c r="I10" t="str">
-        <v>https://static.ordnet.dk/mp3/11002/11002018_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11006/11006414_1.mp3</v>
       </c>
       <c r="J10" t="str">
-        <v>det at ansøge om noget</v>
+        <v>person der udøver sportsgrenen brydning</v>
       </c>
       <c r="K10" t="str">
-        <v>Application</v>
+        <v>breaks</v>
       </c>
       <c r="L10" t="str">
-        <v/>
+        <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb</v>
       </c>
       <c r="M10" t="str">
-        <v>miljoegodkendelse_-_gaeldende_270917_dok_121943-17_v1_0.pdf</v>
+        <v>Ingeniøren - nyheder om teknologi og samfund</v>
       </c>
       <c r="N10" t="str">
-        <v/>
+        <v>https://ing.dk/</v>
       </c>
       <c r="O10" t="str">
-        <v/>
+        <v>https://ing.dk/#:~:text=bryder</v>
       </c>
       <c r="P10" t="str">
         <v/>
@@ -1224,87 +1224,87 @@
         <v/>
       </c>
       <c r="S10" t="str">
-        <v>2026-07-28</v>
+        <v>2026-08-09</v>
       </c>
       <c r="T10" t="str">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="U10" t="str">
         <v>2.5</v>
       </c>
       <c r="V10" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W10" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X10" t="str">
-        <v>2026-07-28</v>
+        <v/>
       </c>
       <c r="Y10" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="Z10" t="str">
-        <v>2.5</v>
+        <v/>
       </c>
       <c r="AA10" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="AB10" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AC10" t="str">
-        <v>0.46</v>
+        <v>15.05</v>
       </c>
       <c r="AD10" t="str">
-        <v>9.29</v>
+        <v>5.27</v>
       </c>
       <c r="AE10" t="str">
-        <v>2026-07-27</v>
+        <v>2026-07-25</v>
       </c>
       <c r="AF10" t="str">
-        <v>3.17</v>
+        <v/>
       </c>
       <c r="AG10" t="str">
-        <v>5.28</v>
+        <v/>
       </c>
       <c r="AH10" t="str">
-        <v>2026-07-25</v>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>87f910eb-6aa4-4751-ad3a-14ec49047ac6</v>
+        <v>c2d45936-5793-42b4-968a-e066bcb27036</v>
       </c>
       <c r="B11" t="str">
         <v>2026-07-02</v>
       </c>
       <c r="C11" t="str">
-        <v>bryder</v>
+        <v>Pløjer</v>
       </c>
       <c r="D11" t="str">
-        <v>bryder</v>
+        <v>pløje</v>
       </c>
       <c r="E11" t="str">
-        <v>substantiv</v>
+        <v>verbum</v>
       </c>
       <c r="F11" t="str">
-        <v>en</v>
+        <v/>
       </c>
       <c r="G11" t="str">
-        <v>-en, -e, -ne</v>
+        <v>-r, -de, -t</v>
       </c>
       <c r="H11" t="str">
-        <v>[ˈbʁyːðʌ]</v>
+        <v>[ˈplʌjə]</v>
       </c>
       <c r="I11" t="str">
-        <v>https://static.ordnet.dk/mp3/11006/11006414_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11040/11040224_1.mp3</v>
       </c>
       <c r="J11" t="str">
-        <v>person der udøver sportsgrenen brydning</v>
+        <v>vende det øverste jordlag med en plov inden man sår eller planter afgrøder</v>
       </c>
       <c r="K11" t="str">
-        <v>breaks</v>
+        <v>Plows</v>
       </c>
       <c r="L11" t="str">
         <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb</v>
@@ -1316,7 +1316,7 @@
         <v>https://ing.dk/</v>
       </c>
       <c r="O11" t="str">
-        <v>https://ing.dk/#:~:text=bryder</v>
+        <v>https://ing.dk/#:~:text=Pl%C3%B8jer</v>
       </c>
       <c r="P11" t="str">
         <v/>
@@ -1328,10 +1328,10 @@
         <v/>
       </c>
       <c r="S11" t="str">
-        <v>2026-08-09</v>
+        <v>2026-08-02</v>
       </c>
       <c r="T11" t="str">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="U11" t="str">
         <v>2.5</v>
@@ -1340,7 +1340,7 @@
         <v>2</v>
       </c>
       <c r="W11" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X11" t="str">
         <v/>
@@ -1358,13 +1358,13 @@
         <v/>
       </c>
       <c r="AC11" t="str">
-        <v>15.05</v>
+        <v>7.08</v>
       </c>
       <c r="AD11" t="str">
-        <v>5.27</v>
+        <v>6.76</v>
       </c>
       <c r="AE11" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-27</v>
       </c>
       <c r="AF11" t="str">
         <v/>
@@ -1378,37 +1378,37 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>c2d45936-5793-42b4-968a-e066bcb27036</v>
+        <v>03f5e6c8-8aee-4335-872b-3d6af367eeee</v>
       </c>
       <c r="B12" t="str">
         <v>2026-07-02</v>
       </c>
       <c r="C12" t="str">
-        <v>Pløjer</v>
+        <v>vandløb</v>
       </c>
       <c r="D12" t="str">
-        <v>pløje</v>
+        <v>vandløb</v>
       </c>
       <c r="E12" t="str">
-        <v>verbum</v>
+        <v>substantiv</v>
       </c>
       <c r="F12" t="str">
-        <v/>
+        <v>et</v>
       </c>
       <c r="G12" t="str">
-        <v>-r, -de, -t</v>
+        <v>-et, -, -ene</v>
       </c>
       <c r="H12" t="str">
-        <v>[ˈplʌjə]</v>
+        <v/>
       </c>
       <c r="I12" t="str">
-        <v>https://static.ordnet.dk/mp3/11040/11040224_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/12005/12005692_1.mp3</v>
       </c>
       <c r="J12" t="str">
-        <v>vende det øverste jordlag med en plov inden man sår eller planter afgrøder</v>
+        <v>lang, let skrånende fordybning i landskabet med strømmende vand fx en bæk, en å eller en flod</v>
       </c>
       <c r="K12" t="str">
-        <v>Plows</v>
+        <v>stream</v>
       </c>
       <c r="L12" t="str">
         <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb</v>
@@ -1420,7 +1420,7 @@
         <v>https://ing.dk/</v>
       </c>
       <c r="O12" t="str">
-        <v>https://ing.dk/#:~:text=Pl%C3%B8jer</v>
+        <v>https://ing.dk/#:~:text=vandl%C3%B8b</v>
       </c>
       <c r="P12" t="str">
         <v/>
@@ -1432,10 +1432,10 @@
         <v/>
       </c>
       <c r="S12" t="str">
-        <v>2026-08-02</v>
+        <v>2026-07-29</v>
       </c>
       <c r="T12" t="str">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U12" t="str">
         <v>2.5</v>
@@ -1444,7 +1444,7 @@
         <v>2</v>
       </c>
       <c r="W12" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X12" t="str">
         <v/>
@@ -1462,13 +1462,13 @@
         <v/>
       </c>
       <c r="AC12" t="str">
-        <v>7.08</v>
+        <v>5.83</v>
       </c>
       <c r="AD12" t="str">
-        <v>6.76</v>
+        <v>7.15</v>
       </c>
       <c r="AE12" t="str">
-        <v>2026-07-27</v>
+        <v>2026-07-24</v>
       </c>
       <c r="AF12" t="str">
         <v/>
@@ -1482,49 +1482,49 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>03f5e6c8-8aee-4335-872b-3d6af367eeee</v>
+        <v>6d8e9813-5550-45ab-9874-78033b6c2cd6</v>
       </c>
       <c r="B13" t="str">
         <v>2026-07-02</v>
       </c>
       <c r="C13" t="str">
-        <v>vandløb</v>
+        <v>utroligt</v>
       </c>
       <c r="D13" t="str">
-        <v>vandløb</v>
+        <v>utrolig</v>
       </c>
       <c r="E13" t="str">
-        <v>substantiv</v>
+        <v>adjektiv</v>
       </c>
       <c r="F13" t="str">
-        <v>et</v>
+        <v/>
       </c>
       <c r="G13" t="str">
-        <v>-et, -, -ene</v>
+        <v>-t, -e</v>
       </c>
       <c r="H13" t="str">
-        <v/>
+        <v>[uˈtʁoˀli]</v>
       </c>
       <c r="I13" t="str">
-        <v>https://static.ordnet.dk/mp3/12005/12005692_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/12005/12005364_1.mp3</v>
       </c>
       <c r="J13" t="str">
-        <v>lang, let skrånende fordybning i landskabet med strømmende vand fx en bæk, en å eller en flod</v>
+        <v>for usædvanlig eller usandsynlig til at man kan tro det</v>
       </c>
       <c r="K13" t="str">
-        <v>stream</v>
+        <v>Unbelievable</v>
       </c>
       <c r="L13" t="str">
-        <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb</v>
+        <v>DN: »Helt utroligt«</v>
       </c>
       <c r="M13" t="str">
-        <v>Ingeniøren - nyheder om teknologi og samfund</v>
+        <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb | Ingeniøren</v>
       </c>
       <c r="N13" t="str">
-        <v>https://ing.dk/</v>
+        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb</v>
       </c>
       <c r="O13" t="str">
-        <v>https://ing.dk/#:~:text=vandl%C3%B8b</v>
+        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb#:~:text=utroligt</v>
       </c>
       <c r="P13" t="str">
         <v/>
@@ -1536,10 +1536,10 @@
         <v/>
       </c>
       <c r="S13" t="str">
-        <v>2026-07-29</v>
+        <v>2026-07-31</v>
       </c>
       <c r="T13" t="str">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U13" t="str">
         <v>2.5</v>
@@ -1551,75 +1551,75 @@
         <v>0</v>
       </c>
       <c r="X13" t="str">
-        <v/>
+        <v>2026-07-26</v>
       </c>
       <c r="Y13" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Z13" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA13" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="AB13" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC13" t="str">
-        <v>5.83</v>
+        <v>6.54</v>
       </c>
       <c r="AD13" t="str">
         <v>7.15</v>
       </c>
       <c r="AE13" t="str">
-        <v>2026-07-24</v>
+        <v>2026-07-25</v>
       </c>
       <c r="AF13" t="str">
-        <v/>
+        <v>1.18</v>
       </c>
       <c r="AG13" t="str">
-        <v/>
+        <v>6.49</v>
       </c>
       <c r="AH13" t="str">
-        <v/>
+        <v>2026-07-25</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>6d8e9813-5550-45ab-9874-78033b6c2cd6</v>
+        <v>369d0ecd-e56f-4e9b-882e-e7c44c687a79</v>
       </c>
       <c r="B14" t="str">
         <v>2026-07-02</v>
       </c>
       <c r="C14" t="str">
-        <v>utroligt</v>
+        <v>forargede</v>
       </c>
       <c r="D14" t="str">
-        <v>utrolig</v>
+        <v>forarge</v>
       </c>
       <c r="E14" t="str">
-        <v>adjektiv</v>
+        <v>verbum</v>
       </c>
       <c r="F14" t="str">
         <v/>
       </c>
       <c r="G14" t="str">
-        <v>-t, -e</v>
+        <v>-r, -de, -t</v>
       </c>
       <c r="H14" t="str">
-        <v>[uˈtʁoˀli]</v>
+        <v>[fʌˈɑˀwə]</v>
       </c>
       <c r="I14" t="str">
-        <v>https://static.ordnet.dk/mp3/12005/12005364_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11014/11014199_1.mp3</v>
       </c>
       <c r="J14" t="str">
-        <v>for usædvanlig eller usandsynlig til at man kan tro det</v>
+        <v>vække afsky, harme, vrede, modvilje el.lign. ved at krænke moralske normer</v>
       </c>
       <c r="K14" t="str">
-        <v>Unbelievable</v>
+        <v>Outraged</v>
       </c>
       <c r="L14" t="str">
-        <v>DN: »Helt utroligt«</v>
+        <v>Også i Danmarks Naturfredningsforening (DN) er man forargede over, at der ikke er større fokus på naturbeskyttelsen både hos landbruget og på kommunernes kontorer.</v>
       </c>
       <c r="M14" t="str">
         <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb | Ingeniøren</v>
@@ -1628,7 +1628,7 @@
         <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb</v>
       </c>
       <c r="O14" t="str">
-        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb#:~:text=utroligt</v>
+        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb#:~:text=forargede</v>
       </c>
       <c r="P14" t="str">
         <v/>
@@ -1640,99 +1640,99 @@
         <v/>
       </c>
       <c r="S14" t="str">
-        <v>2026-07-31</v>
+        <v>2026-07-28</v>
       </c>
       <c r="T14" t="str">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="U14" t="str">
         <v>2.5</v>
       </c>
       <c r="V14" t="str">
+        <v>1</v>
+      </c>
+      <c r="W14" t="str">
         <v>2</v>
       </c>
-      <c r="W14" t="str">
-        <v>0</v>
-      </c>
       <c r="X14" t="str">
-        <v>2026-07-26</v>
+        <v/>
       </c>
       <c r="Y14" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="Z14" t="str">
-        <v>2.5</v>
+        <v/>
       </c>
       <c r="AA14" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="AB14" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AC14" t="str">
-        <v>6.54</v>
+        <v>0.08</v>
       </c>
       <c r="AD14" t="str">
-        <v>7.15</v>
+        <v>9.4</v>
       </c>
       <c r="AE14" t="str">
-        <v>2026-07-25</v>
+        <v>2026-07-27</v>
       </c>
       <c r="AF14" t="str">
-        <v>1.18</v>
+        <v/>
       </c>
       <c r="AG14" t="str">
-        <v>6.49</v>
+        <v/>
       </c>
       <c r="AH14" t="str">
-        <v>2026-07-25</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>369d0ecd-e56f-4e9b-882e-e7c44c687a79</v>
+        <v>94801dbf-f81c-46cc-a320-3e40b0903e79</v>
       </c>
       <c r="B15" t="str">
         <v>2026-07-02</v>
       </c>
       <c r="C15" t="str">
-        <v>forargede</v>
+        <v>Rådgivning</v>
       </c>
       <c r="D15" t="str">
-        <v>forarge</v>
+        <v>rådgivning</v>
       </c>
       <c r="E15" t="str">
-        <v>verbum</v>
+        <v>substantiv</v>
       </c>
       <c r="F15" t="str">
-        <v/>
+        <v>en</v>
       </c>
       <c r="G15" t="str">
-        <v>-r, -de, -t</v>
+        <v>-en, -er, -erne</v>
       </c>
       <c r="H15" t="str">
-        <v>[fʌˈɑˀwə]</v>
+        <v>[ˈʁʌðˌgiwˀneŋ]</v>
       </c>
       <c r="I15" t="str">
-        <v>https://static.ordnet.dk/mp3/11014/11014199_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11044/11044289_1.mp3</v>
       </c>
       <c r="J15" t="str">
-        <v>vække afsky, harme, vrede, modvilje el.lign. ved at krænke moralske normer</v>
+        <v>det at rådgive</v>
       </c>
       <c r="K15" t="str">
-        <v>Outraged</v>
+        <v>counseling</v>
       </c>
       <c r="L15" t="str">
-        <v>Også i Danmarks Naturfredningsforening (DN) er man forargede over, at der ikke er større fokus på naturbeskyttelsen både hos landbruget og på kommunernes kontorer.</v>
+        <v/>
       </c>
       <c r="M15" t="str">
-        <v>Landmænd over hele landet bryder loven: Pløjer kilometer efter kilometer helt ud til vandløb | Ingeniøren</v>
+        <v/>
       </c>
       <c r="N15" t="str">
-        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb</v>
+        <v/>
       </c>
       <c r="O15" t="str">
-        <v>https://ing.dk/artikel/landmaend-over-hele-landet-bryder-loven-ploejer-kilometer-efter-kilometer-helt-ud-til-vandloeb#:~:text=forargede</v>
+        <v/>
       </c>
       <c r="P15" t="str">
         <v/>
@@ -1744,99 +1744,99 @@
         <v/>
       </c>
       <c r="S15" t="str">
-        <v>2026-07-27</v>
+        <v>2026-07-31</v>
       </c>
       <c r="T15" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="U15" t="str">
         <v>2.5</v>
       </c>
       <c r="V15" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W15" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X15" t="str">
-        <v/>
+        <v>2026-07-27</v>
       </c>
       <c r="Y15" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="Z15" t="str">
-        <v/>
+        <v>2.5</v>
       </c>
       <c r="AA15" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AB15" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="AC15" t="str">
-        <v>0.1</v>
+        <v>3.88</v>
       </c>
       <c r="AD15" t="str">
-        <v>9.32</v>
+        <v>7.15</v>
       </c>
       <c r="AE15" t="str">
         <v>2026-07-27</v>
       </c>
       <c r="AF15" t="str">
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="AG15" t="str">
-        <v/>
+        <v>7.19</v>
       </c>
       <c r="AH15" t="str">
-        <v/>
+        <v>2026-07-27</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>94801dbf-f81c-46cc-a320-3e40b0903e79</v>
+        <v>71eb02a5-f505-41e4-b9a7-2dd955f74d3e</v>
       </c>
       <c r="B16" t="str">
         <v>2026-07-02</v>
       </c>
       <c r="C16" t="str">
-        <v>Rådgivning</v>
+        <v>indgreb</v>
       </c>
       <c r="D16" t="str">
-        <v>rådgivning</v>
+        <v>indgreb</v>
       </c>
       <c r="E16" t="str">
         <v>substantiv</v>
       </c>
       <c r="F16" t="str">
-        <v>en</v>
+        <v>et</v>
       </c>
       <c r="G16" t="str">
-        <v>-en, -er, -erne</v>
+        <v>-et, -, -ene</v>
       </c>
       <c r="H16" t="str">
-        <v>[ˈʁʌðˌgiwˀneŋ]</v>
+        <v/>
       </c>
       <c r="I16" t="str">
-        <v>https://static.ordnet.dk/mp3/11044/11044289_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11023/11023304_1.mp3</v>
       </c>
       <c r="J16" t="str">
-        <v>det at rådgive</v>
+        <v>handling hvormed man blander sig i noget for at ændre den aktuelle situation</v>
       </c>
       <c r="K16" t="str">
-        <v>counseling</v>
+        <v>intervention</v>
       </c>
       <c r="L16" t="str">
-        <v/>
+        <v>Datacentre jagter sort energi efter politisk indgreb: »Det vil være en katastrofe«</v>
       </c>
       <c r="M16" t="str">
-        <v/>
+        <v>AI-lyskryds fjerner bilkøer på vejene: Men nogle må holde længe for rødt - yihengldavid@gmail.com - Gmail</v>
       </c>
       <c r="N16" t="str">
-        <v/>
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
       </c>
       <c r="O16" t="str">
-        <v/>
+        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=indgreb</v>
       </c>
       <c r="P16" t="str">
         <v/>
@@ -1848,66 +1848,66 @@
         <v/>
       </c>
       <c r="S16" t="str">
-        <v>2026-07-31</v>
+        <v>2026-07-28</v>
       </c>
       <c r="T16" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U16" t="str">
         <v>2.5</v>
       </c>
       <c r="V16" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W16" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X16" t="str">
-        <v>2026-07-27</v>
+        <v/>
       </c>
       <c r="Y16" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="Z16" t="str">
-        <v>2.5</v>
+        <v/>
       </c>
       <c r="AA16" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AB16" t="str">
-        <v>0</v>
+        <v/>
       </c>
       <c r="AC16" t="str">
-        <v>3.88</v>
+        <v>0.55</v>
       </c>
       <c r="AD16" t="str">
-        <v>7.15</v>
+        <v>8.05</v>
       </c>
       <c r="AE16" t="str">
         <v>2026-07-27</v>
       </c>
       <c r="AF16" t="str">
-        <v>0.4</v>
+        <v/>
       </c>
       <c r="AG16" t="str">
-        <v>7.19</v>
+        <v/>
       </c>
       <c r="AH16" t="str">
-        <v>2026-07-27</v>
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>71eb02a5-f505-41e4-b9a7-2dd955f74d3e</v>
+        <v>23d95731-816a-467a-a38d-9e6f6a7dced9</v>
       </c>
       <c r="B17" t="str">
         <v>2026-07-02</v>
       </c>
       <c r="C17" t="str">
-        <v>indgreb</v>
+        <v>lovbrud</v>
       </c>
       <c r="D17" t="str">
-        <v>indgreb</v>
+        <v>lovbrud</v>
       </c>
       <c r="E17" t="str">
         <v>substantiv</v>
@@ -1916,31 +1916,31 @@
         <v>et</v>
       </c>
       <c r="G17" t="str">
-        <v>-et, -, -ene</v>
+        <v>-det, -, -dene</v>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>[-ˌbʁuð]</v>
       </c>
       <c r="I17" t="str">
-        <v>https://static.ordnet.dk/mp3/11023/11023304_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11030/11030992_1.mp3</v>
       </c>
       <c r="J17" t="str">
-        <v>handling hvormed man blander sig i noget for at ændre den aktuelle situation</v>
+        <v>det at bryde loven; overtrædelse af loven</v>
       </c>
       <c r="K17" t="str">
-        <v>intervention</v>
+        <v>violation of law</v>
       </c>
       <c r="L17" t="str">
-        <v>Datacentre jagter sort energi efter politisk indgreb: »Det vil være en katastrofe«</v>
+        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark</v>
       </c>
       <c r="M17" t="str">
-        <v>AI-lyskryds fjerner bilkøer på vejene: Men nogle må holde længe for rødt - yihengldavid@gmail.com - Gmail</v>
+        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark | Ingeniøren</v>
       </c>
       <c r="N17" t="str">
-        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl</v>
+        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
       </c>
       <c r="O17" t="str">
-        <v>https://mail.google.com/mail/u/0/?tab=rm&amp;ogbl#:~:text=indgreb</v>
+        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=lovbrud</v>
       </c>
       <c r="P17" t="str">
         <v/>
@@ -1952,19 +1952,19 @@
         <v/>
       </c>
       <c r="S17" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-31</v>
       </c>
       <c r="T17" t="str">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U17" t="str">
         <v>2.5</v>
       </c>
       <c r="V17" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W17" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X17" t="str">
         <v/>
@@ -1982,10 +1982,10 @@
         <v/>
       </c>
       <c r="AC17" t="str">
-        <v>0.55</v>
+        <v>3.88</v>
       </c>
       <c r="AD17" t="str">
-        <v>8.05</v>
+        <v>7.15</v>
       </c>
       <c r="AE17" t="str">
         <v>2026-07-27</v>
@@ -2002,49 +2002,49 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>23d95731-816a-467a-a38d-9e6f6a7dced9</v>
+        <v>039ba62e-8413-430f-ac17-4b365506303e</v>
       </c>
       <c r="B18" t="str">
-        <v>2026-07-02</v>
+        <v>2026-07-22</v>
       </c>
       <c r="C18" t="str">
-        <v>lovbrud</v>
+        <v>overvejer</v>
       </c>
       <c r="D18" t="str">
-        <v>lovbrud</v>
+        <v>overveje</v>
       </c>
       <c r="E18" t="str">
-        <v>substantiv</v>
+        <v>verbum</v>
       </c>
       <c r="F18" t="str">
-        <v>et</v>
+        <v/>
       </c>
       <c r="G18" t="str">
-        <v>-det, -, -dene</v>
+        <v>-r, -de, -t</v>
       </c>
       <c r="H18" t="str">
-        <v>[-ˌbʁuð]</v>
+        <v>[-ˌvɑjˀə]</v>
       </c>
       <c r="I18" t="str">
-        <v>https://static.ordnet.dk/mp3/11030/11030992_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11038/11038552_1.mp3</v>
       </c>
       <c r="J18" t="str">
-        <v>det at bryde loven; overtrædelse af loven</v>
+        <v>tænke over noget eller tænke på at gøre noget idet man vurderer hvad der taler for og imod</v>
       </c>
       <c r="K18" t="str">
-        <v>violation of law</v>
+        <v>reflect</v>
       </c>
       <c r="L18" t="str">
-        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark</v>
+        <v/>
       </c>
       <c r="M18" t="str">
-        <v>Se billeder og video: Sådan afslørede vi landmænds lovbrud i store dele af Danmark | Ingeniøren</v>
+        <v/>
       </c>
       <c r="N18" t="str">
-        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig</v>
+        <v/>
       </c>
       <c r="O18" t="str">
-        <v>https://ing.dk/artikel/se-billeder-og-video-saadan-afsloerede-vi-landmaends-lovbrud-i-store-dele-af-danmark?utm_source=nyhedsbrev&amp;utm_medium=email&amp;utm_campaign=ing_daglig#:~:text=lovbrud</v>
+        <v/>
       </c>
       <c r="P18" t="str">
         <v/>
@@ -2056,19 +2056,19 @@
         <v/>
       </c>
       <c r="S18" t="str">
-        <v>2026-07-31</v>
+        <v>2026-07-28</v>
       </c>
       <c r="T18" t="str">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U18" t="str">
         <v>2.5</v>
       </c>
       <c r="V18" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W18" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X18" t="str">
         <v/>
@@ -2086,10 +2086,10 @@
         <v/>
       </c>
       <c r="AC18" t="str">
-        <v>3.88</v>
+        <v>0.08</v>
       </c>
       <c r="AD18" t="str">
-        <v>7.15</v>
+        <v>9.19</v>
       </c>
       <c r="AE18" t="str">
         <v>2026-07-27</v>
@@ -2106,49 +2106,49 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>039ba62e-8413-430f-ac17-4b365506303e</v>
+        <v>c8b4f170-aa1f-4fe2-a8d4-5be8e34cc7a2</v>
       </c>
       <c r="B19" t="str">
         <v>2026-07-22</v>
       </c>
       <c r="C19" t="str">
-        <v>overvejer</v>
+        <v>Knapt</v>
       </c>
       <c r="D19" t="str">
-        <v>overveje</v>
+        <v>knap</v>
       </c>
       <c r="E19" t="str">
-        <v>verbum</v>
+        <v>adjektiv</v>
       </c>
       <c r="F19" t="str">
         <v/>
       </c>
       <c r="G19" t="str">
-        <v>-r, -de, -t</v>
+        <v>-t, -pe</v>
       </c>
       <c r="H19" t="str">
-        <v>[-ˌvɑjˀə]</v>
+        <v>[ˈknɑb]</v>
       </c>
       <c r="I19" t="str">
-        <v>https://static.ordnet.dk/mp3/11038/11038552_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11026/11026578_1.mp3</v>
       </c>
       <c r="J19" t="str">
-        <v>tænke over noget eller tænke på at gøre noget idet man vurderer hvad der taler for og imod</v>
+        <v>af begrænset eller ringe omfang eller mængde</v>
       </c>
       <c r="K19" t="str">
-        <v>reflect</v>
+        <v>barely</v>
       </c>
       <c r="L19" t="str">
-        <v/>
+        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse</v>
       </c>
       <c r="M19" t="str">
-        <v/>
+        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse | SønderborgNYT</v>
       </c>
       <c r="N19" t="str">
-        <v/>
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA</v>
       </c>
       <c r="O19" t="str">
-        <v/>
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA#:~:text=Knapt</v>
       </c>
       <c r="P19" t="str">
         <v/>
@@ -2190,10 +2190,10 @@
         <v/>
       </c>
       <c r="AC19" t="str">
-        <v>0.08</v>
+        <v>0.02</v>
       </c>
       <c r="AD19" t="str">
-        <v>9.19</v>
+        <v>9.76</v>
       </c>
       <c r="AE19" t="str">
         <v>2026-07-27</v>
@@ -2210,40 +2210,40 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>c8b4f170-aa1f-4fe2-a8d4-5be8e34cc7a2</v>
+        <v>e370b465-1be4-4af6-9ce3-6dbf2118fc91</v>
       </c>
       <c r="B20" t="str">
         <v>2026-07-22</v>
       </c>
       <c r="C20" t="str">
-        <v>Knapt</v>
+        <v>gennemsnit</v>
       </c>
       <c r="D20" t="str">
-        <v>knap</v>
+        <v>gennemsnit</v>
       </c>
       <c r="E20" t="str">
-        <v>adjektiv</v>
+        <v>substantiv</v>
       </c>
       <c r="F20" t="str">
-        <v/>
+        <v>et</v>
       </c>
       <c r="G20" t="str">
-        <v>-t, -pe</v>
+        <v>-tet, -, -tene</v>
       </c>
       <c r="H20" t="str">
-        <v>[ˈknɑb]</v>
+        <v>[ˈgεnəmˌsnid]</v>
       </c>
       <c r="I20" t="str">
-        <v>https://static.ordnet.dk/mp3/11026/11026578_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11017/11017684_1.mp3</v>
       </c>
       <c r="J20" t="str">
-        <v>af begrænset eller ringe omfang eller mængde</v>
+        <v>værdi der fås ved at dividere en sammenlagt sum med antallet af værdier der indgår i den sammenlagte sum</v>
       </c>
       <c r="K20" t="str">
-        <v>barely</v>
+        <v>average</v>
       </c>
       <c r="L20" t="str">
-        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse</v>
+        <v>375 studenter fra Sønderborg Kommune står uden en uddannelse fem år efter gymnasiet. Det svarer til knap hver tiende eller 9,5 procent. Selv om det er lidt under landsgennemsnittet på 10,3 procent, er andelen steget med to procentpoint siden 2020.</v>
       </c>
       <c r="M20" t="str">
         <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse | SønderborgNYT</v>
@@ -2252,7 +2252,7 @@
         <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA</v>
       </c>
       <c r="O20" t="str">
-        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA#:~:text=Knapt</v>
+        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA#:~:text=gennemsnit</v>
       </c>
       <c r="P20" t="str">
         <v/>
@@ -2294,10 +2294,10 @@
         <v/>
       </c>
       <c r="AC20" t="str">
-        <v>0.02</v>
+        <v>0.33</v>
       </c>
       <c r="AD20" t="str">
-        <v>9.76</v>
+        <v>8.36</v>
       </c>
       <c r="AE20" t="str">
         <v>2026-07-27</v>
@@ -2314,49 +2314,49 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>e370b465-1be4-4af6-9ce3-6dbf2118fc91</v>
+        <v>7d3ca2e1-b34b-415c-90c7-5e9eabfa1296</v>
       </c>
       <c r="B21" t="str">
-        <v>2026-07-22</v>
+        <v>2026-07-24</v>
       </c>
       <c r="C21" t="str">
-        <v>gennemsnit</v>
+        <v>offentliggjort</v>
       </c>
       <c r="D21" t="str">
-        <v>gennemsnit</v>
+        <v>offentliggøre</v>
       </c>
       <c r="E21" t="str">
-        <v>substantiv</v>
+        <v>verbum</v>
       </c>
       <c r="F21" t="str">
-        <v>et</v>
+        <v/>
       </c>
       <c r="G21" t="str">
-        <v>-tet, -, -tene</v>
+        <v>..gør, ..gjorde, ..gjort</v>
       </c>
       <c r="H21" t="str">
-        <v>[ˈgεnəmˌsnid]</v>
+        <v>[-ˌgɶˀʌ]</v>
       </c>
       <c r="I21" t="str">
-        <v>https://static.ordnet.dk/mp3/11017/11017684_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11036/11036843_1.mp3</v>
       </c>
       <c r="J21" t="str">
-        <v>værdi der fås ved at dividere en sammenlagt sum med antallet af værdier der indgår i den sammenlagte sum</v>
+        <v>gøre kendt eller tilgængelig for offentligheden</v>
       </c>
       <c r="K21" t="str">
-        <v>average</v>
+        <v>publish</v>
       </c>
       <c r="L21" t="str">
-        <v>375 studenter fra Sønderborg Kommune står uden en uddannelse fem år efter gymnasiet. Det svarer til knap hver tiende eller 9,5 procent. Selv om det er lidt under landsgennemsnittet på 10,3 procent, er andelen steget med to procentpoint siden 2020.</v>
+        <v/>
       </c>
       <c r="M21" t="str">
-        <v>Knapt hver tiende student i Sønderborg kommer ikke videre i uddannelse | SønderborgNYT</v>
+        <v/>
       </c>
       <c r="N21" t="str">
-        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA</v>
+        <v/>
       </c>
       <c r="O21" t="str">
-        <v>https://www.sonderborgnyt.dk/flere-studenter-i-soenderborg-kommer-ikke-videre-i-uddannelse/?fbclid=IwY2xjawTN8JBleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHnMKyyOkL-DV8ZLJyDbADYzgRhMkBnDpEe4tPEJcoXUItlptwICADgtDbCSL_aem_AUXsDOls3E-N_sJmj0iFQA#:~:text=gennemsnit</v>
+        <v/>
       </c>
       <c r="P21" t="str">
         <v/>
@@ -2398,10 +2398,10 @@
         <v/>
       </c>
       <c r="AC21" t="str">
-        <v>0.33</v>
+        <v>0.11</v>
       </c>
       <c r="AD21" t="str">
-        <v>8.36</v>
+        <v>9.41</v>
       </c>
       <c r="AE21" t="str">
         <v>2026-07-27</v>
@@ -2418,49 +2418,49 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>7d3ca2e1-b34b-415c-90c7-5e9eabfa1296</v>
+        <v>47f625fa-3dac-4f40-bed4-2654ab45fb25</v>
       </c>
       <c r="B22" t="str">
-        <v>2026-07-24</v>
+        <v>2026-07-25</v>
       </c>
       <c r="C22" t="str">
-        <v>offentliggjort</v>
+        <v>stemning</v>
       </c>
       <c r="D22" t="str">
-        <v>offentliggøre</v>
+        <v>stemning</v>
       </c>
       <c r="E22" t="str">
-        <v>verbum</v>
+        <v>substantiv</v>
       </c>
       <c r="F22" t="str">
-        <v/>
+        <v>en</v>
       </c>
       <c r="G22" t="str">
-        <v>..gør, ..gjorde, ..gjort</v>
+        <v>-en, -er, -erne</v>
       </c>
       <c r="H22" t="str">
-        <v>[-ˌgɶˀʌ]</v>
+        <v>[ˈsdεmneŋ]</v>
       </c>
       <c r="I22" t="str">
-        <v>https://static.ordnet.dk/mp3/11036/11036843_1.mp3</v>
+        <v>https://static.ordnet.dk/mp3/11050/11050102_1.mp3</v>
       </c>
       <c r="J22" t="str">
-        <v>gøre kendt eller tilgængelig for offentligheden</v>
+        <v>sammenfatning af de følelser og den øjeblikkelige sindstilstand der præger en gruppe mennesker og deres indbyrdes forhold i en bestemt situation</v>
       </c>
       <c r="K22" t="str">
-        <v>publish</v>
+        <v>mood</v>
       </c>
       <c r="L22" t="str">
-        <v/>
+        <v>Vores Sønderborg byder igen velkommen til årets Rosé Festival – den ’pinkeste’ og hyggeligste festival med masser af stemning og iskold rosé. Det sker torsdag den 30. juli til lørdag den 1. august i forskellige butikker og restauranter i Sønderborg og Augustenborg.</v>
       </c>
       <c r="M22" t="str">
-        <v/>
+        <v>Rosé Festival byder på smagsoplevelser og sommerhygge | SønderborgNYT</v>
       </c>
       <c r="N22" t="str">
-        <v/>
+        <v>https://www.sonderborgnyt.dk/rose-festival-byder-paa-smagsoplevelser-og-sommerhygge/?fbclid=IwY2xjawTRhJdleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHge_fZTEDNzDWf19K8JQU6fpM4aw7usy9G6cfkJztjRA89165T3TwHWMwDBp_aem_7a90aBcMi5Vez32IFt7oNw</v>
       </c>
       <c r="O22" t="str">
-        <v/>
+        <v>https://www.sonderborgnyt.dk/rose-festival-byder-paa-smagsoplevelser-og-sommerhygge/?fbclid=IwY2xjawTRhJdleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHge_fZTEDNzDWf19K8JQU6fpM4aw7usy9G6cfkJztjRA89165T3TwHWMwDBp_aem_7a90aBcMi5Vez32IFt7oNw#:~:text=stemning</v>
       </c>
       <c r="P22" t="str">
         <v/>
@@ -2472,19 +2472,19 @@
         <v/>
       </c>
       <c r="S22" t="str">
-        <v>2026-07-28</v>
+        <v/>
       </c>
       <c r="T22" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="U22" t="str">
-        <v>2.5</v>
+        <v/>
       </c>
       <c r="V22" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="W22" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="X22" t="str">
         <v/>
@@ -2502,13 +2502,13 @@
         <v/>
       </c>
       <c r="AC22" t="str">
-        <v>0.11</v>
+        <v/>
       </c>
       <c r="AD22" t="str">
-        <v>9.41</v>
+        <v/>
       </c>
       <c r="AE22" t="str">
-        <v>2026-07-27</v>
+        <v/>
       </c>
       <c r="AF22" t="str">
         <v/>
@@ -2517,116 +2517,12 @@
         <v/>
       </c>
       <c r="AH22" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>47f625fa-3dac-4f40-bed4-2654ab45fb25</v>
-      </c>
-      <c r="B23" t="str">
-        <v>2026-07-25</v>
-      </c>
-      <c r="C23" t="str">
-        <v>stemning</v>
-      </c>
-      <c r="D23" t="str">
-        <v>stemning</v>
-      </c>
-      <c r="E23" t="str">
-        <v>substantiv</v>
-      </c>
-      <c r="F23" t="str">
-        <v>en</v>
-      </c>
-      <c r="G23" t="str">
-        <v>-en, -er, -erne</v>
-      </c>
-      <c r="H23" t="str">
-        <v>[ˈsdεmneŋ]</v>
-      </c>
-      <c r="I23" t="str">
-        <v>https://static.ordnet.dk/mp3/11050/11050102_1.mp3</v>
-      </c>
-      <c r="J23" t="str">
-        <v>sammenfatning af de følelser og den øjeblikkelige sindstilstand der præger en gruppe mennesker og deres indbyrdes forhold i en bestemt situation</v>
-      </c>
-      <c r="K23" t="str">
-        <v>mood</v>
-      </c>
-      <c r="L23" t="str">
-        <v>Vores Sønderborg byder igen velkommen til årets Rosé Festival – den ’pinkeste’ og hyggeligste festival med masser af stemning og iskold rosé. Det sker torsdag den 30. juli til lørdag den 1. august i forskellige butikker og restauranter i Sønderborg og Augustenborg.</v>
-      </c>
-      <c r="M23" t="str">
-        <v>Rosé Festival byder på smagsoplevelser og sommerhygge | SønderborgNYT</v>
-      </c>
-      <c r="N23" t="str">
-        <v>https://www.sonderborgnyt.dk/rose-festival-byder-paa-smagsoplevelser-og-sommerhygge/?fbclid=IwY2xjawTRhJdleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHge_fZTEDNzDWf19K8JQU6fpM4aw7usy9G6cfkJztjRA89165T3TwHWMwDBp_aem_7a90aBcMi5Vez32IFt7oNw</v>
-      </c>
-      <c r="O23" t="str">
-        <v>https://www.sonderborgnyt.dk/rose-festival-byder-paa-smagsoplevelser-og-sommerhygge/?fbclid=IwY2xjawTRhJdleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHge_fZTEDNzDWf19K8JQU6fpM4aw7usy9G6cfkJztjRA89165T3TwHWMwDBp_aem_7a90aBcMi5Vez32IFt7oNw#:~:text=stemning</v>
-      </c>
-      <c r="P23" t="str">
-        <v/>
-      </c>
-      <c r="Q23" t="str">
-        <v>ok</v>
-      </c>
-      <c r="R23" t="str">
-        <v/>
-      </c>
-      <c r="S23" t="str">
-        <v/>
-      </c>
-      <c r="T23" t="str">
-        <v/>
-      </c>
-      <c r="U23" t="str">
-        <v/>
-      </c>
-      <c r="V23" t="str">
-        <v/>
-      </c>
-      <c r="W23" t="str">
-        <v/>
-      </c>
-      <c r="X23" t="str">
-        <v/>
-      </c>
-      <c r="Y23" t="str">
-        <v/>
-      </c>
-      <c r="Z23" t="str">
-        <v/>
-      </c>
-      <c r="AA23" t="str">
-        <v/>
-      </c>
-      <c r="AB23" t="str">
-        <v/>
-      </c>
-      <c r="AC23" t="str">
-        <v/>
-      </c>
-      <c r="AD23" t="str">
-        <v/>
-      </c>
-      <c r="AE23" t="str">
-        <v/>
-      </c>
-      <c r="AF23" t="str">
-        <v/>
-      </c>
-      <c r="AG23" t="str">
-        <v/>
-      </c>
-      <c r="AH23" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH22"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3058,7 +2954,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H185"/>
+  <dimension ref="A1:H186"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -7880,10 +7776,36 @@
         <v>1</v>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>369d0ecd-e56f-4e9b-882e-e7c44c687a79</v>
+      </c>
+      <c r="B186" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C186" t="str">
+        <v>2026-07-27T19:43:21.405Z</v>
+      </c>
+      <c r="D186" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E186" t="str">
+        <v>0</v>
+      </c>
+      <c r="F186" t="str">
+        <v>0.08</v>
+      </c>
+      <c r="G186" t="str">
+        <v>9.4</v>
+      </c>
+      <c r="H186" t="str">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H185"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H186"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add word "stigende" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -194,42 +194,42 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH22"/>
+  <dimension ref="A1:AH23"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
-    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
-    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
+    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2520,9 +2520,113 @@
         <v/>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>f4603fa3-f60f-497a-be2a-560f7ae1a574</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="C23" t="str">
+        <v>stigende</v>
+      </c>
+      <c r="D23" t="str">
+        <v>stige</v>
+      </c>
+      <c r="E23" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
+      <c r="G23" t="str">
+        <v>-r, steg, steget</v>
+      </c>
+      <c r="H23" t="str">
+        <v>[ˈsdiːə]</v>
+      </c>
+      <c r="I23" t="str">
+        <v>https://static.ordnet.dk/mp3/11050/11050237_1.mp3</v>
+      </c>
+      <c r="J23" t="str">
+        <v>(langsomt) vokse i værdi, omfang, mængde, styrke eller intensitet; nå et højere niveau på en skala; blive bedre; gå op</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Increasing</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Efter flere år med stigende optag på de videregående uddannelser i Sønderborg er udviklingen vendt. De nye optagstal viser, at både SDU Sønderborg og Syddansk Erhvervsakademi får færre nye studerende i år, og det får nu de lokale politikere til at efterlyse en nærmere analyse af udviklingen.</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Borgmester og udvalgsformand kalder til dialog efter fald i studieoptaget | SønderborgNYT</v>
+      </c>
+      <c r="N23" t="str">
+        <v>https://www.sonderborgnyt.dk/borgmester-og-udvalgsformand-kalder-til-dialog-efter-fald-i-studieoptaget/?fbclid=IwY2xjawTWyAxleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHuqWRSt9XngA17uSV_aWIPnq8lUCgM9xnjm4yAQgiLICGZv5Fz6O3iMh9au1_aem_kSV0AXKpfgo0f6H6jMogWQ</v>
+      </c>
+      <c r="O23" t="str">
+        <v>https://www.sonderborgnyt.dk/borgmester-og-udvalgsformand-kalder-til-dialog-efter-fald-i-studieoptaget/?fbclid=IwY2xjawTWyAxleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHuqWRSt9XngA17uSV_aWIPnq8lUCgM9xnjm4yAQgiLICGZv5Fz6O3iMh9au1_aem_kSV0AXKpfgo0f6H6jMogWQ#:~:text=stigende</v>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str">
+        <v/>
+      </c>
+      <c r="V23" t="str">
+        <v/>
+      </c>
+      <c r="W23" t="str">
+        <v/>
+      </c>
+      <c r="X23" t="str">
+        <v/>
+      </c>
+      <c r="Y23" t="str">
+        <v/>
+      </c>
+      <c r="Z23" t="str">
+        <v/>
+      </c>
+      <c r="AA23" t="str">
+        <v/>
+      </c>
+      <c r="AB23" t="str">
+        <v/>
+      </c>
+      <c r="AC23" t="str">
+        <v/>
+      </c>
+      <c r="AD23" t="str">
+        <v/>
+      </c>
+      <c r="AE23" t="str">
+        <v/>
+      </c>
+      <c r="AF23" t="str">
+        <v/>
+      </c>
+      <c r="AG23" t="str">
+        <v/>
+      </c>
+      <c r="AH23" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "optag" to Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -194,7 +194,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AH22"/>
+  <dimension ref="A1:AH23"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -2520,9 +2520,113 @@
         <v/>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>0b10c54f-474f-48c3-ab2a-200976499aa8</v>
+      </c>
+      <c r="B23" t="str">
+        <v>2026-07-29</v>
+      </c>
+      <c r="C23" t="str">
+        <v>optag</v>
+      </c>
+      <c r="D23" t="str">
+        <v>optag</v>
+      </c>
+      <c r="E23" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F23" t="str">
+        <v>et</v>
+      </c>
+      <c r="G23" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H23" t="str">
+        <v>[ˈʌbˌtæˀj]</v>
+      </c>
+      <c r="I23" t="str">
+        <v>https://static.ordnet.dk/mp3/11037/11037785_1.mp3</v>
+      </c>
+      <c r="J23" t="str">
+        <v>en uddannelses optagelse af studerende, elever eller lærlinge med særligt henblik på eventuelle begrænsninger eller på antal</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Record</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Efter flere år med stigende optag på de videregående uddannelser i Sønderborg er udviklingen vendt. De nye optagstal viser, at både SDU Sønderborg og Syddansk Erhvervsakademi får færre nye studerende i år, og det får nu de lokale politikere til at efterlyse en nærmere analyse af udviklingen.</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Borgmester og udvalgsformand kalder til dialog efter fald i studieoptaget | SønderborgNYT</v>
+      </c>
+      <c r="N23" t="str">
+        <v>https://www.sonderborgnyt.dk/borgmester-og-udvalgsformand-kalder-til-dialog-efter-fald-i-studieoptaget/?fbclid=IwY2xjawTWyAxleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHuqWRSt9XngA17uSV_aWIPnq8lUCgM9xnjm4yAQgiLICGZv5Fz6O3iMh9au1_aem_kSV0AXKpfgo0f6H6jMogWQ</v>
+      </c>
+      <c r="O23" t="str">
+        <v>https://www.sonderborgnyt.dk/borgmester-og-udvalgsformand-kalder-til-dialog-efter-fald-i-studieoptaget/?fbclid=IwY2xjawTWyAxleHRuA2FlbQIxMABicmlkETBCWEhsczVHdmhWQWJiMUFqc3J0YwZhcHBfaWQQMjIyMDM5MTc4ODIwMDg5MgABHuqWRSt9XngA17uSV_aWIPnq8lUCgM9xnjm4yAQgiLICGZv5Fz6O3iMh9au1_aem_kSV0AXKpfgo0f6H6jMogWQ#:~:text=optag</v>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str">
+        <v/>
+      </c>
+      <c r="V23" t="str">
+        <v/>
+      </c>
+      <c r="W23" t="str">
+        <v/>
+      </c>
+      <c r="X23" t="str">
+        <v/>
+      </c>
+      <c r="Y23" t="str">
+        <v/>
+      </c>
+      <c r="Z23" t="str">
+        <v/>
+      </c>
+      <c r="AA23" t="str">
+        <v/>
+      </c>
+      <c r="AB23" t="str">
+        <v/>
+      </c>
+      <c r="AC23" t="str">
+        <v/>
+      </c>
+      <c r="AD23" t="str">
+        <v/>
+      </c>
+      <c r="AE23" t="str">
+        <v/>
+      </c>
+      <c r="AF23" t="str">
+        <v/>
+      </c>
+      <c r="AG23" t="str">
+        <v/>
+      </c>
+      <c r="AH23" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AH22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AH23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: progress 1, log 2 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -196,40 +196,40 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AH23"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="24" max="24" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="25" max="25" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="26" max="26" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="27" max="27" width="8.83203125" customWidth="1" hidden="true"/>
-    <col min="28" max="28" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="29" max="29" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="30" max="30" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="31" max="31" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="32" max="32" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="33" max="33" width="14.83203125" customWidth="1" hidden="true"/>
-    <col min="34" max="34" width="14.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="24" max="24" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="25" max="25" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="26" max="26" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="27" max="27" customWidth="1" width="8.83203125" hidden="true"/>
+    <col min="28" max="28" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="29" max="29" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="30" max="30" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="31" max="31" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="32" max="32" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="33" max="33" customWidth="1" width="14.83203125" hidden="true"/>
+    <col min="34" max="34" customWidth="1" width="14.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2472,7 +2472,7 @@
         <v/>
       </c>
       <c r="S22" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
       <c r="T22" t="str">
         <v>1</v>
@@ -2484,7 +2484,7 @@
         <v>1</v>
       </c>
       <c r="W22" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X22" t="str">
         <v/>
@@ -2502,13 +2502,13 @@
         <v/>
       </c>
       <c r="AC22" t="str">
-        <v>0.34</v>
+        <v>0.44</v>
       </c>
       <c r="AD22" t="str">
-        <v>7.63</v>
+        <v>8.36</v>
       </c>
       <c r="AE22" t="str">
-        <v>2026-07-27</v>
+        <v>2026-07-29</v>
       </c>
       <c r="AF22" t="str">
         <v/>
@@ -3058,7 +3058,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H190"/>
+  <dimension ref="A1:H192"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -8010,10 +8010,62 @@
         <v>1</v>
       </c>
     </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>47f625fa-3dac-4f40-bed4-2654ab45fb25</v>
+      </c>
+      <c r="B191" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C191" t="str">
+        <v>2026-07-29T12:58:32.093Z</v>
+      </c>
+      <c r="D191" t="str">
+        <v>again</v>
+      </c>
+      <c r="E191" t="str">
+        <v>2</v>
+      </c>
+      <c r="F191" t="str">
+        <v>0.31</v>
+      </c>
+      <c r="G191" t="str">
+        <v>8.38</v>
+      </c>
+      <c r="H191" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>47f625fa-3dac-4f40-bed4-2654ab45fb25</v>
+      </c>
+      <c r="B192" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C192" t="str">
+        <v>2026-07-29T12:58:49.468Z</v>
+      </c>
+      <c r="D192" t="str">
+        <v>good</v>
+      </c>
+      <c r="E192" t="str">
+        <v>0</v>
+      </c>
+      <c r="F192" t="str">
+        <v>0.44</v>
+      </c>
+      <c r="G192" t="str">
+        <v>8.36</v>
+      </c>
+      <c r="H192" t="str">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H190"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H192"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 4, log 6 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -496,7 +496,7 @@
         <v/>
       </c>
       <c r="S3" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
       <c r="T3" t="str">
         <v>1</v>
@@ -508,7 +508,7 @@
         <v>1</v>
       </c>
       <c r="W3" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X3" t="str">
         <v>2026-07-26</v>
@@ -526,13 +526,13 @@
         <v>0</v>
       </c>
       <c r="AC3" t="str">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="AD3" t="str">
-        <v>9.29</v>
+        <v>9.54</v>
       </c>
       <c r="AE3" t="str">
-        <v>2026-07-27</v>
+        <v>2026-07-29</v>
       </c>
       <c r="AF3" t="str">
         <v>1.18</v>
@@ -1432,19 +1432,19 @@
         <v/>
       </c>
       <c r="S12" t="str">
-        <v>2026-07-29</v>
+        <v>2026-07-31</v>
       </c>
       <c r="T12" t="str">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="U12" t="str">
         <v>2.5</v>
       </c>
       <c r="V12" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W12" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X12" t="str">
         <v/>
@@ -1462,13 +1462,13 @@
         <v/>
       </c>
       <c r="AC12" t="str">
-        <v>5.83</v>
+        <v>2.03</v>
       </c>
       <c r="AD12" t="str">
-        <v>7.15</v>
+        <v>8.03</v>
       </c>
       <c r="AE12" t="str">
-        <v>2026-07-24</v>
+        <v>2026-07-29</v>
       </c>
       <c r="AF12" t="str">
         <v/>
@@ -1848,16 +1848,16 @@
         <v/>
       </c>
       <c r="S16" t="str">
-        <v>2026-07-28</v>
+        <v>2026-08-01</v>
       </c>
       <c r="T16" t="str">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="U16" t="str">
         <v>2.5</v>
       </c>
       <c r="V16" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W16" t="str">
         <v>1</v>
@@ -1878,13 +1878,13 @@
         <v/>
       </c>
       <c r="AC16" t="str">
-        <v>0.55</v>
+        <v>3.11</v>
       </c>
       <c r="AD16" t="str">
-        <v>8.05</v>
+        <v>8.03</v>
       </c>
       <c r="AE16" t="str">
-        <v>2026-07-27</v>
+        <v>2026-07-29</v>
       </c>
       <c r="AF16" t="str">
         <v/>
@@ -2952,19 +2952,19 @@
         <v/>
       </c>
       <c r="M4" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-29</v>
       </c>
       <c r="N4" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O4" t="str">
         <v>2.5</v>
       </c>
       <c r="P4" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R4" t="str">
         <v/>
@@ -2985,10 +2985,10 @@
         <v>0.06</v>
       </c>
       <c r="X4" t="str">
-        <v>9.41</v>
+        <v>9.57</v>
       </c>
       <c r="Y4" t="str">
-        <v>2026-07-27</v>
+        <v>2026-07-29</v>
       </c>
       <c r="Z4" t="str">
         <v/>
@@ -3058,7 +3058,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H198"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -8062,10 +8062,166 @@
         <v>1</v>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>05d5014c-1bc9-48f5-ac80-9c6659843c67</v>
+      </c>
+      <c r="B193" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C193" t="str">
+        <v>2026-07-29T12:59:54.144Z</v>
+      </c>
+      <c r="D193" t="str">
+        <v>again</v>
+      </c>
+      <c r="E193" t="str">
+        <v>2</v>
+      </c>
+      <c r="F193" t="str">
+        <v>0.2</v>
+      </c>
+      <c r="G193" t="str">
+        <v>9.49</v>
+      </c>
+      <c r="H193" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>03f5e6c8-8aee-4335-872b-3d6af367eeee</v>
+      </c>
+      <c r="B194" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C194" t="str">
+        <v>2026-07-29T13:00:05.913Z</v>
+      </c>
+      <c r="D194" t="str">
+        <v>again</v>
+      </c>
+      <c r="E194" t="str">
+        <v>5</v>
+      </c>
+      <c r="F194" t="str">
+        <v>1.44</v>
+      </c>
+      <c r="G194" t="str">
+        <v>8.05</v>
+      </c>
+      <c r="H194" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>71eb02a5-f505-41e4-b9a7-2dd955f74d3e</v>
+      </c>
+      <c r="B195" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C195" t="str">
+        <v>2026-07-29T13:00:18.001Z</v>
+      </c>
+      <c r="D195" t="str">
+        <v>good</v>
+      </c>
+      <c r="E195" t="str">
+        <v>2</v>
+      </c>
+      <c r="F195" t="str">
+        <v>3.11</v>
+      </c>
+      <c r="G195" t="str">
+        <v>8.03</v>
+      </c>
+      <c r="H195" t="str">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>05d5014c-1bc9-48f5-ac80-9c6659843c67</v>
+      </c>
+      <c r="B196" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C196" t="str">
+        <v>2026-07-29T13:00:29.081Z</v>
+      </c>
+      <c r="D196" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E196" t="str">
+        <v>0</v>
+      </c>
+      <c r="F196" t="str">
+        <v>0.17</v>
+      </c>
+      <c r="G196" t="str">
+        <v>9.54</v>
+      </c>
+      <c r="H196" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>03f5e6c8-8aee-4335-872b-3d6af367eeee</v>
+      </c>
+      <c r="B197" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C197" t="str">
+        <v>2026-07-29T13:00:34.783Z</v>
+      </c>
+      <c r="D197" t="str">
+        <v>good</v>
+      </c>
+      <c r="E197" t="str">
+        <v>0</v>
+      </c>
+      <c r="F197" t="str">
+        <v>2.03</v>
+      </c>
+      <c r="G197" t="str">
+        <v>8.03</v>
+      </c>
+      <c r="H197" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>7bea74c7-5aab-4f05-909c-e9bdd96906fb</v>
+      </c>
+      <c r="B198" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C198" t="str">
+        <v>2026-07-29T13:00:40.490Z</v>
+      </c>
+      <c r="D198" t="str">
+        <v>again</v>
+      </c>
+      <c r="E198" t="str">
+        <v>2</v>
+      </c>
+      <c r="F198" t="str">
+        <v>0.06</v>
+      </c>
+      <c r="G198" t="str">
+        <v>9.57</v>
+      </c>
+      <c r="H198" t="str">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H192"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H198"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Phone: progress 3, log 4 in Arbejde.xlsx
</commit_message>
<xml_diff>
--- a/sets/Arbejde.xlsx
+++ b/sets/Arbejde.xlsx
@@ -912,16 +912,16 @@
         <v/>
       </c>
       <c r="S7" t="str">
-        <v>2026-07-29</v>
+        <v>2026-08-10</v>
       </c>
       <c r="T7" t="str">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="U7" t="str">
         <v>2.5</v>
       </c>
       <c r="V7" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W7" t="str">
         <v>0</v>
@@ -942,13 +942,13 @@
         <v>0</v>
       </c>
       <c r="AC7" t="str">
-        <v>8.57</v>
+        <v>11.31</v>
       </c>
       <c r="AD7" t="str">
-        <v>7.17</v>
+        <v>7.61</v>
       </c>
       <c r="AE7" t="str">
-        <v>2026-07-20</v>
+        <v>2026-07-29</v>
       </c>
       <c r="AF7" t="str">
         <v>0.56</v>
@@ -1640,7 +1640,7 @@
         <v/>
       </c>
       <c r="S14" t="str">
-        <v>2026-07-28</v>
+        <v>2026-07-30</v>
       </c>
       <c r="T14" t="str">
         <v>1</v>
@@ -1652,7 +1652,7 @@
         <v>1</v>
       </c>
       <c r="W14" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X14" t="str">
         <v/>
@@ -1670,13 +1670,13 @@
         <v/>
       </c>
       <c r="AC14" t="str">
-        <v>0.08</v>
+        <v>0.07</v>
       </c>
       <c r="AD14" t="str">
-        <v>9.4</v>
+        <v>9.61</v>
       </c>
       <c r="AE14" t="str">
-        <v>2026-07-27</v>
+        <v>2026-07-29</v>
       </c>
       <c r="AF14" t="str">
         <v/>
@@ -2952,16 +2952,16 @@
         <v/>
       </c>
       <c r="M4" t="str">
-        <v>2026-07-29</v>
+        <v>2026-07-30</v>
       </c>
       <c r="N4" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4" t="str">
         <v>2.5</v>
       </c>
       <c r="P4" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="str">
         <v>2</v>
@@ -2982,10 +2982,10 @@
         <v/>
       </c>
       <c r="W4" t="str">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="X4" t="str">
-        <v>9.57</v>
+        <v>9.61</v>
       </c>
       <c r="Y4" t="str">
         <v>2026-07-29</v>
@@ -3058,7 +3058,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H198"/>
+  <dimension ref="A1:H202"/>
   <cols>
     <col min="1" max="1" customWidth="1" width="12.83203125"/>
     <col min="2" max="2" customWidth="1" width="12.83203125"/>
@@ -8218,10 +8218,114 @@
         <v>0</v>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>0254c900-1cbd-4360-853b-baf63aadaf10</v>
+      </c>
+      <c r="B199" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C199" t="str">
+        <v>2026-07-29T13:01:20.091Z</v>
+      </c>
+      <c r="D199" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E199" t="str">
+        <v>9</v>
+      </c>
+      <c r="F199" t="str">
+        <v>11.31</v>
+      </c>
+      <c r="G199" t="str">
+        <v>7.61</v>
+      </c>
+      <c r="H199" t="str">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>7bea74c7-5aab-4f05-909c-e9bdd96906fb</v>
+      </c>
+      <c r="B200" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C200" t="str">
+        <v>2026-07-29T13:01:26.051Z</v>
+      </c>
+      <c r="D200" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E200" t="str">
+        <v>0</v>
+      </c>
+      <c r="F200" t="str">
+        <v>0.05</v>
+      </c>
+      <c r="G200" t="str">
+        <v>9.61</v>
+      </c>
+      <c r="H200" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>369d0ecd-e56f-4e9b-882e-e7c44c687a79</v>
+      </c>
+      <c r="B201" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C201" t="str">
+        <v>2026-07-29T13:01:42.808Z</v>
+      </c>
+      <c r="D201" t="str">
+        <v>again</v>
+      </c>
+      <c r="E201" t="str">
+        <v>2</v>
+      </c>
+      <c r="F201" t="str">
+        <v>0.08</v>
+      </c>
+      <c r="G201" t="str">
+        <v>9.57</v>
+      </c>
+      <c r="H201" t="str">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>369d0ecd-e56f-4e9b-882e-e7c44c687a79</v>
+      </c>
+      <c r="B202" t="str">
+        <v>da2en</v>
+      </c>
+      <c r="C202" t="str">
+        <v>2026-07-29T13:02:24.054Z</v>
+      </c>
+      <c r="D202" t="str">
+        <v>hard</v>
+      </c>
+      <c r="E202" t="str">
+        <v>0</v>
+      </c>
+      <c r="F202" t="str">
+        <v>0.07</v>
+      </c>
+      <c r="G202" t="str">
+        <v>9.61</v>
+      </c>
+      <c r="H202" t="str">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H198"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H202"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>